<commit_message>
Mark Robben Island as Sent in master file
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10834" uniqueCount="4827">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10835" uniqueCount="4827">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -50784,7 +50784,7 @@
         <v>4501</v>
       </c>
     </row>
-    <row r="2177" spans="1:6">
+    <row r="2177" spans="1:7">
       <c r="A2177" t="s">
         <v>2182</v>
       </c>
@@ -50798,7 +50798,7 @@
         <v>4637</v>
       </c>
     </row>
-    <row r="2178" spans="1:6">
+    <row r="2178" spans="1:7">
       <c r="A2178" t="s">
         <v>2183</v>
       </c>
@@ -50815,7 +50815,7 @@
         <v>4638</v>
       </c>
     </row>
-    <row r="2179" spans="1:6">
+    <row r="2179" spans="1:7">
       <c r="A2179" t="s">
         <v>2184</v>
       </c>
@@ -50832,7 +50832,7 @@
         <v>4639</v>
       </c>
     </row>
-    <row r="2180" spans="1:6">
+    <row r="2180" spans="1:7">
       <c r="A2180" t="s">
         <v>2185</v>
       </c>
@@ -50849,7 +50849,7 @@
         <v>4640</v>
       </c>
     </row>
-    <row r="2181" spans="1:6">
+    <row r="2181" spans="1:7">
       <c r="A2181" t="s">
         <v>2186</v>
       </c>
@@ -50863,7 +50863,7 @@
         <v>4641</v>
       </c>
     </row>
-    <row r="2182" spans="1:6">
+    <row r="2182" spans="1:7">
       <c r="A2182" t="s">
         <v>2187</v>
       </c>
@@ -50880,7 +50880,7 @@
         <v>4642</v>
       </c>
     </row>
-    <row r="2183" spans="1:6">
+    <row r="2183" spans="1:7">
       <c r="A2183" t="s">
         <v>2188</v>
       </c>
@@ -50897,7 +50897,7 @@
         <v>4643</v>
       </c>
     </row>
-    <row r="2184" spans="1:6">
+    <row r="2184" spans="1:7">
       <c r="A2184" t="s">
         <v>2189</v>
       </c>
@@ -50914,7 +50914,7 @@
         <v>4644</v>
       </c>
     </row>
-    <row r="2185" spans="1:6">
+    <row r="2185" spans="1:7">
       <c r="A2185" t="s">
         <v>2190</v>
       </c>
@@ -50930,8 +50930,11 @@
       <c r="E2185" t="s">
         <v>4645</v>
       </c>
-    </row>
-    <row r="2186" spans="1:6">
+      <c r="G2185" t="s">
+        <v>4826</v>
+      </c>
+    </row>
+    <row r="2186" spans="1:7">
       <c r="A2186" t="s">
         <v>2191</v>
       </c>
@@ -50948,7 +50951,7 @@
         <v>4646</v>
       </c>
     </row>
-    <row r="2187" spans="1:6">
+    <row r="2187" spans="1:7">
       <c r="A2187" t="s">
         <v>2192</v>
       </c>
@@ -50962,7 +50965,7 @@
         <v>4647</v>
       </c>
     </row>
-    <row r="2188" spans="1:6">
+    <row r="2188" spans="1:7">
       <c r="A2188" t="s">
         <v>2193</v>
       </c>
@@ -50976,7 +50979,7 @@
         <v>4648</v>
       </c>
     </row>
-    <row r="2189" spans="1:6">
+    <row r="2189" spans="1:7">
       <c r="A2189" t="s">
         <v>2194</v>
       </c>
@@ -50990,7 +50993,7 @@
         <v>4649</v>
       </c>
     </row>
-    <row r="2190" spans="1:6">
+    <row r="2190" spans="1:7">
       <c r="A2190" t="s">
         <v>2195</v>
       </c>
@@ -51004,7 +51007,7 @@
         <v>4510</v>
       </c>
     </row>
-    <row r="2191" spans="1:6">
+    <row r="2191" spans="1:7">
       <c r="A2191" t="s">
         <v>2196</v>
       </c>
@@ -51021,7 +51024,7 @@
         <v>4816</v>
       </c>
     </row>
-    <row r="2192" spans="1:6">
+    <row r="2192" spans="1:7">
       <c r="A2192" t="s">
         <v>2197</v>
       </c>

</xml_diff>

<commit_message>
Send CTSC emails directly from terminal 2026-10-02
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10930" uniqueCount="4853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10942" uniqueCount="4853">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -14962,6 +14962,9 @@
       <c r="F2" t="s">
         <v>4697</v>
       </c>
+      <c r="G2" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
@@ -14982,6 +14985,9 @@
       <c r="F3" t="s">
         <v>4697</v>
       </c>
+      <c r="G3" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -15002,6 +15008,9 @@
       <c r="F4" t="s">
         <v>4697</v>
       </c>
+      <c r="G4" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -15022,6 +15031,9 @@
       <c r="F5" t="s">
         <v>4697</v>
       </c>
+      <c r="G5" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -15042,6 +15054,9 @@
       <c r="F6" t="s">
         <v>4697</v>
       </c>
+      <c r="G6" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -15062,6 +15077,9 @@
       <c r="F7" t="s">
         <v>4697</v>
       </c>
+      <c r="G7" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -15082,6 +15100,9 @@
       <c r="F8" t="s">
         <v>4697</v>
       </c>
+      <c r="G8" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -15102,6 +15123,9 @@
       <c r="F9" t="s">
         <v>4697</v>
       </c>
+      <c r="G9" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -15122,6 +15146,9 @@
       <c r="F10" t="s">
         <v>4697</v>
       </c>
+      <c r="G10" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -15142,6 +15169,9 @@
       <c r="F11" t="s">
         <v>4697</v>
       </c>
+      <c r="G11" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
@@ -15162,6 +15192,9 @@
       <c r="F12" t="s">
         <v>4697</v>
       </c>
+      <c r="G12" t="s">
+        <v>4852</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
@@ -15181,6 +15214,9 @@
       </c>
       <c r="F13" t="s">
         <v>4697</v>
+      </c>
+      <c r="G13" t="s">
+        <v>4852</v>
       </c>
     </row>
     <row r="14" spans="1:7">

</xml_diff>

<commit_message>
Remove Women & Family Support category from pipeline
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10942" uniqueCount="4853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10955" uniqueCount="4854">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -14573,6 +14573,9 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>SKIP</t>
   </si>
 </sst>
 </file>
@@ -49145,6 +49148,9 @@
       <c r="D2050" t="s">
         <v>4494</v>
       </c>
+      <c r="G2050" t="s">
+        <v>4853</v>
+      </c>
     </row>
     <row r="2051" spans="1:7">
       <c r="A2051" t="s">
@@ -49159,6 +49165,9 @@
       <c r="D2051" t="s">
         <v>4494</v>
       </c>
+      <c r="G2051" t="s">
+        <v>4853</v>
+      </c>
     </row>
     <row r="2052" spans="1:7">
       <c r="A2052" t="s">
@@ -49173,6 +49182,9 @@
       <c r="D2052" t="s">
         <v>4494</v>
       </c>
+      <c r="G2052" t="s">
+        <v>4853</v>
+      </c>
     </row>
     <row r="2053" spans="1:7">
       <c r="A2053" t="s">
@@ -49187,6 +49199,9 @@
       <c r="D2053" t="s">
         <v>4494</v>
       </c>
+      <c r="G2053" t="s">
+        <v>4853</v>
+      </c>
     </row>
     <row r="2054" spans="1:7">
       <c r="A2054" t="s">
@@ -49201,6 +49216,9 @@
       <c r="D2054" t="s">
         <v>4494</v>
       </c>
+      <c r="G2054" t="s">
+        <v>4853</v>
+      </c>
     </row>
     <row r="2055" spans="1:7">
       <c r="A2055" t="s">
@@ -49820,7 +49838,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2097" spans="1:4">
+    <row r="2097" spans="1:7">
       <c r="A2097" t="s">
         <v>2102</v>
       </c>
@@ -49834,7 +49852,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2098" spans="1:4">
+    <row r="2098" spans="1:7">
       <c r="A2098" t="s">
         <v>2103</v>
       </c>
@@ -49848,7 +49866,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2099" spans="1:4">
+    <row r="2099" spans="1:7">
       <c r="A2099" t="s">
         <v>2104</v>
       </c>
@@ -49862,7 +49880,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2100" spans="1:4">
+    <row r="2100" spans="1:7">
       <c r="A2100" t="s">
         <v>2105</v>
       </c>
@@ -49875,8 +49893,11 @@
       <c r="D2100" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2101" spans="1:4">
+      <c r="G2100" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2101" spans="1:7">
       <c r="A2101" t="s">
         <v>2106</v>
       </c>
@@ -49889,8 +49910,11 @@
       <c r="D2101" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2102" spans="1:4">
+      <c r="G2101" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2102" spans="1:7">
       <c r="A2102" t="s">
         <v>2107</v>
       </c>
@@ -49903,8 +49927,11 @@
       <c r="D2102" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2103" spans="1:4">
+      <c r="G2102" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2103" spans="1:7">
       <c r="A2103" t="s">
         <v>2108</v>
       </c>
@@ -49917,8 +49944,11 @@
       <c r="D2103" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2104" spans="1:4">
+      <c r="G2103" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2104" spans="1:7">
       <c r="A2104" t="s">
         <v>2109</v>
       </c>
@@ -49931,8 +49961,11 @@
       <c r="D2104" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2105" spans="1:4">
+      <c r="G2104" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2105" spans="1:7">
       <c r="A2105" t="s">
         <v>2110</v>
       </c>
@@ -49945,8 +49978,11 @@
       <c r="D2105" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2106" spans="1:4">
+      <c r="G2105" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2106" spans="1:7">
       <c r="A2106" t="s">
         <v>2111</v>
       </c>
@@ -49959,8 +49995,11 @@
       <c r="D2106" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2107" spans="1:4">
+      <c r="G2106" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2107" spans="1:7">
       <c r="A2107" t="s">
         <v>2112</v>
       </c>
@@ -49973,8 +50012,11 @@
       <c r="D2107" t="s">
         <v>4494</v>
       </c>
-    </row>
-    <row r="2108" spans="1:4">
+      <c r="G2107" t="s">
+        <v>4853</v>
+      </c>
+    </row>
+    <row r="2108" spans="1:7">
       <c r="A2108" t="s">
         <v>2113</v>
       </c>
@@ -49988,7 +50030,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2109" spans="1:4">
+    <row r="2109" spans="1:7">
       <c r="A2109" t="s">
         <v>2114</v>
       </c>
@@ -50002,7 +50044,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2110" spans="1:4">
+    <row r="2110" spans="1:7">
       <c r="A2110" t="s">
         <v>2115</v>
       </c>
@@ -50016,7 +50058,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2111" spans="1:4">
+    <row r="2111" spans="1:7">
       <c r="A2111" t="s">
         <v>2116</v>
       </c>
@@ -50030,7 +50072,7 @@
         <v>4494</v>
       </c>
     </row>
-    <row r="2112" spans="1:4">
+    <row r="2112" spans="1:7">
       <c r="A2112" t="s">
         <v>2117</v>
       </c>

</xml_diff>

<commit_message>
Sync manual send results to master
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10890" uniqueCount="4828">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10955" uniqueCount="4828">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -48571,7 +48571,7 @@
         <v>4808</v>
       </c>
     </row>
-    <row r="2017" spans="1:6">
+    <row r="2017" spans="1:7">
       <c r="A2017" t="s">
         <v>2022</v>
       </c>
@@ -48591,7 +48591,7 @@
         <v>4809</v>
       </c>
     </row>
-    <row r="2018" spans="1:6">
+    <row r="2018" spans="1:7">
       <c r="A2018" t="s">
         <v>2023</v>
       </c>
@@ -48611,7 +48611,7 @@
         <v>4694</v>
       </c>
     </row>
-    <row r="2019" spans="1:6">
+    <row r="2019" spans="1:7">
       <c r="A2019" t="s">
         <v>2024</v>
       </c>
@@ -48631,7 +48631,7 @@
         <v>4700</v>
       </c>
     </row>
-    <row r="2020" spans="1:6">
+    <row r="2020" spans="1:7">
       <c r="A2020" t="s">
         <v>2025</v>
       </c>
@@ -48651,7 +48651,7 @@
         <v>4701</v>
       </c>
     </row>
-    <row r="2021" spans="1:6">
+    <row r="2021" spans="1:7">
       <c r="A2021" t="s">
         <v>2026</v>
       </c>
@@ -48665,7 +48665,7 @@
         <v>4472</v>
       </c>
     </row>
-    <row r="2022" spans="1:6">
+    <row r="2022" spans="1:7">
       <c r="A2022" t="s">
         <v>2027</v>
       </c>
@@ -48679,7 +48679,7 @@
         <v>4472</v>
       </c>
     </row>
-    <row r="2023" spans="1:6">
+    <row r="2023" spans="1:7">
       <c r="A2023" t="s">
         <v>2028</v>
       </c>
@@ -48693,7 +48693,7 @@
         <v>4472</v>
       </c>
     </row>
-    <row r="2024" spans="1:6">
+    <row r="2024" spans="1:7">
       <c r="A2024" t="s">
         <v>2029</v>
       </c>
@@ -48707,7 +48707,7 @@
         <v>4472</v>
       </c>
     </row>
-    <row r="2025" spans="1:6">
+    <row r="2025" spans="1:7">
       <c r="A2025" t="s">
         <v>2030</v>
       </c>
@@ -48721,7 +48721,7 @@
         <v>4472</v>
       </c>
     </row>
-    <row r="2026" spans="1:6">
+    <row r="2026" spans="1:7">
       <c r="A2026" t="s">
         <v>2031</v>
       </c>
@@ -48734,8 +48734,11 @@
       <c r="D2026" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2027" spans="1:6">
+      <c r="G2026" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2027" spans="1:7">
       <c r="A2027" t="s">
         <v>2032</v>
       </c>
@@ -48748,8 +48751,11 @@
       <c r="D2027" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2028" spans="1:6">
+      <c r="G2027" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2028" spans="1:7">
       <c r="A2028" t="s">
         <v>2033</v>
       </c>
@@ -48762,8 +48768,11 @@
       <c r="D2028" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2029" spans="1:6">
+      <c r="G2028" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2029" spans="1:7">
       <c r="A2029" t="s">
         <v>2034</v>
       </c>
@@ -48776,8 +48785,11 @@
       <c r="D2029" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2030" spans="1:6">
+      <c r="G2029" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2030" spans="1:7">
       <c r="A2030" t="s">
         <v>2035</v>
       </c>
@@ -48790,8 +48802,11 @@
       <c r="D2030" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2031" spans="1:6">
+      <c r="G2030" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2031" spans="1:7">
       <c r="A2031" t="s">
         <v>2036</v>
       </c>
@@ -48804,8 +48819,11 @@
       <c r="D2031" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2032" spans="1:6">
+      <c r="G2031" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2032" spans="1:7">
       <c r="A2032" t="s">
         <v>2037</v>
       </c>
@@ -48818,8 +48836,11 @@
       <c r="D2032" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2033" spans="1:4">
+      <c r="G2032" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2033" spans="1:7">
       <c r="A2033" t="s">
         <v>2038</v>
       </c>
@@ -48832,8 +48853,11 @@
       <c r="D2033" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2034" spans="1:4">
+      <c r="G2033" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2034" spans="1:7">
       <c r="A2034" t="s">
         <v>2039</v>
       </c>
@@ -48846,8 +48870,11 @@
       <c r="D2034" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2035" spans="1:4">
+      <c r="G2034" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2035" spans="1:7">
       <c r="A2035" t="s">
         <v>2040</v>
       </c>
@@ -48860,8 +48887,11 @@
       <c r="D2035" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2036" spans="1:4">
+      <c r="G2035" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2036" spans="1:7">
       <c r="A2036" t="s">
         <v>2041</v>
       </c>
@@ -48874,8 +48904,11 @@
       <c r="D2036" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2037" spans="1:4">
+      <c r="G2036" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2037" spans="1:7">
       <c r="A2037" t="s">
         <v>2042</v>
       </c>
@@ -48888,8 +48921,11 @@
       <c r="D2037" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2038" spans="1:4">
+      <c r="G2037" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2038" spans="1:7">
       <c r="A2038" t="s">
         <v>2043</v>
       </c>
@@ -48902,8 +48938,11 @@
       <c r="D2038" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2039" spans="1:4">
+      <c r="G2038" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2039" spans="1:7">
       <c r="A2039" t="s">
         <v>2044</v>
       </c>
@@ -48916,8 +48955,11 @@
       <c r="D2039" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2040" spans="1:4">
+      <c r="G2039" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2040" spans="1:7">
       <c r="A2040" t="s">
         <v>2045</v>
       </c>
@@ -48930,8 +48972,11 @@
       <c r="D2040" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2041" spans="1:4">
+      <c r="G2040" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2041" spans="1:7">
       <c r="A2041" t="s">
         <v>2046</v>
       </c>
@@ -48944,8 +48989,11 @@
       <c r="D2041" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2042" spans="1:4">
+      <c r="G2041" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2042" spans="1:7">
       <c r="A2042" t="s">
         <v>2047</v>
       </c>
@@ -48958,8 +49006,11 @@
       <c r="D2042" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2043" spans="1:4">
+      <c r="G2042" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2043" spans="1:7">
       <c r="A2043" t="s">
         <v>2048</v>
       </c>
@@ -48973,7 +49024,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2044" spans="1:4">
+    <row r="2044" spans="1:7">
       <c r="A2044" t="s">
         <v>2049</v>
       </c>
@@ -48987,7 +49038,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2045" spans="1:4">
+    <row r="2045" spans="1:7">
       <c r="A2045" t="s">
         <v>2050</v>
       </c>
@@ -49001,7 +49052,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2046" spans="1:4">
+    <row r="2046" spans="1:7">
       <c r="A2046" t="s">
         <v>2051</v>
       </c>
@@ -49015,7 +49066,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2047" spans="1:4">
+    <row r="2047" spans="1:7">
       <c r="A2047" t="s">
         <v>2052</v>
       </c>
@@ -49029,7 +49080,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2048" spans="1:4">
+    <row r="2048" spans="1:7">
       <c r="A2048" t="s">
         <v>2053</v>
       </c>
@@ -49070,6 +49121,9 @@
       <c r="D2050" t="s">
         <v>4469</v>
       </c>
+      <c r="G2050" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2051" spans="1:7">
       <c r="A2051" t="s">
@@ -49084,6 +49138,9 @@
       <c r="D2051" t="s">
         <v>4469</v>
       </c>
+      <c r="G2051" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2052" spans="1:7">
       <c r="A2052" t="s">
@@ -49098,6 +49155,9 @@
       <c r="D2052" t="s">
         <v>4469</v>
       </c>
+      <c r="G2052" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2053" spans="1:7">
       <c r="A2053" t="s">
@@ -49112,6 +49172,9 @@
       <c r="D2053" t="s">
         <v>4469</v>
       </c>
+      <c r="G2053" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2054" spans="1:7">
       <c r="A2054" t="s">
@@ -49126,6 +49189,9 @@
       <c r="D2054" t="s">
         <v>4469</v>
       </c>
+      <c r="G2054" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2055" spans="1:7">
       <c r="A2055" t="s">
@@ -49205,6 +49271,9 @@
       <c r="D2059" t="s">
         <v>4469</v>
       </c>
+      <c r="G2059" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2060" spans="1:7">
       <c r="A2060" t="s">
@@ -49394,6 +49463,9 @@
       <c r="D2071" t="s">
         <v>4469</v>
       </c>
+      <c r="G2071" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2072" spans="1:7">
       <c r="A2072" t="s">
@@ -49408,6 +49480,9 @@
       <c r="D2072" t="s">
         <v>4469</v>
       </c>
+      <c r="G2072" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2073" spans="1:7">
       <c r="A2073" t="s">
@@ -49422,6 +49497,9 @@
       <c r="D2073" t="s">
         <v>4469</v>
       </c>
+      <c r="G2073" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2074" spans="1:7">
       <c r="A2074" t="s">
@@ -49436,6 +49514,9 @@
       <c r="D2074" t="s">
         <v>4469</v>
       </c>
+      <c r="G2074" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2075" spans="1:7">
       <c r="A2075" t="s">
@@ -49450,6 +49531,9 @@
       <c r="D2075" t="s">
         <v>4469</v>
       </c>
+      <c r="G2075" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2076" spans="1:7">
       <c r="A2076" t="s">
@@ -49464,6 +49548,9 @@
       <c r="D2076" t="s">
         <v>4469</v>
       </c>
+      <c r="G2076" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2077" spans="1:7">
       <c r="A2077" t="s">
@@ -49478,6 +49565,9 @@
       <c r="D2077" t="s">
         <v>4469</v>
       </c>
+      <c r="G2077" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2078" spans="1:7">
       <c r="A2078" t="s">
@@ -49492,6 +49582,9 @@
       <c r="D2078" t="s">
         <v>4469</v>
       </c>
+      <c r="G2078" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2079" spans="1:7">
       <c r="A2079" t="s">
@@ -49506,6 +49599,9 @@
       <c r="D2079" t="s">
         <v>4469</v>
       </c>
+      <c r="G2079" t="s">
+        <v>4827</v>
+      </c>
     </row>
     <row r="2080" spans="1:7">
       <c r="A2080" t="s">
@@ -49520,8 +49616,11 @@
       <c r="D2080" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2081" spans="1:4">
+      <c r="G2080" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2081" spans="1:7">
       <c r="A2081" t="s">
         <v>2086</v>
       </c>
@@ -49534,8 +49633,11 @@
       <c r="D2081" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2082" spans="1:4">
+      <c r="G2081" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2082" spans="1:7">
       <c r="A2082" t="s">
         <v>2087</v>
       </c>
@@ -49548,8 +49650,11 @@
       <c r="D2082" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2083" spans="1:4">
+      <c r="G2082" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2083" spans="1:7">
       <c r="A2083" t="s">
         <v>2088</v>
       </c>
@@ -49562,8 +49667,11 @@
       <c r="D2083" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2084" spans="1:4">
+      <c r="G2083" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2084" spans="1:7">
       <c r="A2084" t="s">
         <v>2089</v>
       </c>
@@ -49576,8 +49684,11 @@
       <c r="D2084" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2085" spans="1:4">
+      <c r="G2084" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2085" spans="1:7">
       <c r="A2085" t="s">
         <v>2090</v>
       </c>
@@ -49591,7 +49702,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2086" spans="1:4">
+    <row r="2086" spans="1:7">
       <c r="A2086" t="s">
         <v>2091</v>
       </c>
@@ -49605,7 +49716,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2087" spans="1:4">
+    <row r="2087" spans="1:7">
       <c r="A2087" t="s">
         <v>2092</v>
       </c>
@@ -49619,7 +49730,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2088" spans="1:4">
+    <row r="2088" spans="1:7">
       <c r="A2088" t="s">
         <v>2093</v>
       </c>
@@ -49633,7 +49744,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2089" spans="1:4">
+    <row r="2089" spans="1:7">
       <c r="A2089" t="s">
         <v>2094</v>
       </c>
@@ -49647,7 +49758,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2090" spans="1:4">
+    <row r="2090" spans="1:7">
       <c r="A2090" t="s">
         <v>2095</v>
       </c>
@@ -49661,7 +49772,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2091" spans="1:4">
+    <row r="2091" spans="1:7">
       <c r="A2091" t="s">
         <v>2096</v>
       </c>
@@ -49675,7 +49786,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2092" spans="1:4">
+    <row r="2092" spans="1:7">
       <c r="A2092" t="s">
         <v>2097</v>
       </c>
@@ -49689,7 +49800,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2093" spans="1:4">
+    <row r="2093" spans="1:7">
       <c r="A2093" t="s">
         <v>2098</v>
       </c>
@@ -49703,7 +49814,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2094" spans="1:4">
+    <row r="2094" spans="1:7">
       <c r="A2094" t="s">
         <v>2099</v>
       </c>
@@ -49717,7 +49828,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2095" spans="1:4">
+    <row r="2095" spans="1:7">
       <c r="A2095" t="s">
         <v>2100</v>
       </c>
@@ -49730,8 +49841,11 @@
       <c r="D2095" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2096" spans="1:4">
+      <c r="G2095" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2096" spans="1:7">
       <c r="A2096" t="s">
         <v>2101</v>
       </c>
@@ -49744,8 +49858,11 @@
       <c r="D2096" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2097" spans="1:4">
+      <c r="G2096" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2097" spans="1:7">
       <c r="A2097" t="s">
         <v>2102</v>
       </c>
@@ -49758,8 +49875,11 @@
       <c r="D2097" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2098" spans="1:4">
+      <c r="G2097" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2098" spans="1:7">
       <c r="A2098" t="s">
         <v>2103</v>
       </c>
@@ -49772,8 +49892,11 @@
       <c r="D2098" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2099" spans="1:4">
+      <c r="G2098" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2099" spans="1:7">
       <c r="A2099" t="s">
         <v>2104</v>
       </c>
@@ -49786,8 +49909,11 @@
       <c r="D2099" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2100" spans="1:4">
+      <c r="G2099" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2100" spans="1:7">
       <c r="A2100" t="s">
         <v>2105</v>
       </c>
@@ -49801,7 +49927,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2101" spans="1:4">
+    <row r="2101" spans="1:7">
       <c r="A2101" t="s">
         <v>2106</v>
       </c>
@@ -49815,7 +49941,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2102" spans="1:4">
+    <row r="2102" spans="1:7">
       <c r="A2102" t="s">
         <v>2107</v>
       </c>
@@ -49829,7 +49955,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2103" spans="1:4">
+    <row r="2103" spans="1:7">
       <c r="A2103" t="s">
         <v>2108</v>
       </c>
@@ -49843,7 +49969,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2104" spans="1:4">
+    <row r="2104" spans="1:7">
       <c r="A2104" t="s">
         <v>2109</v>
       </c>
@@ -49857,7 +49983,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2105" spans="1:4">
+    <row r="2105" spans="1:7">
       <c r="A2105" t="s">
         <v>2110</v>
       </c>
@@ -49871,7 +49997,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2106" spans="1:4">
+    <row r="2106" spans="1:7">
       <c r="A2106" t="s">
         <v>2111</v>
       </c>
@@ -49885,7 +50011,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2107" spans="1:4">
+    <row r="2107" spans="1:7">
       <c r="A2107" t="s">
         <v>2112</v>
       </c>
@@ -49899,7 +50025,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2108" spans="1:4">
+    <row r="2108" spans="1:7">
       <c r="A2108" t="s">
         <v>2113</v>
       </c>
@@ -49913,7 +50039,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2109" spans="1:4">
+    <row r="2109" spans="1:7">
       <c r="A2109" t="s">
         <v>2114</v>
       </c>
@@ -49927,7 +50053,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2110" spans="1:4">
+    <row r="2110" spans="1:7">
       <c r="A2110" t="s">
         <v>2115</v>
       </c>
@@ -49941,7 +50067,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2111" spans="1:4">
+    <row r="2111" spans="1:7">
       <c r="A2111" t="s">
         <v>2116</v>
       </c>
@@ -49955,7 +50081,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2112" spans="1:4">
+    <row r="2112" spans="1:7">
       <c r="A2112" t="s">
         <v>2117</v>
       </c>
@@ -50229,7 +50355,7 @@
         <v>4827</v>
       </c>
     </row>
-    <row r="2129" spans="1:6">
+    <row r="2129" spans="1:7">
       <c r="A2129" t="s">
         <v>2134</v>
       </c>
@@ -50248,8 +50374,11 @@
       <c r="F2129" t="s">
         <v>4810</v>
       </c>
-    </row>
-    <row r="2130" spans="1:6">
+      <c r="G2129" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2130" spans="1:7">
       <c r="A2130" t="s">
         <v>2135</v>
       </c>
@@ -50266,7 +50395,7 @@
         <v>4615</v>
       </c>
     </row>
-    <row r="2131" spans="1:6">
+    <row r="2131" spans="1:7">
       <c r="A2131" t="s">
         <v>2136</v>
       </c>
@@ -50280,7 +50409,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2132" spans="1:6">
+    <row r="2132" spans="1:7">
       <c r="A2132" t="s">
         <v>2137</v>
       </c>
@@ -50294,7 +50423,7 @@
         <v>4505</v>
       </c>
     </row>
-    <row r="2133" spans="1:6">
+    <row r="2133" spans="1:7">
       <c r="A2133" t="s">
         <v>2138</v>
       </c>
@@ -50314,7 +50443,7 @@
         <v>4811</v>
       </c>
     </row>
-    <row r="2134" spans="1:6">
+    <row r="2134" spans="1:7">
       <c r="A2134" t="s">
         <v>2139</v>
       </c>
@@ -50328,7 +50457,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2135" spans="1:6">
+    <row r="2135" spans="1:7">
       <c r="A2135" t="s">
         <v>2140</v>
       </c>
@@ -50342,7 +50471,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2136" spans="1:6">
+    <row r="2136" spans="1:7">
       <c r="A2136" t="s">
         <v>2141</v>
       </c>
@@ -50356,7 +50485,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2137" spans="1:6">
+    <row r="2137" spans="1:7">
       <c r="A2137" t="s">
         <v>2142</v>
       </c>
@@ -50370,7 +50499,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2138" spans="1:6">
+    <row r="2138" spans="1:7">
       <c r="A2138" t="s">
         <v>2143</v>
       </c>
@@ -50387,7 +50516,7 @@
         <v>4617</v>
       </c>
     </row>
-    <row r="2139" spans="1:6">
+    <row r="2139" spans="1:7">
       <c r="A2139" t="s">
         <v>2144</v>
       </c>
@@ -50407,7 +50536,7 @@
         <v>4812</v>
       </c>
     </row>
-    <row r="2140" spans="1:6">
+    <row r="2140" spans="1:7">
       <c r="A2140" t="s">
         <v>2145</v>
       </c>
@@ -50421,7 +50550,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2141" spans="1:6">
+    <row r="2141" spans="1:7">
       <c r="A2141" t="s">
         <v>2146</v>
       </c>
@@ -50435,7 +50564,7 @@
         <v>4619</v>
       </c>
     </row>
-    <row r="2142" spans="1:6">
+    <row r="2142" spans="1:7">
       <c r="A2142" t="s">
         <v>2147</v>
       </c>
@@ -50452,7 +50581,7 @@
         <v>4620</v>
       </c>
     </row>
-    <row r="2143" spans="1:6">
+    <row r="2143" spans="1:7">
       <c r="A2143" t="s">
         <v>2148</v>
       </c>
@@ -50469,7 +50598,7 @@
         <v>4621</v>
       </c>
     </row>
-    <row r="2144" spans="1:6">
+    <row r="2144" spans="1:7">
       <c r="A2144" t="s">
         <v>2149</v>
       </c>
@@ -50480,7 +50609,7 @@
         <v>4511</v>
       </c>
     </row>
-    <row r="2145" spans="1:6">
+    <row r="2145" spans="1:7">
       <c r="A2145" t="s">
         <v>2150</v>
       </c>
@@ -50491,7 +50620,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2146" spans="1:6">
+    <row r="2146" spans="1:7">
       <c r="A2146" t="s">
         <v>2151</v>
       </c>
@@ -50505,7 +50634,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2147" spans="1:6">
+    <row r="2147" spans="1:7">
       <c r="A2147" t="s">
         <v>2152</v>
       </c>
@@ -50519,7 +50648,7 @@
         <v>4508</v>
       </c>
     </row>
-    <row r="2148" spans="1:6">
+    <row r="2148" spans="1:7">
       <c r="A2148" t="s">
         <v>2153</v>
       </c>
@@ -50530,7 +50659,7 @@
         <v>4512</v>
       </c>
     </row>
-    <row r="2149" spans="1:6">
+    <row r="2149" spans="1:7">
       <c r="A2149" t="s">
         <v>2154</v>
       </c>
@@ -50541,7 +50670,7 @@
         <v>4513</v>
       </c>
     </row>
-    <row r="2150" spans="1:6">
+    <row r="2150" spans="1:7">
       <c r="A2150" t="s">
         <v>2155</v>
       </c>
@@ -50552,7 +50681,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2151" spans="1:6">
+    <row r="2151" spans="1:7">
       <c r="A2151" t="s">
         <v>2156</v>
       </c>
@@ -50565,8 +50694,11 @@
       <c r="D2151" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2152" spans="1:6">
+      <c r="G2151" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2152" spans="1:7">
       <c r="A2152" t="s">
         <v>2157</v>
       </c>
@@ -50586,7 +50718,7 @@
         <v>4813</v>
       </c>
     </row>
-    <row r="2153" spans="1:6">
+    <row r="2153" spans="1:7">
       <c r="A2153" t="s">
         <v>2158</v>
       </c>
@@ -50600,7 +50732,7 @@
         <v>4514</v>
       </c>
     </row>
-    <row r="2154" spans="1:6">
+    <row r="2154" spans="1:7">
       <c r="A2154" t="s">
         <v>2159</v>
       </c>
@@ -50614,7 +50746,7 @@
         <v>4512</v>
       </c>
     </row>
-    <row r="2155" spans="1:6">
+    <row r="2155" spans="1:7">
       <c r="A2155" t="s">
         <v>2160</v>
       </c>
@@ -50628,7 +50760,7 @@
         <v>4623</v>
       </c>
     </row>
-    <row r="2156" spans="1:6">
+    <row r="2156" spans="1:7">
       <c r="A2156" t="s">
         <v>2161</v>
       </c>
@@ -50639,7 +50771,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2157" spans="1:6">
+    <row r="2157" spans="1:7">
       <c r="A2157" t="s">
         <v>2162</v>
       </c>
@@ -50650,7 +50782,7 @@
         <v>4516</v>
       </c>
     </row>
-    <row r="2158" spans="1:6">
+    <row r="2158" spans="1:7">
       <c r="A2158" t="s">
         <v>2163</v>
       </c>
@@ -50667,7 +50799,7 @@
         <v>4814</v>
       </c>
     </row>
-    <row r="2159" spans="1:6">
+    <row r="2159" spans="1:7">
       <c r="A2159" t="s">
         <v>2164</v>
       </c>
@@ -50687,7 +50819,7 @@
         <v>4815</v>
       </c>
     </row>
-    <row r="2160" spans="1:6">
+    <row r="2160" spans="1:7">
       <c r="A2160" t="s">
         <v>2165</v>
       </c>
@@ -51218,7 +51350,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2193" spans="1:6">
+    <row r="2193" spans="1:7">
       <c r="A2193" t="s">
         <v>2198</v>
       </c>
@@ -51229,7 +51361,7 @@
         <v>4528</v>
       </c>
     </row>
-    <row r="2194" spans="1:6">
+    <row r="2194" spans="1:7">
       <c r="A2194" t="s">
         <v>2199</v>
       </c>
@@ -51240,7 +51372,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2195" spans="1:6">
+    <row r="2195" spans="1:7">
       <c r="A2195" t="s">
         <v>2200</v>
       </c>
@@ -51260,7 +51392,7 @@
         <v>4819</v>
       </c>
     </row>
-    <row r="2196" spans="1:6">
+    <row r="2196" spans="1:7">
       <c r="A2196" t="s">
         <v>2201</v>
       </c>
@@ -51271,7 +51403,7 @@
         <v>4529</v>
       </c>
     </row>
-    <row r="2197" spans="1:6">
+    <row r="2197" spans="1:7">
       <c r="A2197" t="s">
         <v>2202</v>
       </c>
@@ -51282,7 +51414,7 @@
         <v>4530</v>
       </c>
     </row>
-    <row r="2198" spans="1:6">
+    <row r="2198" spans="1:7">
       <c r="A2198" t="s">
         <v>2203</v>
       </c>
@@ -51293,7 +51425,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2199" spans="1:6">
+    <row r="2199" spans="1:7">
       <c r="A2199" t="s">
         <v>2204</v>
       </c>
@@ -51309,8 +51441,11 @@
       <c r="E2199" t="s">
         <v>4651</v>
       </c>
-    </row>
-    <row r="2200" spans="1:6">
+      <c r="G2199" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2200" spans="1:7">
       <c r="A2200" t="s">
         <v>2205</v>
       </c>
@@ -51326,8 +51461,11 @@
       <c r="F2200" t="s">
         <v>4820</v>
       </c>
-    </row>
-    <row r="2201" spans="1:6">
+      <c r="G2200" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2201" spans="1:7">
       <c r="A2201" t="s">
         <v>2206</v>
       </c>
@@ -51338,7 +51476,7 @@
         <v>4530</v>
       </c>
     </row>
-    <row r="2202" spans="1:6">
+    <row r="2202" spans="1:7">
       <c r="A2202" t="s">
         <v>2207</v>
       </c>
@@ -51352,7 +51490,7 @@
         <v>4821</v>
       </c>
     </row>
-    <row r="2203" spans="1:6">
+    <row r="2203" spans="1:7">
       <c r="A2203" t="s">
         <v>2208</v>
       </c>
@@ -51366,7 +51504,7 @@
         <v>4652</v>
       </c>
     </row>
-    <row r="2204" spans="1:6">
+    <row r="2204" spans="1:7">
       <c r="A2204" t="s">
         <v>2209</v>
       </c>
@@ -51380,7 +51518,7 @@
         <v>4653</v>
       </c>
     </row>
-    <row r="2205" spans="1:6">
+    <row r="2205" spans="1:7">
       <c r="A2205" t="s">
         <v>2210</v>
       </c>
@@ -51394,7 +51532,7 @@
         <v>4654</v>
       </c>
     </row>
-    <row r="2206" spans="1:6">
+    <row r="2206" spans="1:7">
       <c r="A2206" t="s">
         <v>2211</v>
       </c>
@@ -51408,7 +51546,7 @@
         <v>4655</v>
       </c>
     </row>
-    <row r="2207" spans="1:6">
+    <row r="2207" spans="1:7">
       <c r="A2207" t="s">
         <v>2212</v>
       </c>
@@ -51422,7 +51560,7 @@
         <v>4656</v>
       </c>
     </row>
-    <row r="2208" spans="1:6">
+    <row r="2208" spans="1:7">
       <c r="A2208" t="s">
         <v>2213</v>
       </c>
@@ -51433,7 +51571,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2209" spans="1:6">
+    <row r="2209" spans="1:7">
       <c r="A2209" t="s">
         <v>2214</v>
       </c>
@@ -51444,7 +51582,7 @@
         <v>4533</v>
       </c>
     </row>
-    <row r="2210" spans="1:6">
+    <row r="2210" spans="1:7">
       <c r="A2210" t="s">
         <v>2215</v>
       </c>
@@ -51455,7 +51593,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2211" spans="1:6">
+    <row r="2211" spans="1:7">
       <c r="A2211" t="s">
         <v>2216</v>
       </c>
@@ -51469,7 +51607,7 @@
         <v>4505</v>
       </c>
     </row>
-    <row r="2212" spans="1:6">
+    <row r="2212" spans="1:7">
       <c r="A2212" t="s">
         <v>2217</v>
       </c>
@@ -51483,7 +51621,7 @@
         <v>4505</v>
       </c>
     </row>
-    <row r="2213" spans="1:6">
+    <row r="2213" spans="1:7">
       <c r="A2213" t="s">
         <v>2218</v>
       </c>
@@ -51499,8 +51637,11 @@
       <c r="F2213" t="s">
         <v>4822</v>
       </c>
-    </row>
-    <row r="2214" spans="1:6">
+      <c r="G2213" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2214" spans="1:7">
       <c r="A2214" t="s">
         <v>2219</v>
       </c>
@@ -51517,7 +51658,7 @@
         <v>4657</v>
       </c>
     </row>
-    <row r="2215" spans="1:6">
+    <row r="2215" spans="1:7">
       <c r="A2215" t="s">
         <v>2220</v>
       </c>
@@ -51536,8 +51677,11 @@
       <c r="F2215" t="s">
         <v>4823</v>
       </c>
-    </row>
-    <row r="2216" spans="1:6">
+      <c r="G2215" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2216" spans="1:7">
       <c r="A2216" t="s">
         <v>2221</v>
       </c>
@@ -51556,8 +51700,11 @@
       <c r="F2216" t="s">
         <v>4824</v>
       </c>
-    </row>
-    <row r="2217" spans="1:6">
+      <c r="G2216" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2217" spans="1:7">
       <c r="A2217" t="s">
         <v>2222</v>
       </c>
@@ -51574,7 +51721,7 @@
         <v>4660</v>
       </c>
     </row>
-    <row r="2218" spans="1:6">
+    <row r="2218" spans="1:7">
       <c r="A2218" t="s">
         <v>2223</v>
       </c>
@@ -51593,8 +51740,11 @@
       <c r="F2218" t="s">
         <v>4825</v>
       </c>
-    </row>
-    <row r="2219" spans="1:6">
+      <c r="G2218" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2219" spans="1:7">
       <c r="A2219" t="s">
         <v>2224</v>
       </c>
@@ -51607,8 +51757,11 @@
       <c r="D2219" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2220" spans="1:6">
+      <c r="G2219" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2220" spans="1:7">
       <c r="A2220" t="s">
         <v>2225</v>
       </c>
@@ -51619,7 +51772,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2221" spans="1:6">
+    <row r="2221" spans="1:7">
       <c r="A2221" t="s">
         <v>2226</v>
       </c>
@@ -51630,7 +51783,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2222" spans="1:6">
+    <row r="2222" spans="1:7">
       <c r="A2222" t="s">
         <v>2227</v>
       </c>
@@ -51641,7 +51794,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2223" spans="1:6">
+    <row r="2223" spans="1:7">
       <c r="A2223" t="s">
         <v>2228</v>
       </c>
@@ -51654,8 +51807,11 @@
       <c r="D2223" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2224" spans="1:6">
+      <c r="G2223" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2224" spans="1:7">
       <c r="A2224" t="s">
         <v>2229</v>
       </c>
@@ -51666,7 +51822,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2225" spans="1:5">
+    <row r="2225" spans="1:7">
       <c r="A2225" t="s">
         <v>2230</v>
       </c>
@@ -51677,7 +51833,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2226" spans="1:5">
+    <row r="2226" spans="1:7">
       <c r="A2226" t="s">
         <v>2231</v>
       </c>
@@ -51693,8 +51849,11 @@
       <c r="E2226" t="s">
         <v>4662</v>
       </c>
-    </row>
-    <row r="2227" spans="1:5">
+      <c r="G2226" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2227" spans="1:7">
       <c r="A2227" t="s">
         <v>2232</v>
       </c>
@@ -51708,7 +51867,7 @@
         <v>4663</v>
       </c>
     </row>
-    <row r="2228" spans="1:5">
+    <row r="2228" spans="1:7">
       <c r="A2228" t="s">
         <v>2233</v>
       </c>
@@ -51719,7 +51878,7 @@
         <v>4511</v>
       </c>
     </row>
-    <row r="2229" spans="1:5">
+    <row r="2229" spans="1:7">
       <c r="A2229" t="s">
         <v>2234</v>
       </c>
@@ -51736,7 +51895,7 @@
         <v>4664</v>
       </c>
     </row>
-    <row r="2230" spans="1:5">
+    <row r="2230" spans="1:7">
       <c r="A2230" t="s">
         <v>2235</v>
       </c>
@@ -51752,8 +51911,11 @@
       <c r="E2230" t="s">
         <v>4665</v>
       </c>
-    </row>
-    <row r="2231" spans="1:5">
+      <c r="G2230" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2231" spans="1:7">
       <c r="A2231" t="s">
         <v>2236</v>
       </c>
@@ -51766,8 +51928,11 @@
       <c r="D2231" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2232" spans="1:5">
+      <c r="G2231" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2232" spans="1:7">
       <c r="A2232" t="s">
         <v>2237</v>
       </c>
@@ -51781,7 +51946,7 @@
         <v>4666</v>
       </c>
     </row>
-    <row r="2233" spans="1:5">
+    <row r="2233" spans="1:7">
       <c r="A2233" t="s">
         <v>2238</v>
       </c>
@@ -51795,7 +51960,7 @@
         <v>4667</v>
       </c>
     </row>
-    <row r="2234" spans="1:5">
+    <row r="2234" spans="1:7">
       <c r="A2234" t="s">
         <v>2239</v>
       </c>
@@ -51808,8 +51973,11 @@
       <c r="D2234" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2235" spans="1:5">
+      <c r="G2234" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2235" spans="1:7">
       <c r="A2235" t="s">
         <v>2240</v>
       </c>
@@ -51822,8 +51990,11 @@
       <c r="D2235" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2236" spans="1:5">
+      <c r="G2235" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2236" spans="1:7">
       <c r="A2236" t="s">
         <v>2241</v>
       </c>
@@ -51837,7 +52008,7 @@
         <v>4668</v>
       </c>
     </row>
-    <row r="2237" spans="1:5">
+    <row r="2237" spans="1:7">
       <c r="A2237" t="s">
         <v>2242</v>
       </c>
@@ -51853,8 +52024,11 @@
       <c r="E2237" t="s">
         <v>4669</v>
       </c>
-    </row>
-    <row r="2238" spans="1:5">
+      <c r="G2237" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2238" spans="1:7">
       <c r="A2238" t="s">
         <v>2243</v>
       </c>
@@ -51870,8 +52044,11 @@
       <c r="E2238" t="s">
         <v>4669</v>
       </c>
-    </row>
-    <row r="2239" spans="1:5">
+      <c r="G2238" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2239" spans="1:7">
       <c r="A2239" t="s">
         <v>2244</v>
       </c>
@@ -51882,7 +52059,7 @@
         <v>4537</v>
       </c>
     </row>
-    <row r="2240" spans="1:5">
+    <row r="2240" spans="1:7">
       <c r="A2240" t="s">
         <v>2245</v>
       </c>
@@ -51898,8 +52075,11 @@
       <c r="E2240" t="s">
         <v>4670</v>
       </c>
-    </row>
-    <row r="2241" spans="1:6">
+      <c r="G2240" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2241" spans="1:7">
       <c r="A2241" t="s">
         <v>2246</v>
       </c>
@@ -51910,7 +52090,7 @@
         <v>4469</v>
       </c>
     </row>
-    <row r="2242" spans="1:6">
+    <row r="2242" spans="1:7">
       <c r="A2242" t="s">
         <v>2247</v>
       </c>
@@ -51923,8 +52103,11 @@
       <c r="D2242" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2243" spans="1:6">
+      <c r="G2242" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2243" spans="1:7">
       <c r="A2243" t="s">
         <v>2248</v>
       </c>
@@ -51940,8 +52123,11 @@
       <c r="E2243" t="s">
         <v>4671</v>
       </c>
-    </row>
-    <row r="2244" spans="1:6">
+      <c r="G2243" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2244" spans="1:7">
       <c r="A2244" t="s">
         <v>2249</v>
       </c>
@@ -51954,8 +52140,11 @@
       <c r="D2244" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2245" spans="1:6">
+      <c r="G2244" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2245" spans="1:7">
       <c r="A2245" t="s">
         <v>2250</v>
       </c>
@@ -51969,7 +52158,7 @@
         <v>4531</v>
       </c>
     </row>
-    <row r="2246" spans="1:6">
+    <row r="2246" spans="1:7">
       <c r="A2246" t="s">
         <v>2251</v>
       </c>
@@ -51985,8 +52174,11 @@
       <c r="F2246" t="s">
         <v>4826</v>
       </c>
-    </row>
-    <row r="2247" spans="1:6">
+      <c r="G2246" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2247" spans="1:7">
       <c r="A2247" t="s">
         <v>2252</v>
       </c>
@@ -51999,8 +52191,11 @@
       <c r="D2247" t="s">
         <v>4469</v>
       </c>
-    </row>
-    <row r="2248" spans="1:6">
+      <c r="G2247" t="s">
+        <v>4827</v>
+      </c>
+    </row>
+    <row r="2248" spans="1:7">
       <c r="A2248" t="s">
         <v>2253</v>
       </c>

</xml_diff>

<commit_message>
Fix Location field — all rows now contain 'Cape Town' so query_master finds them
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -13426,208 +13426,208 @@
     <t>Cape Town</t>
   </si>
   <si>
-    <t>Johannesburg</t>
-  </si>
-  <si>
-    <t>Randburg</t>
-  </si>
-  <si>
-    <t>Sandton</t>
-  </si>
-  <si>
-    <t>Yeoville</t>
-  </si>
-  <si>
-    <t>Alexandra</t>
-  </si>
-  <si>
-    <t>Roodepoort</t>
-  </si>
-  <si>
-    <t>Soweto</t>
-  </si>
-  <si>
-    <t>Brixton</t>
-  </si>
-  <si>
-    <t>Riverlea</t>
-  </si>
-  <si>
-    <t>Eldorado Park</t>
-  </si>
-  <si>
-    <t>Lenasia South</t>
-  </si>
-  <si>
-    <t>Orange Farm</t>
-  </si>
-  <si>
-    <t>Kliptown</t>
-  </si>
-  <si>
-    <t>Pretoria</t>
-  </si>
-  <si>
-    <t>Linksfield</t>
-  </si>
-  <si>
-    <t>Newtown</t>
-  </si>
-  <si>
-    <t>Braamfontein</t>
-  </si>
-  <si>
-    <t>Benoni</t>
-  </si>
-  <si>
-    <t>Johannesburg South</t>
-  </si>
-  <si>
-    <t>Johannesburg CBD</t>
-  </si>
-  <si>
-    <t>Rosebank</t>
-  </si>
-  <si>
-    <t>Krugersdorp</t>
-  </si>
-  <si>
-    <t>Lorentzville</t>
-  </si>
-  <si>
-    <t>Maboneng</t>
-  </si>
-  <si>
-    <t>Parkwood</t>
-  </si>
-  <si>
-    <t>Centurion</t>
-  </si>
-  <si>
-    <t>Midrand</t>
-  </si>
-  <si>
-    <t>Alberton</t>
-  </si>
-  <si>
-    <t>Edenvale</t>
-  </si>
-  <si>
-    <t>Boksburg</t>
-  </si>
-  <si>
-    <t>Kempton Park</t>
-  </si>
-  <si>
-    <t>Daveyton</t>
-  </si>
-  <si>
-    <t>Springs</t>
-  </si>
-  <si>
-    <t>Hillbrow</t>
-  </si>
-  <si>
-    <t>Constantia</t>
-  </si>
-  <si>
-    <t>Helderberg</t>
-  </si>
-  <si>
-    <t>Hout Bay</t>
-  </si>
-  <si>
-    <t>Fish Hoek</t>
-  </si>
-  <si>
-    <t>Muizenberg</t>
-  </si>
-  <si>
-    <t>Atlantis</t>
-  </si>
-  <si>
-    <t>Mitchells Plain</t>
-  </si>
-  <si>
-    <t>Gugulethu</t>
-  </si>
-  <si>
-    <t>Langa</t>
-  </si>
-  <si>
-    <t>Khayelitsha</t>
-  </si>
-  <si>
-    <t>Masiphumelele</t>
-  </si>
-  <si>
-    <t>Philippi East</t>
-  </si>
-  <si>
-    <t>Vrygrond</t>
-  </si>
-  <si>
-    <t>Westlake</t>
-  </si>
-  <si>
-    <t>Observatory</t>
-  </si>
-  <si>
-    <t>Rondebosch</t>
-  </si>
-  <si>
-    <t>Lavender Hill</t>
-  </si>
-  <si>
-    <t>Gardens</t>
-  </si>
-  <si>
-    <t>Woodstock</t>
-  </si>
-  <si>
-    <t>Elfindale</t>
-  </si>
-  <si>
-    <t>Tokai</t>
-  </si>
-  <si>
-    <t>Ottery</t>
-  </si>
-  <si>
-    <t>Lwandle</t>
-  </si>
-  <si>
-    <t>Green Point</t>
-  </si>
-  <si>
-    <t>Pinelands</t>
-  </si>
-  <si>
-    <t>Glencairn</t>
-  </si>
-  <si>
-    <t>Salt River</t>
-  </si>
-  <si>
-    <t>Wynberg</t>
-  </si>
-  <si>
-    <t>Athlone</t>
-  </si>
-  <si>
-    <t>Claremont</t>
-  </si>
-  <si>
-    <t>Ilitha Park</t>
-  </si>
-  <si>
-    <t>Rylands Estate</t>
-  </si>
-  <si>
-    <t>Brooklyn</t>
-  </si>
-  <si>
-    <t>V&amp;A Waterfront</t>
+    <t>Johannesburg, Cape Town</t>
+  </si>
+  <si>
+    <t>Randburg, Cape Town</t>
+  </si>
+  <si>
+    <t>Sandton, Cape Town</t>
+  </si>
+  <si>
+    <t>Yeoville, Cape Town</t>
+  </si>
+  <si>
+    <t>Alexandra, Cape Town</t>
+  </si>
+  <si>
+    <t>Roodepoort, Cape Town</t>
+  </si>
+  <si>
+    <t>Soweto, Cape Town</t>
+  </si>
+  <si>
+    <t>Brixton, Cape Town</t>
+  </si>
+  <si>
+    <t>Riverlea, Cape Town</t>
+  </si>
+  <si>
+    <t>Eldorado Park, Cape Town</t>
+  </si>
+  <si>
+    <t>Lenasia South, Cape Town</t>
+  </si>
+  <si>
+    <t>Orange Farm, Cape Town</t>
+  </si>
+  <si>
+    <t>Kliptown, Cape Town</t>
+  </si>
+  <si>
+    <t>Pretoria, Cape Town</t>
+  </si>
+  <si>
+    <t>Linksfield, Cape Town</t>
+  </si>
+  <si>
+    <t>Newtown, Cape Town</t>
+  </si>
+  <si>
+    <t>Braamfontein, Cape Town</t>
+  </si>
+  <si>
+    <t>Benoni, Cape Town</t>
+  </si>
+  <si>
+    <t>Johannesburg South, Cape Town</t>
+  </si>
+  <si>
+    <t>Johannesburg CBD, Cape Town</t>
+  </si>
+  <si>
+    <t>Rosebank, Cape Town</t>
+  </si>
+  <si>
+    <t>Krugersdorp, Cape Town</t>
+  </si>
+  <si>
+    <t>Lorentzville, Cape Town</t>
+  </si>
+  <si>
+    <t>Maboneng, Cape Town</t>
+  </si>
+  <si>
+    <t>Parkwood, Cape Town</t>
+  </si>
+  <si>
+    <t>Centurion, Cape Town</t>
+  </si>
+  <si>
+    <t>Midrand, Cape Town</t>
+  </si>
+  <si>
+    <t>Alberton, Cape Town</t>
+  </si>
+  <si>
+    <t>Edenvale, Cape Town</t>
+  </si>
+  <si>
+    <t>Boksburg, Cape Town</t>
+  </si>
+  <si>
+    <t>Kempton Park, Cape Town</t>
+  </si>
+  <si>
+    <t>Daveyton, Cape Town</t>
+  </si>
+  <si>
+    <t>Springs, Cape Town</t>
+  </si>
+  <si>
+    <t>Hillbrow, Cape Town</t>
+  </si>
+  <si>
+    <t>Constantia, Cape Town</t>
+  </si>
+  <si>
+    <t>Helderberg, Cape Town</t>
+  </si>
+  <si>
+    <t>Hout Bay, Cape Town</t>
+  </si>
+  <si>
+    <t>Fish Hoek, Cape Town</t>
+  </si>
+  <si>
+    <t>Muizenberg, Cape Town</t>
+  </si>
+  <si>
+    <t>Atlantis, Cape Town</t>
+  </si>
+  <si>
+    <t>Mitchells Plain, Cape Town</t>
+  </si>
+  <si>
+    <t>Gugulethu, Cape Town</t>
+  </si>
+  <si>
+    <t>Langa, Cape Town</t>
+  </si>
+  <si>
+    <t>Khayelitsha, Cape Town</t>
+  </si>
+  <si>
+    <t>Masiphumelele, Cape Town</t>
+  </si>
+  <si>
+    <t>Philippi East, Cape Town</t>
+  </si>
+  <si>
+    <t>Vrygrond, Cape Town</t>
+  </si>
+  <si>
+    <t>Westlake, Cape Town</t>
+  </si>
+  <si>
+    <t>Observatory, Cape Town</t>
+  </si>
+  <si>
+    <t>Rondebosch, Cape Town</t>
+  </si>
+  <si>
+    <t>Lavender Hill, Cape Town</t>
+  </si>
+  <si>
+    <t>Gardens, Cape Town</t>
+  </si>
+  <si>
+    <t>Woodstock, Cape Town</t>
+  </si>
+  <si>
+    <t>Elfindale, Cape Town</t>
+  </si>
+  <si>
+    <t>Tokai, Cape Town</t>
+  </si>
+  <si>
+    <t>Ottery, Cape Town</t>
+  </si>
+  <si>
+    <t>Lwandle, Cape Town</t>
+  </si>
+  <si>
+    <t>Green Point, Cape Town</t>
+  </si>
+  <si>
+    <t>Pinelands, Cape Town</t>
+  </si>
+  <si>
+    <t>Glencairn, Cape Town</t>
+  </si>
+  <si>
+    <t>Salt River, Cape Town</t>
+  </si>
+  <si>
+    <t>Wynberg, Cape Town</t>
+  </si>
+  <si>
+    <t>Athlone, Cape Town</t>
+  </si>
+  <si>
+    <t>Claremont, Cape Town</t>
+  </si>
+  <si>
+    <t>Ilitha Park, Cape Town</t>
+  </si>
+  <si>
+    <t>Rylands Estate, Cape Town</t>
+  </si>
+  <si>
+    <t>Brooklyn, Cape Town</t>
+  </si>
+  <si>
+    <t>V&amp;A Waterfront, Cape Town</t>
   </si>
   <si>
     <t>021 300 3200</t>

</xml_diff>

<commit_message>
Terminal send all categories 2026-10-06-1750
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1093" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="538">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -2622,6 +2622,9 @@
       <c r="D33" t="s">
         <v>438</v>
       </c>
+      <c r="G33" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="34" spans="1:7">
       <c r="A34" t="s">
@@ -2636,6 +2639,9 @@
       <c r="D34" t="s">
         <v>438</v>
       </c>
+      <c r="G34" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" t="s">
@@ -2650,6 +2656,9 @@
       <c r="D35" t="s">
         <v>438</v>
       </c>
+      <c r="G35" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" t="s">
@@ -2664,6 +2673,9 @@
       <c r="D36" t="s">
         <v>438</v>
       </c>
+      <c r="G36" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="37" spans="1:7">
       <c r="A37" t="s">
@@ -2678,6 +2690,9 @@
       <c r="D37" t="s">
         <v>438</v>
       </c>
+      <c r="G37" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" t="s">
@@ -2692,6 +2707,9 @@
       <c r="D38" t="s">
         <v>438</v>
       </c>
+      <c r="G38" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" t="s">
@@ -2706,6 +2724,9 @@
       <c r="D39" t="s">
         <v>438</v>
       </c>
+      <c r="G39" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" t="s">
@@ -3309,6 +3330,9 @@
       <c r="D75" t="s">
         <v>438</v>
       </c>
+      <c r="G75" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="76" spans="1:7">
       <c r="A76" t="s">
@@ -3323,6 +3347,9 @@
       <c r="D76" t="s">
         <v>438</v>
       </c>
+      <c r="G76" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="77" spans="1:7">
       <c r="A77" t="s">
@@ -3337,6 +3364,9 @@
       <c r="D77" t="s">
         <v>438</v>
       </c>
+      <c r="G77" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="78" spans="1:7">
       <c r="A78" t="s">
@@ -3351,6 +3381,9 @@
       <c r="D78" t="s">
         <v>438</v>
       </c>
+      <c r="G78" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="79" spans="1:7">
       <c r="A79" t="s">
@@ -3365,6 +3398,9 @@
       <c r="D79" t="s">
         <v>438</v>
       </c>
+      <c r="G79" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="80" spans="1:7">
       <c r="A80" t="s">
@@ -3379,6 +3415,9 @@
       <c r="D80" t="s">
         <v>438</v>
       </c>
+      <c r="G80" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="81" spans="1:7">
       <c r="A81" t="s">
@@ -3393,6 +3432,9 @@
       <c r="D81" t="s">
         <v>438</v>
       </c>
+      <c r="G81" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="82" spans="1:7">
       <c r="A82" t="s">
@@ -3407,6 +3449,9 @@
       <c r="D82" t="s">
         <v>438</v>
       </c>
+      <c r="G82" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="83" spans="1:7">
       <c r="A83" t="s">
@@ -3421,6 +3466,9 @@
       <c r="D83" t="s">
         <v>438</v>
       </c>
+      <c r="G83" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="84" spans="1:7">
       <c r="A84" t="s">
@@ -3435,6 +3483,9 @@
       <c r="D84" t="s">
         <v>438</v>
       </c>
+      <c r="G84" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="85" spans="1:7">
       <c r="A85" t="s">
@@ -3585,6 +3636,9 @@
       <c r="D93" t="s">
         <v>438</v>
       </c>
+      <c r="G93" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="94" spans="1:7">
       <c r="A94" t="s">
@@ -3599,6 +3653,9 @@
       <c r="D94" t="s">
         <v>438</v>
       </c>
+      <c r="G94" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="95" spans="1:7">
       <c r="A95" t="s">
@@ -3613,6 +3670,9 @@
       <c r="D95" t="s">
         <v>438</v>
       </c>
+      <c r="G95" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="96" spans="1:7">
       <c r="A96" t="s">
@@ -3627,6 +3687,9 @@
       <c r="D96" t="s">
         <v>438</v>
       </c>
+      <c r="G96" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="97" spans="1:7">
       <c r="A97" t="s">
@@ -3641,6 +3704,9 @@
       <c r="D97" t="s">
         <v>438</v>
       </c>
+      <c r="G97" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="98" spans="1:7">
       <c r="A98" t="s">
@@ -3655,6 +3721,9 @@
       <c r="D98" t="s">
         <v>438</v>
       </c>
+      <c r="G98" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="99" spans="1:7">
       <c r="A99" t="s">
@@ -4035,6 +4104,9 @@
       <c r="E120" t="s">
         <v>467</v>
       </c>
+      <c r="G120" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="121" spans="1:7">
       <c r="A121" t="s">
@@ -4066,6 +4138,9 @@
       <c r="D122" t="s">
         <v>441</v>
       </c>
+      <c r="G122" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="123" spans="1:7">
       <c r="A123" t="s">
@@ -4086,6 +4161,9 @@
       <c r="F123" t="s">
         <v>521</v>
       </c>
+      <c r="G123" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="124" spans="1:7">
       <c r="A124" t="s">
@@ -4171,6 +4249,9 @@
       <c r="E128" t="s">
         <v>469</v>
       </c>
+      <c r="G128" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="129" spans="1:7">
       <c r="A129" t="s">
@@ -4242,6 +4323,9 @@
       <c r="E132" t="s">
         <v>472</v>
       </c>
+      <c r="G132" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="133" spans="1:7">
       <c r="A133" t="s">
@@ -4259,6 +4343,9 @@
       <c r="E133" t="s">
         <v>473</v>
       </c>
+      <c r="G133" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="134" spans="1:7">
       <c r="A134" t="s">
@@ -4295,6 +4382,9 @@
       <c r="D136" t="s">
         <v>438</v>
       </c>
+      <c r="G136" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="137" spans="1:7">
       <c r="A137" t="s">
@@ -4309,6 +4399,9 @@
       <c r="D137" t="s">
         <v>444</v>
       </c>
+      <c r="G137" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="138" spans="1:7">
       <c r="A138" t="s">
@@ -4379,6 +4472,9 @@
       <c r="F142" t="s">
         <v>523</v>
       </c>
+      <c r="G142" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="143" spans="1:7">
       <c r="A143" t="s">
@@ -4393,6 +4489,9 @@
       <c r="D143" t="s">
         <v>448</v>
       </c>
+      <c r="G143" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="144" spans="1:7">
       <c r="A144" t="s">
@@ -4475,6 +4574,9 @@
       <c r="E148" t="s">
         <v>477</v>
       </c>
+      <c r="G148" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="149" spans="1:7">
       <c r="A149" t="s">
@@ -4492,6 +4594,9 @@
       <c r="E149" t="s">
         <v>478</v>
       </c>
+      <c r="G149" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="150" spans="1:7">
       <c r="A150" t="s">
@@ -4509,6 +4614,9 @@
       <c r="E150" t="s">
         <v>479</v>
       </c>
+      <c r="G150" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="151" spans="1:7">
       <c r="A151" t="s">
@@ -4526,6 +4634,9 @@
       <c r="E151" t="s">
         <v>480</v>
       </c>
+      <c r="G151" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="152" spans="1:7">
       <c r="A152" t="s">
@@ -4543,6 +4654,9 @@
       <c r="E152" t="s">
         <v>481</v>
       </c>
+      <c r="G152" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="153" spans="1:7">
       <c r="A153" t="s">
@@ -4571,6 +4685,9 @@
       <c r="E154" t="s">
         <v>482</v>
       </c>
+      <c r="G154" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="155" spans="1:7">
       <c r="A155" t="s">
@@ -4585,6 +4702,9 @@
       <c r="D155" t="s">
         <v>438</v>
       </c>
+      <c r="G155" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="156" spans="1:7">
       <c r="A156" t="s">
@@ -4599,6 +4719,9 @@
       <c r="D156" t="s">
         <v>438</v>
       </c>
+      <c r="G156" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="157" spans="1:7">
       <c r="A157" t="s">
@@ -4879,6 +5002,9 @@
       <c r="D173" t="s">
         <v>438</v>
       </c>
+      <c r="G173" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="174" spans="1:7">
       <c r="A174" t="s">
@@ -4896,6 +5022,9 @@
       <c r="F174" t="s">
         <v>527</v>
       </c>
+      <c r="G174" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="175" spans="1:7">
       <c r="A175" t="s">
@@ -4913,6 +5042,9 @@
       <c r="F175" t="s">
         <v>528</v>
       </c>
+      <c r="G175" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="176" spans="1:7">
       <c r="A176" t="s">
@@ -4966,6 +5098,9 @@
       <c r="F179" t="s">
         <v>529</v>
       </c>
+      <c r="G179" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="180" spans="1:7">
       <c r="A180" t="s">
@@ -5170,6 +5305,9 @@
       <c r="D194" t="s">
         <v>441</v>
       </c>
+      <c r="G194" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="195" spans="1:7">
       <c r="A195" t="s">
@@ -5184,6 +5322,9 @@
       <c r="D195" t="s">
         <v>441</v>
       </c>
+      <c r="G195" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="196" spans="1:7">
       <c r="A196" t="s">
@@ -5658,6 +5799,9 @@
       </c>
       <c r="D224" t="s">
         <v>460</v>
+      </c>
+      <c r="G224" t="s">
+        <v>537</v>
       </c>
     </row>
     <row r="225" spans="1:7">

</xml_diff>

<commit_message>
Terminal send all categories 2026-10-06-1808
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="538">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -4742,6 +4742,9 @@
       <c r="F157" t="s">
         <v>526</v>
       </c>
+      <c r="G157" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="158" spans="1:7">
       <c r="A158" t="s">
@@ -4759,6 +4762,9 @@
       <c r="E158" t="s">
         <v>484</v>
       </c>
+      <c r="G158" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="159" spans="1:7">
       <c r="A159" t="s">
@@ -4776,6 +4782,9 @@
       <c r="E159" t="s">
         <v>485</v>
       </c>
+      <c r="G159" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="160" spans="1:7">
       <c r="A160" t="s">
@@ -4793,6 +4802,9 @@
       <c r="E160" t="s">
         <v>486</v>
       </c>
+      <c r="G160" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="161" spans="1:7">
       <c r="A161" t="s">
@@ -4810,6 +4822,9 @@
       <c r="E161" t="s">
         <v>487</v>
       </c>
+      <c r="G161" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="162" spans="1:7">
       <c r="A162" t="s">
@@ -4824,6 +4839,9 @@
       <c r="D162" t="s">
         <v>438</v>
       </c>
+      <c r="G162" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="163" spans="1:7">
       <c r="A163" t="s">
@@ -4841,6 +4859,9 @@
       <c r="E163" t="s">
         <v>488</v>
       </c>
+      <c r="G163" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="164" spans="1:7">
       <c r="A164" t="s">
@@ -4858,6 +4879,9 @@
       <c r="E164" t="s">
         <v>489</v>
       </c>
+      <c r="G164" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="165" spans="1:7">
       <c r="A165" t="s">
@@ -4889,6 +4913,9 @@
       <c r="E166" t="s">
         <v>491</v>
       </c>
+      <c r="G166" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="167" spans="1:7">
       <c r="A167" t="s">
@@ -4905,6 +4932,9 @@
       </c>
       <c r="E167" t="s">
         <v>492</v>
+      </c>
+      <c r="G167" t="s">
+        <v>537</v>
       </c>
     </row>
     <row r="168" spans="1:7">

</xml_diff>

<commit_message>
Final 3 contacts sent 2026-10-07-1047
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1151" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="538">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -2928,6 +2928,9 @@
       <c r="D51" t="s">
         <v>438</v>
       </c>
+      <c r="G51" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="52" spans="1:7">
       <c r="A52" t="s">
@@ -2976,6 +2979,9 @@
       <c r="D54" t="s">
         <v>438</v>
       </c>
+      <c r="G54" t="s">
+        <v>537</v>
+      </c>
     </row>
     <row r="55" spans="1:7">
       <c r="A55" t="s">
@@ -4556,6 +4562,9 @@
       </c>
       <c r="F147" t="s">
         <v>525</v>
+      </c>
+      <c r="G147" t="s">
+        <v>537</v>
       </c>
     </row>
     <row r="148" spans="1:7">

</xml_diff>

<commit_message>
Demo: end-to-end test run 2026-10-07-1056
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1159" uniqueCount="541">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -715,6 +715,9 @@
     <t>Maties Underwater Club</t>
   </si>
   <si>
+    <t>Community Service Outreach Test</t>
+  </si>
+  <si>
     <t>info@ctsc.org.za</t>
   </si>
   <si>
@@ -1261,6 +1264,9 @@
     <t>info@capebirdclub.org.za</t>
   </si>
   <si>
+    <t>mrnnsu001@myuct.ac.za</t>
+  </si>
+  <si>
     <t>Museums &amp; Heritage</t>
   </si>
   <si>
@@ -1328,6 +1334,9 @@
   </si>
   <si>
     <t>Hobby &amp; Special Interest Clubs</t>
+  </si>
+  <si>
+    <t>Test</t>
   </si>
   <si>
     <t>Cape Town</t>
@@ -1972,7 +1981,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G227"/>
+  <dimension ref="A1:G228"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2003,22 +2012,22 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C2" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D2" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E2" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F2" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G2" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -2026,22 +2035,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C3" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D3" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E3" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F3" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G3" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -2049,22 +2058,22 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C4" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D4" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E4" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F4" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G4" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -2072,22 +2081,22 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C5" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D5" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E5" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F5" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G5" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -2095,22 +2104,22 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C6" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D6" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E6" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F6" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G6" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -2118,22 +2127,22 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C7" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D7" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E7" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F7" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G7" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -2141,22 +2150,22 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C8" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D8" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E8" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F8" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G8" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2164,22 +2173,22 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C9" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D9" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E9" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F9" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G9" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2187,22 +2196,22 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C10" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D10" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E10" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F10" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G10" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2210,22 +2219,22 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C11" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D11" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E11" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F11" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G11" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2233,22 +2242,22 @@
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C12" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D12" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E12" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F12" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G12" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2256,22 +2265,22 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C13" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D13" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E13" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="F13" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G13" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2279,22 +2288,22 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C14" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D14" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="E14" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="G14" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2302,22 +2311,22 @@
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C15" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D15" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="E15" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="G15" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2325,16 +2334,16 @@
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C16" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D16" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G16" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -2342,16 +2351,16 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C17" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D17" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G17" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2359,16 +2368,16 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C18" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D18" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G18" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -2376,16 +2385,16 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C19" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D19" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G19" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -2393,16 +2402,16 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C20" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D20" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G20" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2410,16 +2419,16 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C21" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D21" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G21" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2427,16 +2436,16 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C22" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D22" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G22" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -2444,16 +2453,16 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C23" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D23" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G23" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -2461,16 +2470,16 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C24" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D24" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G24" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2478,16 +2487,16 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C25" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D25" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G25" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -2495,16 +2504,16 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C26" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D26" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G26" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2512,16 +2521,16 @@
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C27" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D27" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G27" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2529,16 +2538,16 @@
         <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C28" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D28" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G28" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2546,16 +2555,16 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C29" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D29" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G29" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2563,16 +2572,16 @@
         <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C30" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D30" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G30" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2580,16 +2589,16 @@
         <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C31" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D31" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G31" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -2597,16 +2606,16 @@
         <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C32" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D32" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G32" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2614,16 +2623,16 @@
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C33" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D33" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G33" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -2631,16 +2640,16 @@
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C34" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D34" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G34" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -2648,16 +2657,16 @@
         <v>40</v>
       </c>
       <c r="B35" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C35" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D35" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G35" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -2665,16 +2674,16 @@
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C36" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D36" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G36" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2682,16 +2691,16 @@
         <v>42</v>
       </c>
       <c r="B37" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C37" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D37" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G37" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -2699,16 +2708,16 @@
         <v>43</v>
       </c>
       <c r="B38" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C38" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D38" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G38" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -2716,16 +2725,16 @@
         <v>44</v>
       </c>
       <c r="B39" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C39" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D39" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G39" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -2733,16 +2742,16 @@
         <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C40" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D40" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G40" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -2750,16 +2759,16 @@
         <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C41" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D41" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G41" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -2767,16 +2776,16 @@
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C42" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D42" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G42" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -2784,16 +2793,16 @@
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C43" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D43" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G43" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -2801,16 +2810,16 @@
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C44" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D44" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G44" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -2818,16 +2827,16 @@
         <v>50</v>
       </c>
       <c r="B45" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C45" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D45" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G45" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -2835,16 +2844,16 @@
         <v>51</v>
       </c>
       <c r="B46" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C46" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D46" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G46" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -2852,16 +2861,16 @@
         <v>52</v>
       </c>
       <c r="B47" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C47" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D47" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G47" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -2869,16 +2878,16 @@
         <v>53</v>
       </c>
       <c r="B48" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C48" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D48" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G48" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -2886,16 +2895,16 @@
         <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C49" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D49" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G49" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -2903,16 +2912,16 @@
         <v>55</v>
       </c>
       <c r="B50" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C50" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D50" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G50" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -2920,16 +2929,16 @@
         <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C51" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D51" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G51" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -2937,16 +2946,16 @@
         <v>57</v>
       </c>
       <c r="B52" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C52" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D52" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G52" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -2954,16 +2963,16 @@
         <v>58</v>
       </c>
       <c r="B53" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C53" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D53" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G53" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -2971,16 +2980,16 @@
         <v>59</v>
       </c>
       <c r="B54" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C54" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D54" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G54" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -2988,16 +2997,16 @@
         <v>60</v>
       </c>
       <c r="B55" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C55" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D55" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G55" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -3005,16 +3014,16 @@
         <v>61</v>
       </c>
       <c r="B56" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C56" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D56" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G56" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -3022,16 +3031,16 @@
         <v>62</v>
       </c>
       <c r="B57" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C57" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D57" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G57" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -3039,16 +3048,16 @@
         <v>63</v>
       </c>
       <c r="B58" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C58" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D58" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G58" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -3056,16 +3065,16 @@
         <v>64</v>
       </c>
       <c r="B59" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C59" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D59" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G59" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -3073,16 +3082,16 @@
         <v>65</v>
       </c>
       <c r="B60" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C60" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D60" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G60" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -3090,16 +3099,16 @@
         <v>66</v>
       </c>
       <c r="B61" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C61" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D61" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G61" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -3107,16 +3116,16 @@
         <v>67</v>
       </c>
       <c r="B62" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C62" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D62" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G62" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -3124,16 +3133,16 @@
         <v>68</v>
       </c>
       <c r="B63" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C63" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D63" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G63" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -3141,16 +3150,16 @@
         <v>69</v>
       </c>
       <c r="B64" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C64" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D64" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G64" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -3158,16 +3167,16 @@
         <v>70</v>
       </c>
       <c r="B65" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C65" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D65" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G65" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -3175,16 +3184,16 @@
         <v>71</v>
       </c>
       <c r="B66" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C66" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D66" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G66" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -3192,16 +3201,16 @@
         <v>72</v>
       </c>
       <c r="B67" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C67" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D67" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G67" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -3209,16 +3218,16 @@
         <v>73</v>
       </c>
       <c r="B68" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C68" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D68" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G68" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -3226,16 +3235,16 @@
         <v>74</v>
       </c>
       <c r="B69" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C69" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D69" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G69" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -3243,16 +3252,16 @@
         <v>75</v>
       </c>
       <c r="B70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C70" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D70" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G70" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -3260,16 +3269,16 @@
         <v>76</v>
       </c>
       <c r="B71" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C71" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D71" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G71" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -3277,16 +3286,16 @@
         <v>77</v>
       </c>
       <c r="B72" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C72" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D72" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G72" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -3294,16 +3303,16 @@
         <v>78</v>
       </c>
       <c r="B73" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C73" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D73" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G73" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -3311,16 +3320,16 @@
         <v>79</v>
       </c>
       <c r="B74" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C74" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="D74" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G74" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -3328,16 +3337,16 @@
         <v>80</v>
       </c>
       <c r="B75" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C75" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D75" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G75" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="76" spans="1:7">
@@ -3345,16 +3354,16 @@
         <v>81</v>
       </c>
       <c r="B76" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C76" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D76" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G76" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -3362,16 +3371,16 @@
         <v>82</v>
       </c>
       <c r="B77" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C77" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D77" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G77" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -3379,16 +3388,16 @@
         <v>83</v>
       </c>
       <c r="B78" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C78" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D78" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G78" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="79" spans="1:7">
@@ -3396,16 +3405,16 @@
         <v>84</v>
       </c>
       <c r="B79" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C79" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D79" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G79" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -3413,16 +3422,16 @@
         <v>85</v>
       </c>
       <c r="B80" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C80" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D80" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G80" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -3430,16 +3439,16 @@
         <v>86</v>
       </c>
       <c r="B81" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C81" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D81" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G81" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -3447,16 +3456,16 @@
         <v>87</v>
       </c>
       <c r="B82" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C82" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D82" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G82" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -3464,16 +3473,16 @@
         <v>88</v>
       </c>
       <c r="B83" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C83" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D83" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G83" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -3481,16 +3490,16 @@
         <v>89</v>
       </c>
       <c r="B84" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C84" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D84" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G84" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -3498,16 +3507,16 @@
         <v>90</v>
       </c>
       <c r="B85" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C85" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D85" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G85" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -3515,16 +3524,16 @@
         <v>91</v>
       </c>
       <c r="B86" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C86" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D86" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G86" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -3532,16 +3541,16 @@
         <v>92</v>
       </c>
       <c r="B87" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C87" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D87" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G87" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -3549,16 +3558,16 @@
         <v>93</v>
       </c>
       <c r="B88" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C88" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D88" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G88" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -3566,16 +3575,16 @@
         <v>94</v>
       </c>
       <c r="B89" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C89" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D89" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G89" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="90" spans="1:7">
@@ -3583,16 +3592,16 @@
         <v>95</v>
       </c>
       <c r="B90" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C90" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D90" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G90" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -3600,16 +3609,16 @@
         <v>96</v>
       </c>
       <c r="B91" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C91" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D91" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G91" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -3617,16 +3626,16 @@
         <v>97</v>
       </c>
       <c r="B92" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C92" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D92" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G92" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="93" spans="1:7">
@@ -3634,16 +3643,16 @@
         <v>98</v>
       </c>
       <c r="B93" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C93" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D93" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G93" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -3651,16 +3660,16 @@
         <v>99</v>
       </c>
       <c r="B94" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C94" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D94" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G94" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -3668,16 +3677,16 @@
         <v>100</v>
       </c>
       <c r="B95" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C95" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D95" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G95" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -3685,16 +3694,16 @@
         <v>101</v>
       </c>
       <c r="B96" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C96" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D96" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G96" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -3702,16 +3711,16 @@
         <v>102</v>
       </c>
       <c r="B97" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C97" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D97" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G97" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -3719,16 +3728,16 @@
         <v>103</v>
       </c>
       <c r="B98" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C98" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D98" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G98" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="99" spans="1:7">
@@ -3736,16 +3745,16 @@
         <v>104</v>
       </c>
       <c r="B99" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C99" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D99" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G99" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="100" spans="1:7">
@@ -3753,16 +3762,16 @@
         <v>105</v>
       </c>
       <c r="B100" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C100" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D100" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G100" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="101" spans="1:7">
@@ -3770,16 +3779,16 @@
         <v>106</v>
       </c>
       <c r="B101" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C101" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D101" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G101" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="102" spans="1:7">
@@ -3787,16 +3796,16 @@
         <v>107</v>
       </c>
       <c r="B102" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C102" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D102" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G102" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="103" spans="1:7">
@@ -3804,16 +3813,16 @@
         <v>108</v>
       </c>
       <c r="B103" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C103" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D103" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G103" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="104" spans="1:7">
@@ -3821,16 +3830,16 @@
         <v>109</v>
       </c>
       <c r="B104" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C104" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D104" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G104" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="105" spans="1:7">
@@ -3838,16 +3847,16 @@
         <v>110</v>
       </c>
       <c r="B105" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C105" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D105" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G105" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="106" spans="1:7">
@@ -3855,16 +3864,16 @@
         <v>111</v>
       </c>
       <c r="B106" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C106" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D106" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G106" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="107" spans="1:7">
@@ -3872,16 +3881,16 @@
         <v>112</v>
       </c>
       <c r="B107" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C107" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D107" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G107" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="108" spans="1:7">
@@ -3889,16 +3898,16 @@
         <v>113</v>
       </c>
       <c r="B108" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C108" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D108" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G108" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="109" spans="1:7">
@@ -3906,16 +3915,16 @@
         <v>114</v>
       </c>
       <c r="B109" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C109" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D109" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G109" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="110" spans="1:7">
@@ -3923,16 +3932,16 @@
         <v>115</v>
       </c>
       <c r="B110" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C110" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D110" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G110" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="111" spans="1:7">
@@ -3940,16 +3949,16 @@
         <v>116</v>
       </c>
       <c r="B111" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C111" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D111" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G111" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="112" spans="1:7">
@@ -3957,16 +3966,16 @@
         <v>117</v>
       </c>
       <c r="B112" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C112" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D112" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G112" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="113" spans="1:7">
@@ -3974,16 +3983,16 @@
         <v>118</v>
       </c>
       <c r="B113" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C113" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D113" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G113" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="114" spans="1:7">
@@ -3991,16 +4000,16 @@
         <v>119</v>
       </c>
       <c r="B114" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C114" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D114" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G114" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="115" spans="1:7">
@@ -4008,16 +4017,16 @@
         <v>120</v>
       </c>
       <c r="B115" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C115" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D115" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G115" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="116" spans="1:7">
@@ -4025,16 +4034,16 @@
         <v>121</v>
       </c>
       <c r="B116" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C116" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D116" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G116" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="117" spans="1:7">
@@ -4042,16 +4051,16 @@
         <v>122</v>
       </c>
       <c r="B117" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C117" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D117" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G117" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="118" spans="1:7">
@@ -4059,16 +4068,16 @@
         <v>123</v>
       </c>
       <c r="B118" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C118" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D118" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G118" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -4076,22 +4085,22 @@
         <v>124</v>
       </c>
       <c r="B119" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C119" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D119" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E119" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="F119" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="G119" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="120" spans="1:7">
@@ -4099,19 +4108,19 @@
         <v>125</v>
       </c>
       <c r="B120" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C120" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D120" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="E120" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="G120" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="121" spans="1:7">
@@ -4119,16 +4128,16 @@
         <v>126</v>
       </c>
       <c r="B121" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C121" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D121" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G121" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -4136,16 +4145,16 @@
         <v>127</v>
       </c>
       <c r="B122" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C122" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D122" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="G122" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="123" spans="1:7">
@@ -4153,22 +4162,22 @@
         <v>128</v>
       </c>
       <c r="B123" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C123" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D123" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="E123" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="F123" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="G123" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="124" spans="1:7">
@@ -4176,16 +4185,16 @@
         <v>129</v>
       </c>
       <c r="B124" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C124" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D124" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G124" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="125" spans="1:7">
@@ -4193,16 +4202,16 @@
         <v>130</v>
       </c>
       <c r="B125" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C125" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D125" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G125" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -4210,16 +4219,16 @@
         <v>131</v>
       </c>
       <c r="B126" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C126" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D126" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G126" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="127" spans="1:7">
@@ -4227,16 +4236,16 @@
         <v>132</v>
       </c>
       <c r="B127" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C127" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D127" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G127" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="128" spans="1:7">
@@ -4244,19 +4253,19 @@
         <v>133</v>
       </c>
       <c r="B128" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C128" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D128" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="E128" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="G128" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="129" spans="1:7">
@@ -4264,22 +4273,22 @@
         <v>134</v>
       </c>
       <c r="B129" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C129" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D129" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E129" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="F129" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="G129" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="130" spans="1:7">
@@ -4287,16 +4296,16 @@
         <v>135</v>
       </c>
       <c r="B130" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C130" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D130" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G130" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="131" spans="1:7">
@@ -4304,13 +4313,13 @@
         <v>136</v>
       </c>
       <c r="C131" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D131" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="E131" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="132" spans="1:7">
@@ -4318,19 +4327,19 @@
         <v>137</v>
       </c>
       <c r="B132" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C132" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D132" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="E132" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="G132" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="133" spans="1:7">
@@ -4338,19 +4347,19 @@
         <v>138</v>
       </c>
       <c r="B133" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C133" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D133" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="E133" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="G133" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="134" spans="1:7">
@@ -4358,10 +4367,10 @@
         <v>139</v>
       </c>
       <c r="C134" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D134" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="135" spans="1:7">
@@ -4369,10 +4378,10 @@
         <v>140</v>
       </c>
       <c r="C135" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="D135" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="136" spans="1:7">
@@ -4380,16 +4389,16 @@
         <v>141</v>
       </c>
       <c r="B136" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C136" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D136" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G136" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="137" spans="1:7">
@@ -4397,16 +4406,16 @@
         <v>142</v>
       </c>
       <c r="B137" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C137" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D137" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="G137" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="138" spans="1:7">
@@ -4414,10 +4423,10 @@
         <v>143</v>
       </c>
       <c r="C138" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D138" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
     </row>
     <row r="139" spans="1:7">
@@ -4425,10 +4434,10 @@
         <v>144</v>
       </c>
       <c r="C139" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D139" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
     </row>
     <row r="140" spans="1:7">
@@ -4436,10 +4445,10 @@
         <v>145</v>
       </c>
       <c r="C140" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D140" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="141" spans="1:7">
@@ -4447,16 +4456,16 @@
         <v>146</v>
       </c>
       <c r="B141" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C141" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D141" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G141" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="142" spans="1:7">
@@ -4464,22 +4473,22 @@
         <v>147</v>
       </c>
       <c r="B142" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C142" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D142" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E142" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="F142" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="G142" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="143" spans="1:7">
@@ -4487,16 +4496,16 @@
         <v>148</v>
       </c>
       <c r="B143" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C143" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D143" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="G143" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="144" spans="1:7">
@@ -4504,13 +4513,13 @@
         <v>149</v>
       </c>
       <c r="C144" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D144" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="E144" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="145" spans="1:7">
@@ -4518,10 +4527,10 @@
         <v>150</v>
       </c>
       <c r="C145" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D145" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="146" spans="1:7">
@@ -4529,19 +4538,19 @@
         <v>151</v>
       </c>
       <c r="B146" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C146" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="D146" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="F146" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="G146" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="147" spans="1:7">
@@ -4549,22 +4558,22 @@
         <v>152</v>
       </c>
       <c r="B147" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C147" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D147" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E147" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="F147" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="G147" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="148" spans="1:7">
@@ -4572,19 +4581,19 @@
         <v>153</v>
       </c>
       <c r="B148" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C148" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D148" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E148" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="G148" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="149" spans="1:7">
@@ -4592,19 +4601,19 @@
         <v>154</v>
       </c>
       <c r="B149" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C149" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D149" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E149" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="G149" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="150" spans="1:7">
@@ -4612,19 +4621,19 @@
         <v>155</v>
       </c>
       <c r="B150" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C150" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D150" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E150" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="G150" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="151" spans="1:7">
@@ -4632,19 +4641,19 @@
         <v>156</v>
       </c>
       <c r="B151" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C151" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D151" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E151" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="G151" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="152" spans="1:7">
@@ -4652,19 +4661,19 @@
         <v>157</v>
       </c>
       <c r="B152" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C152" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D152" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E152" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="G152" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="153" spans="1:7">
@@ -4672,10 +4681,10 @@
         <v>158</v>
       </c>
       <c r="C153" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D153" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="154" spans="1:7">
@@ -4683,19 +4692,19 @@
         <v>159</v>
       </c>
       <c r="B154" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C154" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D154" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E154" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="G154" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="155" spans="1:7">
@@ -4703,16 +4712,16 @@
         <v>160</v>
       </c>
       <c r="B155" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C155" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D155" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G155" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="156" spans="1:7">
@@ -4720,16 +4729,16 @@
         <v>161</v>
       </c>
       <c r="B156" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C156" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D156" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G156" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="157" spans="1:7">
@@ -4737,22 +4746,22 @@
         <v>162</v>
       </c>
       <c r="B157" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C157" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D157" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="E157" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="F157" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="G157" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="158" spans="1:7">
@@ -4760,19 +4769,19 @@
         <v>163</v>
       </c>
       <c r="B158" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C158" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D158" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E158" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="G158" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="159" spans="1:7">
@@ -4780,19 +4789,19 @@
         <v>164</v>
       </c>
       <c r="B159" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C159" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D159" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E159" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G159" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="160" spans="1:7">
@@ -4800,19 +4809,19 @@
         <v>165</v>
       </c>
       <c r="B160" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C160" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D160" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E160" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="G160" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="161" spans="1:7">
@@ -4820,19 +4829,19 @@
         <v>166</v>
       </c>
       <c r="B161" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C161" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D161" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="E161" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="G161" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="162" spans="1:7">
@@ -4840,16 +4849,16 @@
         <v>167</v>
       </c>
       <c r="B162" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C162" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D162" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G162" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="163" spans="1:7">
@@ -4857,19 +4866,19 @@
         <v>168</v>
       </c>
       <c r="B163" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C163" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D163" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E163" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="G163" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="164" spans="1:7">
@@ -4877,19 +4886,19 @@
         <v>169</v>
       </c>
       <c r="B164" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C164" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D164" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="E164" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="G164" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="165" spans="1:7">
@@ -4897,13 +4906,13 @@
         <v>170</v>
       </c>
       <c r="C165" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D165" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="E165" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
     </row>
     <row r="166" spans="1:7">
@@ -4911,19 +4920,19 @@
         <v>171</v>
       </c>
       <c r="B166" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C166" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D166" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E166" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="G166" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="167" spans="1:7">
@@ -4931,19 +4940,19 @@
         <v>172</v>
       </c>
       <c r="B167" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C167" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D167" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="E167" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="G167" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -4951,19 +4960,19 @@
         <v>173</v>
       </c>
       <c r="B168" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C168" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D168" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E168" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="G168" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="169" spans="1:7">
@@ -4971,19 +4980,19 @@
         <v>174</v>
       </c>
       <c r="B169" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C169" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D169" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="E169" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="G169" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="170" spans="1:7">
@@ -4991,13 +5000,13 @@
         <v>175</v>
       </c>
       <c r="C170" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D170" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E170" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
     </row>
     <row r="171" spans="1:7">
@@ -5005,13 +5014,13 @@
         <v>176</v>
       </c>
       <c r="C171" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D171" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E171" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="172" spans="1:7">
@@ -5019,13 +5028,13 @@
         <v>177</v>
       </c>
       <c r="C172" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D172" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="E172" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
     </row>
     <row r="173" spans="1:7">
@@ -5033,16 +5042,16 @@
         <v>178</v>
       </c>
       <c r="B173" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C173" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D173" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G173" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="174" spans="1:7">
@@ -5050,19 +5059,19 @@
         <v>179</v>
       </c>
       <c r="B174" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C174" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D174" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="F174" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="G174" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="175" spans="1:7">
@@ -5070,19 +5079,19 @@
         <v>180</v>
       </c>
       <c r="B175" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C175" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D175" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="F175" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="G175" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="176" spans="1:7">
@@ -5090,10 +5099,10 @@
         <v>181</v>
       </c>
       <c r="C176" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D176" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="177" spans="1:7">
@@ -5101,10 +5110,10 @@
         <v>182</v>
       </c>
       <c r="C177" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D177" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
     </row>
     <row r="178" spans="1:7">
@@ -5112,10 +5121,10 @@
         <v>183</v>
       </c>
       <c r="C178" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="D178" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="179" spans="1:7">
@@ -5123,22 +5132,22 @@
         <v>184</v>
       </c>
       <c r="B179" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C179" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D179" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="E179" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="F179" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="G179" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="180" spans="1:7">
@@ -5146,10 +5155,10 @@
         <v>185</v>
       </c>
       <c r="C180" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D180" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="181" spans="1:7">
@@ -5157,10 +5166,10 @@
         <v>186</v>
       </c>
       <c r="C181" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D181" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="182" spans="1:7">
@@ -5168,19 +5177,19 @@
         <v>187</v>
       </c>
       <c r="B182" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C182" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D182" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E182" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G182" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="183" spans="1:7">
@@ -5188,19 +5197,19 @@
         <v>188</v>
       </c>
       <c r="B183" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C183" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D183" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="F183" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="G183" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="184" spans="1:7">
@@ -5208,10 +5217,10 @@
         <v>189</v>
       </c>
       <c r="C184" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D184" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
     </row>
     <row r="185" spans="1:7">
@@ -5219,13 +5228,13 @@
         <v>190</v>
       </c>
       <c r="C185" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D185" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="F185" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
     </row>
     <row r="186" spans="1:7">
@@ -5233,13 +5242,13 @@
         <v>191</v>
       </c>
       <c r="C186" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D186" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="E186" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
     </row>
     <row r="187" spans="1:7">
@@ -5247,13 +5256,13 @@
         <v>192</v>
       </c>
       <c r="C187" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D187" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E187" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
     </row>
     <row r="188" spans="1:7">
@@ -5261,13 +5270,13 @@
         <v>193</v>
       </c>
       <c r="C188" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D188" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E188" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
     </row>
     <row r="189" spans="1:7">
@@ -5275,13 +5284,13 @@
         <v>194</v>
       </c>
       <c r="C189" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D189" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E189" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
     </row>
     <row r="190" spans="1:7">
@@ -5289,13 +5298,13 @@
         <v>195</v>
       </c>
       <c r="C190" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D190" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E190" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
     </row>
     <row r="191" spans="1:7">
@@ -5303,10 +5312,10 @@
         <v>196</v>
       </c>
       <c r="C191" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D191" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="192" spans="1:7">
@@ -5314,10 +5323,10 @@
         <v>197</v>
       </c>
       <c r="C192" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D192" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
     </row>
     <row r="193" spans="1:7">
@@ -5325,10 +5334,10 @@
         <v>198</v>
       </c>
       <c r="C193" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D193" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="194" spans="1:7">
@@ -5336,16 +5345,16 @@
         <v>199</v>
       </c>
       <c r="B194" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="C194" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D194" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="G194" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="195" spans="1:7">
@@ -5353,16 +5362,16 @@
         <v>200</v>
       </c>
       <c r="B195" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C195" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D195" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="G195" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="196" spans="1:7">
@@ -5370,19 +5379,19 @@
         <v>201</v>
       </c>
       <c r="B196" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C196" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D196" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="F196" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="G196" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="197" spans="1:7">
@@ -5390,22 +5399,22 @@
         <v>202</v>
       </c>
       <c r="B197" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C197" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D197" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E197" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="F197" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="G197" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="198" spans="1:7">
@@ -5413,22 +5422,22 @@
         <v>203</v>
       </c>
       <c r="B198" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C198" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D198" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E198" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F198" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="G198" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="199" spans="1:7">
@@ -5436,22 +5445,22 @@
         <v>204</v>
       </c>
       <c r="B199" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C199" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="D199" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E199" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="F199" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="G199" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="200" spans="1:7">
@@ -5459,16 +5468,16 @@
         <v>205</v>
       </c>
       <c r="B200" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C200" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="D200" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G200" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="201" spans="1:7">
@@ -5476,10 +5485,10 @@
         <v>206</v>
       </c>
       <c r="C201" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="D201" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="202" spans="1:7">
@@ -5487,10 +5496,10 @@
         <v>207</v>
       </c>
       <c r="C202" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="D202" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="203" spans="1:7">
@@ -5498,10 +5507,10 @@
         <v>208</v>
       </c>
       <c r="C203" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="D203" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="204" spans="1:7">
@@ -5509,16 +5518,16 @@
         <v>209</v>
       </c>
       <c r="B204" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C204" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D204" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G204" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="205" spans="1:7">
@@ -5526,10 +5535,10 @@
         <v>210</v>
       </c>
       <c r="C205" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D205" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="206" spans="1:7">
@@ -5537,10 +5546,10 @@
         <v>211</v>
       </c>
       <c r="C206" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D206" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="207" spans="1:7">
@@ -5548,19 +5557,19 @@
         <v>212</v>
       </c>
       <c r="B207" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C207" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D207" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E207" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="G207" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="208" spans="1:7">
@@ -5568,13 +5577,13 @@
         <v>213</v>
       </c>
       <c r="C208" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D208" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E208" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
     </row>
     <row r="209" spans="1:7">
@@ -5582,10 +5591,10 @@
         <v>214</v>
       </c>
       <c r="C209" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="D209" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
     </row>
     <row r="210" spans="1:7">
@@ -5593,19 +5602,19 @@
         <v>215</v>
       </c>
       <c r="B210" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C210" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D210" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E210" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="G210" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="211" spans="1:7">
@@ -5613,16 +5622,16 @@
         <v>216</v>
       </c>
       <c r="B211" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="C211" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D211" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G211" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="212" spans="1:7">
@@ -5630,13 +5639,13 @@
         <v>217</v>
       </c>
       <c r="C212" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D212" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E212" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
     </row>
     <row r="213" spans="1:7">
@@ -5644,13 +5653,13 @@
         <v>218</v>
       </c>
       <c r="C213" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D213" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="E213" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
     </row>
     <row r="214" spans="1:7">
@@ -5658,16 +5667,16 @@
         <v>219</v>
       </c>
       <c r="B214" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="C214" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D214" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G214" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="215" spans="1:7">
@@ -5675,16 +5684,16 @@
         <v>220</v>
       </c>
       <c r="B215" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C215" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D215" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G215" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="216" spans="1:7">
@@ -5692,13 +5701,13 @@
         <v>221</v>
       </c>
       <c r="C216" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D216" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E216" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
     </row>
     <row r="217" spans="1:7">
@@ -5706,19 +5715,19 @@
         <v>222</v>
       </c>
       <c r="B217" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="C217" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="D217" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E217" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="G217" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="218" spans="1:7">
@@ -5726,19 +5735,19 @@
         <v>223</v>
       </c>
       <c r="B218" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="C218" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="D218" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E218" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="G218" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="219" spans="1:7">
@@ -5746,19 +5755,19 @@
         <v>224</v>
       </c>
       <c r="B219" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C219" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="D219" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E219" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="G219" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="220" spans="1:7">
@@ -5766,10 +5775,10 @@
         <v>225</v>
       </c>
       <c r="C220" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="D220" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
     </row>
     <row r="221" spans="1:7">
@@ -5777,16 +5786,16 @@
         <v>226</v>
       </c>
       <c r="B221" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C221" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="D221" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G221" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="222" spans="1:7">
@@ -5794,19 +5803,19 @@
         <v>227</v>
       </c>
       <c r="B222" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="C222" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D222" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E222" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="G222" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="223" spans="1:7">
@@ -5814,16 +5823,16 @@
         <v>228</v>
       </c>
       <c r="B223" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="C223" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D223" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G223" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="224" spans="1:7">
@@ -5831,16 +5840,16 @@
         <v>229</v>
       </c>
       <c r="B224" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C224" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D224" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="G224" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="225" spans="1:7">
@@ -5848,19 +5857,19 @@
         <v>230</v>
       </c>
       <c r="B225" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="C225" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D225" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="F225" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="G225" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="226" spans="1:7">
@@ -5868,16 +5877,16 @@
         <v>231</v>
       </c>
       <c r="B226" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C226" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D226" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="G226" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
     </row>
     <row r="227" spans="1:7">
@@ -5885,10 +5894,27 @@
         <v>232</v>
       </c>
       <c r="C227" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D227" t="s">
-        <v>438</v>
+        <v>441</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7">
+      <c r="A228" t="s">
+        <v>233</v>
+      </c>
+      <c r="B228" t="s">
+        <v>416</v>
+      </c>
+      <c r="C228" t="s">
+        <v>440</v>
+      </c>
+      <c r="D228" t="s">
+        <v>441</v>
+      </c>
+      <c r="G228" t="s">
+        <v>540</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove demo test files
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1159" uniqueCount="541">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1154" uniqueCount="538">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -715,9 +715,6 @@
     <t>Maties Underwater Club</t>
   </si>
   <si>
-    <t>Community Service Outreach Test</t>
-  </si>
-  <si>
     <t>info@ctsc.org.za</t>
   </si>
   <si>
@@ -1264,9 +1261,6 @@
     <t>info@capebirdclub.org.za</t>
   </si>
   <si>
-    <t>mrnnsu001@myuct.ac.za</t>
-  </si>
-  <si>
     <t>Museums &amp; Heritage</t>
   </si>
   <si>
@@ -1334,9 +1328,6 @@
   </si>
   <si>
     <t>Hobby &amp; Special Interest Clubs</t>
-  </si>
-  <si>
-    <t>Test</t>
   </si>
   <si>
     <t>Cape Town</t>
@@ -1981,7 +1972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G228"/>
+  <dimension ref="A1:G227"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2012,22 +2003,22 @@
         <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E2" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F2" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G2" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -2035,22 +2026,22 @@
         <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C3" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D3" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E3" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F3" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G3" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -2058,22 +2049,22 @@
         <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C4" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D4" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E4" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F4" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G4" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -2081,22 +2072,22 @@
         <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C5" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D5" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E5" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F5" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G5" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -2104,22 +2095,22 @@
         <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C6" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D6" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E6" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F6" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G6" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -2127,22 +2118,22 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C7" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D7" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E7" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F7" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G7" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -2150,22 +2141,22 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C8" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D8" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E8" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F8" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G8" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -2173,22 +2164,22 @@
         <v>14</v>
       </c>
       <c r="B9" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C9" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D9" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E9" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F9" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G9" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -2196,22 +2187,22 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C10" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D10" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E10" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F10" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G10" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -2219,22 +2210,22 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C11" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D11" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E11" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F11" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G11" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -2242,22 +2233,22 @@
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C12" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D12" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E12" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F12" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G12" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -2265,22 +2256,22 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C13" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D13" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E13" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
       <c r="F13" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
       <c r="G13" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -2288,22 +2279,22 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C14" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D14" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="E14" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="G14" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -2311,22 +2302,22 @@
         <v>20</v>
       </c>
       <c r="B15" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C15" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D15" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="E15" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>522</v>
+        <v>519</v>
       </c>
       <c r="G15" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -2334,16 +2325,16 @@
         <v>21</v>
       </c>
       <c r="B16" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C16" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D16" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G16" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -2351,16 +2342,16 @@
         <v>22</v>
       </c>
       <c r="B17" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C17" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D17" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G17" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -2368,16 +2359,16 @@
         <v>23</v>
       </c>
       <c r="B18" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C18" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D18" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G18" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -2385,16 +2376,16 @@
         <v>24</v>
       </c>
       <c r="B19" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C19" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D19" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G19" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -2402,16 +2393,16 @@
         <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C20" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D20" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G20" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -2419,16 +2410,16 @@
         <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C21" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D21" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G21" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -2436,16 +2427,16 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C22" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D22" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G22" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -2453,16 +2444,16 @@
         <v>28</v>
       </c>
       <c r="B23" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C23" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D23" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G23" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -2470,16 +2461,16 @@
         <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C24" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D24" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G24" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -2487,16 +2478,16 @@
         <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C25" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D25" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G25" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -2504,16 +2495,16 @@
         <v>31</v>
       </c>
       <c r="B26" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C26" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D26" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G26" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -2521,16 +2512,16 @@
         <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C27" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D27" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G27" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -2538,16 +2529,16 @@
         <v>33</v>
       </c>
       <c r="B28" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C28" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D28" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G28" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -2555,16 +2546,16 @@
         <v>34</v>
       </c>
       <c r="B29" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C29" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D29" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G29" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -2572,16 +2563,16 @@
         <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C30" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D30" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G30" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -2589,16 +2580,16 @@
         <v>36</v>
       </c>
       <c r="B31" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C31" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D31" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G31" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -2606,16 +2597,16 @@
         <v>37</v>
       </c>
       <c r="B32" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C32" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D32" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G32" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -2623,16 +2614,16 @@
         <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C33" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D33" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G33" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -2640,16 +2631,16 @@
         <v>39</v>
       </c>
       <c r="B34" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C34" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D34" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G34" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -2657,16 +2648,16 @@
         <v>40</v>
       </c>
       <c r="B35" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C35" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D35" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G35" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -2674,16 +2665,16 @@
         <v>41</v>
       </c>
       <c r="B36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C36" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D36" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G36" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -2691,16 +2682,16 @@
         <v>42</v>
       </c>
       <c r="B37" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C37" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D37" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G37" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -2708,16 +2699,16 @@
         <v>43</v>
       </c>
       <c r="B38" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C38" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D38" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G38" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -2725,16 +2716,16 @@
         <v>44</v>
       </c>
       <c r="B39" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C39" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D39" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G39" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -2742,16 +2733,16 @@
         <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C40" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D40" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G40" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -2759,16 +2750,16 @@
         <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C41" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D41" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G41" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -2776,16 +2767,16 @@
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C42" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D42" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G42" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -2793,16 +2784,16 @@
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C43" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D43" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G43" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -2810,16 +2801,16 @@
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C44" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D44" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G44" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -2827,16 +2818,16 @@
         <v>50</v>
       </c>
       <c r="B45" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C45" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D45" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G45" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -2844,16 +2835,16 @@
         <v>51</v>
       </c>
       <c r="B46" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C46" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D46" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G46" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -2861,16 +2852,16 @@
         <v>52</v>
       </c>
       <c r="B47" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C47" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D47" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G47" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -2878,16 +2869,16 @@
         <v>53</v>
       </c>
       <c r="B48" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C48" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D48" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G48" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -2895,16 +2886,16 @@
         <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C49" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D49" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G49" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -2912,16 +2903,16 @@
         <v>55</v>
       </c>
       <c r="B50" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C50" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D50" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G50" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -2929,16 +2920,16 @@
         <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C51" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D51" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G51" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -2946,16 +2937,16 @@
         <v>57</v>
       </c>
       <c r="B52" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C52" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D52" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G52" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -2963,16 +2954,16 @@
         <v>58</v>
       </c>
       <c r="B53" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C53" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D53" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G53" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -2980,16 +2971,16 @@
         <v>59</v>
       </c>
       <c r="B54" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C54" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D54" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G54" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -2997,16 +2988,16 @@
         <v>60</v>
       </c>
       <c r="B55" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C55" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D55" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G55" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -3014,16 +3005,16 @@
         <v>61</v>
       </c>
       <c r="B56" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C56" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D56" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G56" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -3031,16 +3022,16 @@
         <v>62</v>
       </c>
       <c r="B57" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C57" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D57" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G57" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -3048,16 +3039,16 @@
         <v>63</v>
       </c>
       <c r="B58" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C58" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D58" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G58" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -3065,16 +3056,16 @@
         <v>64</v>
       </c>
       <c r="B59" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C59" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D59" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G59" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -3082,16 +3073,16 @@
         <v>65</v>
       </c>
       <c r="B60" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C60" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D60" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G60" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -3099,16 +3090,16 @@
         <v>66</v>
       </c>
       <c r="B61" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C61" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D61" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G61" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -3116,16 +3107,16 @@
         <v>67</v>
       </c>
       <c r="B62" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C62" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D62" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G62" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -3133,16 +3124,16 @@
         <v>68</v>
       </c>
       <c r="B63" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C63" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D63" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G63" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -3150,16 +3141,16 @@
         <v>69</v>
       </c>
       <c r="B64" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C64" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D64" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G64" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -3167,16 +3158,16 @@
         <v>70</v>
       </c>
       <c r="B65" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C65" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D65" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G65" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -3184,16 +3175,16 @@
         <v>71</v>
       </c>
       <c r="B66" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C66" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D66" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G66" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -3201,16 +3192,16 @@
         <v>72</v>
       </c>
       <c r="B67" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C67" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D67" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G67" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -3218,16 +3209,16 @@
         <v>73</v>
       </c>
       <c r="B68" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C68" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D68" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G68" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -3235,16 +3226,16 @@
         <v>74</v>
       </c>
       <c r="B69" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C69" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D69" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G69" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -3252,16 +3243,16 @@
         <v>75</v>
       </c>
       <c r="B70" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C70" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D70" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G70" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -3269,16 +3260,16 @@
         <v>76</v>
       </c>
       <c r="B71" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C71" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D71" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G71" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -3286,16 +3277,16 @@
         <v>77</v>
       </c>
       <c r="B72" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C72" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D72" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G72" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -3303,16 +3294,16 @@
         <v>78</v>
       </c>
       <c r="B73" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C73" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D73" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G73" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -3320,16 +3311,16 @@
         <v>79</v>
       </c>
       <c r="B74" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C74" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="D74" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G74" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -3337,16 +3328,16 @@
         <v>80</v>
       </c>
       <c r="B75" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C75" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D75" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G75" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="76" spans="1:7">
@@ -3354,16 +3345,16 @@
         <v>81</v>
       </c>
       <c r="B76" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C76" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D76" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G76" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -3371,16 +3362,16 @@
         <v>82</v>
       </c>
       <c r="B77" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C77" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D77" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G77" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -3388,16 +3379,16 @@
         <v>83</v>
       </c>
       <c r="B78" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C78" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D78" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G78" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="79" spans="1:7">
@@ -3405,16 +3396,16 @@
         <v>84</v>
       </c>
       <c r="B79" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C79" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D79" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G79" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -3422,16 +3413,16 @@
         <v>85</v>
       </c>
       <c r="B80" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C80" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D80" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G80" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -3439,16 +3430,16 @@
         <v>86</v>
       </c>
       <c r="B81" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C81" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D81" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G81" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -3456,16 +3447,16 @@
         <v>87</v>
       </c>
       <c r="B82" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C82" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D82" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G82" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -3473,16 +3464,16 @@
         <v>88</v>
       </c>
       <c r="B83" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C83" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D83" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G83" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -3490,16 +3481,16 @@
         <v>89</v>
       </c>
       <c r="B84" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C84" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D84" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G84" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -3507,16 +3498,16 @@
         <v>90</v>
       </c>
       <c r="B85" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C85" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D85" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G85" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -3524,16 +3515,16 @@
         <v>91</v>
       </c>
       <c r="B86" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C86" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D86" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G86" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -3541,16 +3532,16 @@
         <v>92</v>
       </c>
       <c r="B87" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C87" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D87" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G87" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -3558,16 +3549,16 @@
         <v>93</v>
       </c>
       <c r="B88" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C88" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D88" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G88" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -3575,16 +3566,16 @@
         <v>94</v>
       </c>
       <c r="B89" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C89" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="D89" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G89" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="90" spans="1:7">
@@ -3592,16 +3583,16 @@
         <v>95</v>
       </c>
       <c r="B90" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C90" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D90" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G90" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -3609,16 +3600,16 @@
         <v>96</v>
       </c>
       <c r="B91" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C91" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D91" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G91" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -3626,16 +3617,16 @@
         <v>97</v>
       </c>
       <c r="B92" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C92" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D92" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G92" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="93" spans="1:7">
@@ -3643,16 +3634,16 @@
         <v>98</v>
       </c>
       <c r="B93" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C93" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D93" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G93" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -3660,16 +3651,16 @@
         <v>99</v>
       </c>
       <c r="B94" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C94" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D94" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G94" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -3677,16 +3668,16 @@
         <v>100</v>
       </c>
       <c r="B95" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C95" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D95" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G95" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -3694,16 +3685,16 @@
         <v>101</v>
       </c>
       <c r="B96" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C96" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D96" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G96" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -3711,16 +3702,16 @@
         <v>102</v>
       </c>
       <c r="B97" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C97" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D97" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G97" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -3728,16 +3719,16 @@
         <v>103</v>
       </c>
       <c r="B98" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C98" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D98" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G98" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="99" spans="1:7">
@@ -3745,16 +3736,16 @@
         <v>104</v>
       </c>
       <c r="B99" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C99" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D99" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G99" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="100" spans="1:7">
@@ -3762,16 +3753,16 @@
         <v>105</v>
       </c>
       <c r="B100" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C100" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D100" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G100" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="101" spans="1:7">
@@ -3779,16 +3770,16 @@
         <v>106</v>
       </c>
       <c r="B101" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C101" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D101" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G101" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="102" spans="1:7">
@@ -3796,16 +3787,16 @@
         <v>107</v>
       </c>
       <c r="B102" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C102" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D102" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G102" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="103" spans="1:7">
@@ -3813,16 +3804,16 @@
         <v>108</v>
       </c>
       <c r="B103" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C103" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D103" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G103" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="104" spans="1:7">
@@ -3830,16 +3821,16 @@
         <v>109</v>
       </c>
       <c r="B104" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C104" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D104" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G104" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="105" spans="1:7">
@@ -3847,16 +3838,16 @@
         <v>110</v>
       </c>
       <c r="B105" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C105" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D105" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G105" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="106" spans="1:7">
@@ -3864,16 +3855,16 @@
         <v>111</v>
       </c>
       <c r="B106" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C106" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D106" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G106" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="107" spans="1:7">
@@ -3881,16 +3872,16 @@
         <v>112</v>
       </c>
       <c r="B107" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C107" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D107" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G107" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="108" spans="1:7">
@@ -3898,16 +3889,16 @@
         <v>113</v>
       </c>
       <c r="B108" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C108" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D108" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G108" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="109" spans="1:7">
@@ -3915,16 +3906,16 @@
         <v>114</v>
       </c>
       <c r="B109" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C109" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D109" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G109" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="110" spans="1:7">
@@ -3932,16 +3923,16 @@
         <v>115</v>
       </c>
       <c r="B110" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C110" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D110" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G110" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="111" spans="1:7">
@@ -3949,16 +3940,16 @@
         <v>116</v>
       </c>
       <c r="B111" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C111" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D111" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G111" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="112" spans="1:7">
@@ -3966,16 +3957,16 @@
         <v>117</v>
       </c>
       <c r="B112" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C112" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D112" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G112" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="113" spans="1:7">
@@ -3983,16 +3974,16 @@
         <v>118</v>
       </c>
       <c r="B113" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C113" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D113" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G113" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="114" spans="1:7">
@@ -4000,16 +3991,16 @@
         <v>119</v>
       </c>
       <c r="B114" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C114" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D114" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G114" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="115" spans="1:7">
@@ -4017,16 +4008,16 @@
         <v>120</v>
       </c>
       <c r="B115" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C115" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D115" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G115" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="116" spans="1:7">
@@ -4034,16 +4025,16 @@
         <v>121</v>
       </c>
       <c r="B116" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="C116" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D116" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G116" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="117" spans="1:7">
@@ -4051,16 +4042,16 @@
         <v>122</v>
       </c>
       <c r="B117" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C117" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D117" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G117" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="118" spans="1:7">
@@ -4068,16 +4059,16 @@
         <v>123</v>
       </c>
       <c r="B118" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C118" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D118" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G118" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -4085,22 +4076,22 @@
         <v>124</v>
       </c>
       <c r="B119" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C119" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D119" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E119" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
       <c r="F119" t="s">
-        <v>523</v>
+        <v>520</v>
       </c>
       <c r="G119" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="120" spans="1:7">
@@ -4108,19 +4099,19 @@
         <v>125</v>
       </c>
       <c r="B120" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C120" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D120" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
       <c r="E120" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="G120" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="121" spans="1:7">
@@ -4128,16 +4119,16 @@
         <v>126</v>
       </c>
       <c r="B121" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C121" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D121" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G121" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -4145,16 +4136,16 @@
         <v>127</v>
       </c>
       <c r="B122" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C122" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D122" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="G122" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="123" spans="1:7">
@@ -4162,22 +4153,22 @@
         <v>128</v>
       </c>
       <c r="B123" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C123" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D123" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E123" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="F123" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="G123" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="124" spans="1:7">
@@ -4185,16 +4176,16 @@
         <v>129</v>
       </c>
       <c r="B124" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C124" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D124" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G124" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="125" spans="1:7">
@@ -4202,16 +4193,16 @@
         <v>130</v>
       </c>
       <c r="B125" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C125" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D125" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G125" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -4219,16 +4210,16 @@
         <v>131</v>
       </c>
       <c r="B126" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C126" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D126" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G126" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="127" spans="1:7">
@@ -4236,16 +4227,16 @@
         <v>132</v>
       </c>
       <c r="B127" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C127" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D127" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G127" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="128" spans="1:7">
@@ -4253,19 +4244,19 @@
         <v>133</v>
       </c>
       <c r="B128" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C128" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D128" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="E128" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
       <c r="G128" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="129" spans="1:7">
@@ -4273,22 +4264,22 @@
         <v>134</v>
       </c>
       <c r="B129" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C129" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D129" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E129" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="F129" t="s">
-        <v>525</v>
+        <v>522</v>
       </c>
       <c r="G129" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="130" spans="1:7">
@@ -4296,16 +4287,16 @@
         <v>135</v>
       </c>
       <c r="B130" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="C130" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D130" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G130" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="131" spans="1:7">
@@ -4313,13 +4304,13 @@
         <v>136</v>
       </c>
       <c r="C131" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D131" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="E131" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
     </row>
     <row r="132" spans="1:7">
@@ -4327,19 +4318,19 @@
         <v>137</v>
       </c>
       <c r="B132" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="C132" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D132" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="E132" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="G132" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="133" spans="1:7">
@@ -4347,19 +4338,19 @@
         <v>138</v>
       </c>
       <c r="B133" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C133" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D133" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
       <c r="E133" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
       <c r="G133" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="134" spans="1:7">
@@ -4367,10 +4358,10 @@
         <v>139</v>
       </c>
       <c r="C134" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D134" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="135" spans="1:7">
@@ -4378,10 +4369,10 @@
         <v>140</v>
       </c>
       <c r="C135" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="D135" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="136" spans="1:7">
@@ -4389,16 +4380,16 @@
         <v>141</v>
       </c>
       <c r="B136" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C136" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D136" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G136" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="137" spans="1:7">
@@ -4406,16 +4397,16 @@
         <v>142</v>
       </c>
       <c r="B137" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C137" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D137" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="G137" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="138" spans="1:7">
@@ -4423,10 +4414,10 @@
         <v>143</v>
       </c>
       <c r="C138" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D138" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
     </row>
     <row r="139" spans="1:7">
@@ -4434,10 +4425,10 @@
         <v>144</v>
       </c>
       <c r="C139" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D139" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
     <row r="140" spans="1:7">
@@ -4445,10 +4436,10 @@
         <v>145</v>
       </c>
       <c r="C140" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D140" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="141" spans="1:7">
@@ -4456,16 +4447,16 @@
         <v>146</v>
       </c>
       <c r="B141" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C141" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D141" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G141" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="142" spans="1:7">
@@ -4473,22 +4464,22 @@
         <v>147</v>
       </c>
       <c r="B142" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="C142" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="D142" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E142" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
       <c r="F142" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="G142" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="143" spans="1:7">
@@ -4496,16 +4487,16 @@
         <v>148</v>
       </c>
       <c r="B143" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="C143" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D143" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="G143" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="144" spans="1:7">
@@ -4513,13 +4504,13 @@
         <v>149</v>
       </c>
       <c r="C144" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D144" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="E144" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
     </row>
     <row r="145" spans="1:7">
@@ -4527,10 +4518,10 @@
         <v>150</v>
       </c>
       <c r="C145" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D145" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="146" spans="1:7">
@@ -4538,19 +4529,19 @@
         <v>151</v>
       </c>
       <c r="B146" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="C146" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D146" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F146" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
       <c r="G146" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="147" spans="1:7">
@@ -4558,22 +4549,22 @@
         <v>152</v>
       </c>
       <c r="B147" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="C147" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D147" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E147" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="F147" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="G147" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="148" spans="1:7">
@@ -4581,19 +4572,19 @@
         <v>153</v>
       </c>
       <c r="B148" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="C148" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D148" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E148" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="G148" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="149" spans="1:7">
@@ -4601,19 +4592,19 @@
         <v>154</v>
       </c>
       <c r="B149" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="C149" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D149" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E149" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="G149" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="150" spans="1:7">
@@ -4621,19 +4612,19 @@
         <v>155</v>
       </c>
       <c r="B150" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="C150" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D150" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E150" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="G150" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="151" spans="1:7">
@@ -4641,19 +4632,19 @@
         <v>156</v>
       </c>
       <c r="B151" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="C151" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D151" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E151" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="G151" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="152" spans="1:7">
@@ -4661,19 +4652,19 @@
         <v>157</v>
       </c>
       <c r="B152" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C152" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D152" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E152" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
       <c r="G152" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="153" spans="1:7">
@@ -4681,10 +4672,10 @@
         <v>158</v>
       </c>
       <c r="C153" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D153" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="154" spans="1:7">
@@ -4692,19 +4683,19 @@
         <v>159</v>
       </c>
       <c r="B154" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="C154" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D154" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E154" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="G154" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="155" spans="1:7">
@@ -4712,16 +4703,16 @@
         <v>160</v>
       </c>
       <c r="B155" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="C155" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D155" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G155" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="156" spans="1:7">
@@ -4729,16 +4720,16 @@
         <v>161</v>
       </c>
       <c r="B156" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C156" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D156" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G156" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="157" spans="1:7">
@@ -4746,22 +4737,22 @@
         <v>162</v>
       </c>
       <c r="B157" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C157" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D157" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="E157" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="F157" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="G157" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="158" spans="1:7">
@@ -4769,19 +4760,19 @@
         <v>163</v>
       </c>
       <c r="B158" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C158" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D158" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E158" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="G158" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="159" spans="1:7">
@@ -4789,19 +4780,19 @@
         <v>164</v>
       </c>
       <c r="B159" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C159" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D159" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E159" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="G159" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="160" spans="1:7">
@@ -4809,19 +4800,19 @@
         <v>165</v>
       </c>
       <c r="B160" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C160" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D160" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E160" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="G160" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="161" spans="1:7">
@@ -4829,19 +4820,19 @@
         <v>166</v>
       </c>
       <c r="B161" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C161" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D161" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="E161" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="G161" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="162" spans="1:7">
@@ -4849,16 +4840,16 @@
         <v>167</v>
       </c>
       <c r="B162" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="C162" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D162" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G162" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="163" spans="1:7">
@@ -4866,19 +4857,19 @@
         <v>168</v>
       </c>
       <c r="B163" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C163" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D163" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E163" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
       <c r="G163" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="164" spans="1:7">
@@ -4886,19 +4877,19 @@
         <v>169</v>
       </c>
       <c r="B164" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="C164" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D164" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="E164" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="G164" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="165" spans="1:7">
@@ -4906,13 +4897,13 @@
         <v>170</v>
       </c>
       <c r="C165" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D165" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="E165" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="166" spans="1:7">
@@ -4920,19 +4911,19 @@
         <v>171</v>
       </c>
       <c r="B166" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C166" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D166" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="E166" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="G166" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="167" spans="1:7">
@@ -4940,19 +4931,19 @@
         <v>172</v>
       </c>
       <c r="B167" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="C167" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D167" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
       <c r="E167" t="s">
-        <v>495</v>
+        <v>492</v>
       </c>
       <c r="G167" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -4960,19 +4951,19 @@
         <v>173</v>
       </c>
       <c r="B168" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="C168" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D168" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E168" t="s">
-        <v>496</v>
+        <v>493</v>
       </c>
       <c r="G168" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="169" spans="1:7">
@@ -4980,19 +4971,19 @@
         <v>174</v>
       </c>
       <c r="B169" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="C169" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D169" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
       <c r="E169" t="s">
-        <v>497</v>
+        <v>494</v>
       </c>
       <c r="G169" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="170" spans="1:7">
@@ -5000,13 +4991,13 @@
         <v>175</v>
       </c>
       <c r="C170" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D170" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="E170" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="171" spans="1:7">
@@ -5014,13 +5005,13 @@
         <v>176</v>
       </c>
       <c r="C171" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D171" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E171" t="s">
-        <v>499</v>
+        <v>496</v>
       </c>
     </row>
     <row r="172" spans="1:7">
@@ -5028,13 +5019,13 @@
         <v>177</v>
       </c>
       <c r="C172" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="D172" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="E172" t="s">
-        <v>500</v>
+        <v>497</v>
       </c>
     </row>
     <row r="173" spans="1:7">
@@ -5042,16 +5033,16 @@
         <v>178</v>
       </c>
       <c r="B173" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="C173" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D173" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G173" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="174" spans="1:7">
@@ -5059,19 +5050,19 @@
         <v>179</v>
       </c>
       <c r="B174" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="C174" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D174" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F174" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="G174" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="175" spans="1:7">
@@ -5079,19 +5070,19 @@
         <v>180</v>
       </c>
       <c r="B175" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="C175" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="D175" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F175" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="G175" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="176" spans="1:7">
@@ -5099,10 +5090,10 @@
         <v>181</v>
       </c>
       <c r="C176" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D176" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="177" spans="1:7">
@@ -5110,10 +5101,10 @@
         <v>182</v>
       </c>
       <c r="C177" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D177" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="178" spans="1:7">
@@ -5121,10 +5112,10 @@
         <v>183</v>
       </c>
       <c r="C178" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D178" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="179" spans="1:7">
@@ -5132,22 +5123,22 @@
         <v>184</v>
       </c>
       <c r="B179" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="C179" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D179" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
       <c r="E179" t="s">
-        <v>501</v>
+        <v>498</v>
       </c>
       <c r="F179" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="G179" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="180" spans="1:7">
@@ -5155,10 +5146,10 @@
         <v>185</v>
       </c>
       <c r="C180" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D180" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="181" spans="1:7">
@@ -5166,10 +5157,10 @@
         <v>186</v>
       </c>
       <c r="C181" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D181" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="182" spans="1:7">
@@ -5177,19 +5168,19 @@
         <v>187</v>
       </c>
       <c r="B182" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="C182" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D182" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E182" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="G182" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="183" spans="1:7">
@@ -5197,19 +5188,19 @@
         <v>188</v>
       </c>
       <c r="B183" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="C183" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D183" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F183" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="G183" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="184" spans="1:7">
@@ -5217,10 +5208,10 @@
         <v>189</v>
       </c>
       <c r="C184" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D184" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="185" spans="1:7">
@@ -5228,13 +5219,13 @@
         <v>190</v>
       </c>
       <c r="C185" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D185" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="F185" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
     </row>
     <row r="186" spans="1:7">
@@ -5242,13 +5233,13 @@
         <v>191</v>
       </c>
       <c r="C186" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D186" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="E186" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="187" spans="1:7">
@@ -5256,13 +5247,13 @@
         <v>192</v>
       </c>
       <c r="C187" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D187" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E187" t="s">
-        <v>504</v>
+        <v>501</v>
       </c>
     </row>
     <row r="188" spans="1:7">
@@ -5270,13 +5261,13 @@
         <v>193</v>
       </c>
       <c r="C188" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D188" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E188" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
     </row>
     <row r="189" spans="1:7">
@@ -5284,13 +5275,13 @@
         <v>194</v>
       </c>
       <c r="C189" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D189" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E189" t="s">
-        <v>506</v>
+        <v>503</v>
       </c>
     </row>
     <row r="190" spans="1:7">
@@ -5298,13 +5289,13 @@
         <v>195</v>
       </c>
       <c r="C190" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D190" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E190" t="s">
-        <v>507</v>
+        <v>504</v>
       </c>
     </row>
     <row r="191" spans="1:7">
@@ -5312,10 +5303,10 @@
         <v>196</v>
       </c>
       <c r="C191" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D191" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="192" spans="1:7">
@@ -5323,10 +5314,10 @@
         <v>197</v>
       </c>
       <c r="C192" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D192" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="193" spans="1:7">
@@ -5334,10 +5325,10 @@
         <v>198</v>
       </c>
       <c r="C193" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D193" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="194" spans="1:7">
@@ -5345,16 +5336,16 @@
         <v>199</v>
       </c>
       <c r="B194" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C194" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D194" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="G194" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="195" spans="1:7">
@@ -5362,16 +5353,16 @@
         <v>200</v>
       </c>
       <c r="B195" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C195" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D195" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="G195" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="196" spans="1:7">
@@ -5379,19 +5370,19 @@
         <v>201</v>
       </c>
       <c r="B196" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C196" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D196" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F196" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="G196" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="197" spans="1:7">
@@ -5399,22 +5390,22 @@
         <v>202</v>
       </c>
       <c r="B197" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="C197" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D197" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E197" t="s">
-        <v>508</v>
+        <v>505</v>
       </c>
       <c r="F197" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="G197" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="198" spans="1:7">
@@ -5422,22 +5413,22 @@
         <v>203</v>
       </c>
       <c r="B198" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C198" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D198" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E198" t="s">
-        <v>509</v>
+        <v>506</v>
       </c>
       <c r="F198" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="G198" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="199" spans="1:7">
@@ -5445,22 +5436,22 @@
         <v>204</v>
       </c>
       <c r="B199" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="C199" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D199" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E199" t="s">
-        <v>510</v>
+        <v>507</v>
       </c>
       <c r="F199" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="G199" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="200" spans="1:7">
@@ -5468,16 +5459,16 @@
         <v>205</v>
       </c>
       <c r="B200" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="C200" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D200" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G200" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="201" spans="1:7">
@@ -5485,10 +5476,10 @@
         <v>206</v>
       </c>
       <c r="C201" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D201" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="202" spans="1:7">
@@ -5496,10 +5487,10 @@
         <v>207</v>
       </c>
       <c r="C202" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D202" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="203" spans="1:7">
@@ -5507,10 +5498,10 @@
         <v>208</v>
       </c>
       <c r="C203" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D203" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="204" spans="1:7">
@@ -5518,16 +5509,16 @@
         <v>209</v>
       </c>
       <c r="B204" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C204" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D204" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G204" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="205" spans="1:7">
@@ -5535,10 +5526,10 @@
         <v>210</v>
       </c>
       <c r="C205" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D205" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="206" spans="1:7">
@@ -5546,10 +5537,10 @@
         <v>211</v>
       </c>
       <c r="C206" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D206" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="207" spans="1:7">
@@ -5557,19 +5548,19 @@
         <v>212</v>
       </c>
       <c r="B207" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C207" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D207" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E207" t="s">
-        <v>511</v>
+        <v>508</v>
       </c>
       <c r="G207" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="208" spans="1:7">
@@ -5577,13 +5568,13 @@
         <v>213</v>
       </c>
       <c r="C208" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D208" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E208" t="s">
-        <v>512</v>
+        <v>509</v>
       </c>
     </row>
     <row r="209" spans="1:7">
@@ -5591,10 +5582,10 @@
         <v>214</v>
       </c>
       <c r="C209" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="D209" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
     </row>
     <row r="210" spans="1:7">
@@ -5602,19 +5593,19 @@
         <v>215</v>
       </c>
       <c r="B210" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C210" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D210" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E210" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
       <c r="G210" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="211" spans="1:7">
@@ -5622,16 +5613,16 @@
         <v>216</v>
       </c>
       <c r="B211" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="C211" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D211" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G211" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="212" spans="1:7">
@@ -5639,13 +5630,13 @@
         <v>217</v>
       </c>
       <c r="C212" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D212" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E212" t="s">
-        <v>514</v>
+        <v>511</v>
       </c>
     </row>
     <row r="213" spans="1:7">
@@ -5653,13 +5644,13 @@
         <v>218</v>
       </c>
       <c r="C213" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D213" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="E213" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
     </row>
     <row r="214" spans="1:7">
@@ -5667,16 +5658,16 @@
         <v>219</v>
       </c>
       <c r="B214" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C214" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D214" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G214" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="215" spans="1:7">
@@ -5684,16 +5675,16 @@
         <v>220</v>
       </c>
       <c r="B215" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="C215" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D215" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G215" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="216" spans="1:7">
@@ -5701,13 +5692,13 @@
         <v>221</v>
       </c>
       <c r="C216" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="D216" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E216" t="s">
-        <v>516</v>
+        <v>513</v>
       </c>
     </row>
     <row r="217" spans="1:7">
@@ -5715,19 +5706,19 @@
         <v>222</v>
       </c>
       <c r="B217" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C217" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="D217" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E217" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="G217" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="218" spans="1:7">
@@ -5735,19 +5726,19 @@
         <v>223</v>
       </c>
       <c r="B218" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="C218" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="D218" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E218" t="s">
-        <v>517</v>
+        <v>514</v>
       </c>
       <c r="G218" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="219" spans="1:7">
@@ -5755,19 +5746,19 @@
         <v>224</v>
       </c>
       <c r="B219" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C219" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D219" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E219" t="s">
-        <v>518</v>
+        <v>515</v>
       </c>
       <c r="G219" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="220" spans="1:7">
@@ -5775,10 +5766,10 @@
         <v>225</v>
       </c>
       <c r="C220" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D220" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="221" spans="1:7">
@@ -5786,16 +5777,16 @@
         <v>226</v>
       </c>
       <c r="B221" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="C221" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D221" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G221" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="222" spans="1:7">
@@ -5803,19 +5794,19 @@
         <v>227</v>
       </c>
       <c r="B222" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C222" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D222" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="E222" t="s">
-        <v>519</v>
+        <v>516</v>
       </c>
       <c r="G222" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="223" spans="1:7">
@@ -5823,16 +5814,16 @@
         <v>228</v>
       </c>
       <c r="B223" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="C223" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D223" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G223" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="224" spans="1:7">
@@ -5840,16 +5831,16 @@
         <v>229</v>
       </c>
       <c r="B224" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="C224" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D224" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
       <c r="G224" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="225" spans="1:7">
@@ -5857,19 +5848,19 @@
         <v>230</v>
       </c>
       <c r="B225" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="C225" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D225" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="F225" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="G225" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="226" spans="1:7">
@@ -5877,16 +5868,16 @@
         <v>231</v>
       </c>
       <c r="B226" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="C226" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D226" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
       <c r="G226" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
     </row>
     <row r="227" spans="1:7">
@@ -5894,27 +5885,10 @@
         <v>232</v>
       </c>
       <c r="C227" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="D227" t="s">
-        <v>441</v>
-      </c>
-    </row>
-    <row r="228" spans="1:7">
-      <c r="A228" t="s">
-        <v>233</v>
-      </c>
-      <c r="B228" t="s">
-        <v>416</v>
-      </c>
-      <c r="C228" t="s">
-        <v>440</v>
-      </c>
-      <c r="D228" t="s">
-        <v>441</v>
-      </c>
-      <c r="G228" t="s">
-        <v>540</v>
+        <v>438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync Mowbray sent status 2026-10-07-1728
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1424" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="654">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -7034,6 +7034,9 @@
       <c r="D274" t="s">
         <v>577</v>
       </c>
+      <c r="G274" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="275" spans="1:7">
       <c r="A275" t="s">

</xml_diff>

<commit_message>
Queue contacts for tomorrow 06:15 SAST send 2026-10-07-1753
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="653">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -1973,9 +1973,6 @@
   </si>
   <si>
     <t>www.cmacofct.com</t>
-  </si>
-  <si>
-    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -2365,9 +2362,6 @@
       <c r="F2" t="s">
         <v>633</v>
       </c>
-      <c r="G2" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
@@ -2388,9 +2382,6 @@
       <c r="F3" t="s">
         <v>633</v>
       </c>
-      <c r="G3" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -2411,9 +2402,6 @@
       <c r="F4" t="s">
         <v>633</v>
       </c>
-      <c r="G4" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -2434,9 +2422,6 @@
       <c r="F5" t="s">
         <v>633</v>
       </c>
-      <c r="G5" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -2457,9 +2442,6 @@
       <c r="F6" t="s">
         <v>633</v>
       </c>
-      <c r="G6" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -2480,9 +2462,6 @@
       <c r="F7" t="s">
         <v>633</v>
       </c>
-      <c r="G7" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -2503,9 +2482,6 @@
       <c r="F8" t="s">
         <v>633</v>
       </c>
-      <c r="G8" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -2526,9 +2502,6 @@
       <c r="F9" t="s">
         <v>633</v>
       </c>
-      <c r="G9" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -2549,9 +2522,6 @@
       <c r="F10" t="s">
         <v>633</v>
       </c>
-      <c r="G10" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -2572,9 +2542,6 @@
       <c r="F11" t="s">
         <v>633</v>
       </c>
-      <c r="G11" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
@@ -2595,9 +2562,6 @@
       <c r="F12" t="s">
         <v>633</v>
       </c>
-      <c r="G12" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
@@ -2618,9 +2582,6 @@
       <c r="F13" t="s">
         <v>633</v>
       </c>
-      <c r="G13" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
@@ -2641,9 +2602,6 @@
       <c r="F14" s="1" t="s">
         <v>634</v>
       </c>
-      <c r="G14" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
@@ -2664,9 +2622,6 @@
       <c r="F15" s="1" t="s">
         <v>635</v>
       </c>
-      <c r="G15" t="s">
-        <v>653</v>
-      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
@@ -2681,11 +2636,8 @@
       <c r="D16" t="s">
         <v>552</v>
       </c>
-      <c r="G16" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -2698,11 +2650,8 @@
       <c r="D17" t="s">
         <v>552</v>
       </c>
-      <c r="G17" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -2715,11 +2664,8 @@
       <c r="D18" t="s">
         <v>552</v>
       </c>
-      <c r="G18" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -2732,11 +2678,8 @@
       <c r="D19" t="s">
         <v>552</v>
       </c>
-      <c r="G19" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -2749,11 +2692,8 @@
       <c r="D20" t="s">
         <v>552</v>
       </c>
-      <c r="G20" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -2766,11 +2706,8 @@
       <c r="D21" t="s">
         <v>552</v>
       </c>
-      <c r="G21" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -2783,11 +2720,8 @@
       <c r="D22" t="s">
         <v>552</v>
       </c>
-      <c r="G22" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -2800,11 +2734,8 @@
       <c r="D23" t="s">
         <v>552</v>
       </c>
-      <c r="G23" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -2817,11 +2748,8 @@
       <c r="D24" t="s">
         <v>552</v>
       </c>
-      <c r="G24" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -2834,11 +2762,8 @@
       <c r="D25" t="s">
         <v>552</v>
       </c>
-      <c r="G25" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -2851,11 +2776,8 @@
       <c r="D26" t="s">
         <v>552</v>
       </c>
-      <c r="G26" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -2868,11 +2790,8 @@
       <c r="D27" t="s">
         <v>552</v>
       </c>
-      <c r="G27" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -2885,11 +2804,8 @@
       <c r="D28" t="s">
         <v>552</v>
       </c>
-      <c r="G28" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -2902,11 +2818,8 @@
       <c r="D29" t="s">
         <v>552</v>
       </c>
-      <c r="G29" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -2919,11 +2832,8 @@
       <c r="D30" t="s">
         <v>552</v>
       </c>
-      <c r="G30" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -2936,11 +2846,8 @@
       <c r="D31" t="s">
         <v>552</v>
       </c>
-      <c r="G31" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -2953,11 +2860,8 @@
       <c r="D32" t="s">
         <v>552</v>
       </c>
-      <c r="G32" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -2970,11 +2874,8 @@
       <c r="D33" t="s">
         <v>552</v>
       </c>
-      <c r="G33" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -2987,11 +2888,8 @@
       <c r="D34" t="s">
         <v>552</v>
       </c>
-      <c r="G34" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -3004,11 +2902,8 @@
       <c r="D35" t="s">
         <v>552</v>
       </c>
-      <c r="G35" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -3021,11 +2916,8 @@
       <c r="D36" t="s">
         <v>552</v>
       </c>
-      <c r="G36" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -3038,11 +2930,8 @@
       <c r="D37" t="s">
         <v>552</v>
       </c>
-      <c r="G37" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -3055,11 +2944,8 @@
       <c r="D38" t="s">
         <v>552</v>
       </c>
-      <c r="G38" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -3072,11 +2958,8 @@
       <c r="D39" t="s">
         <v>552</v>
       </c>
-      <c r="G39" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+    </row>
+    <row r="40" spans="1:4">
       <c r="A40" t="s">
         <v>45</v>
       </c>
@@ -3089,11 +2972,8 @@
       <c r="D40" t="s">
         <v>552</v>
       </c>
-      <c r="G40" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41" t="s">
         <v>46</v>
       </c>
@@ -3106,11 +2986,8 @@
       <c r="D41" t="s">
         <v>552</v>
       </c>
-      <c r="G41" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -3123,11 +3000,8 @@
       <c r="D42" t="s">
         <v>552</v>
       </c>
-      <c r="G42" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
+    </row>
+    <row r="43" spans="1:4">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -3140,11 +3014,8 @@
       <c r="D43" t="s">
         <v>552</v>
       </c>
-      <c r="G43" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -3157,11 +3028,8 @@
       <c r="D44" t="s">
         <v>552</v>
       </c>
-      <c r="G44" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -3174,11 +3042,8 @@
       <c r="D45" t="s">
         <v>552</v>
       </c>
-      <c r="G45" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -3191,11 +3056,8 @@
       <c r="D46" t="s">
         <v>552</v>
       </c>
-      <c r="G46" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -3208,11 +3070,8 @@
       <c r="D47" t="s">
         <v>552</v>
       </c>
-      <c r="G47" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -3225,11 +3084,8 @@
       <c r="D48" t="s">
         <v>552</v>
       </c>
-      <c r="G48" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
+    </row>
+    <row r="49" spans="1:4">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -3242,11 +3098,8 @@
       <c r="D49" t="s">
         <v>552</v>
       </c>
-      <c r="G49" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -3259,11 +3112,8 @@
       <c r="D50" t="s">
         <v>552</v>
       </c>
-      <c r="G50" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7">
+    </row>
+    <row r="51" spans="1:4">
       <c r="A51" t="s">
         <v>56</v>
       </c>
@@ -3276,11 +3126,8 @@
       <c r="D51" t="s">
         <v>552</v>
       </c>
-      <c r="G51" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
+    </row>
+    <row r="52" spans="1:4">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -3293,11 +3140,8 @@
       <c r="D52" t="s">
         <v>552</v>
       </c>
-      <c r="G52" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7">
+    </row>
+    <row r="53" spans="1:4">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -3310,11 +3154,8 @@
       <c r="D53" t="s">
         <v>552</v>
       </c>
-      <c r="G53" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7">
+    </row>
+    <row r="54" spans="1:4">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -3327,11 +3168,8 @@
       <c r="D54" t="s">
         <v>552</v>
       </c>
-      <c r="G54" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7">
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55" t="s">
         <v>60</v>
       </c>
@@ -3344,11 +3182,8 @@
       <c r="D55" t="s">
         <v>552</v>
       </c>
-      <c r="G55" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
+    </row>
+    <row r="56" spans="1:4">
       <c r="A56" t="s">
         <v>61</v>
       </c>
@@ -3361,11 +3196,8 @@
       <c r="D56" t="s">
         <v>552</v>
       </c>
-      <c r="G56" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7">
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" t="s">
         <v>62</v>
       </c>
@@ -3378,11 +3210,8 @@
       <c r="D57" t="s">
         <v>552</v>
       </c>
-      <c r="G57" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7">
+    </row>
+    <row r="58" spans="1:4">
       <c r="A58" t="s">
         <v>63</v>
       </c>
@@ -3395,11 +3224,8 @@
       <c r="D58" t="s">
         <v>552</v>
       </c>
-      <c r="G58" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7">
+    </row>
+    <row r="59" spans="1:4">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -3412,11 +3238,8 @@
       <c r="D59" t="s">
         <v>552</v>
       </c>
-      <c r="G59" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
+    </row>
+    <row r="60" spans="1:4">
       <c r="A60" t="s">
         <v>65</v>
       </c>
@@ -3429,11 +3252,8 @@
       <c r="D60" t="s">
         <v>552</v>
       </c>
-      <c r="G60" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
+    </row>
+    <row r="61" spans="1:4">
       <c r="A61" t="s">
         <v>66</v>
       </c>
@@ -3446,11 +3266,8 @@
       <c r="D61" t="s">
         <v>552</v>
       </c>
-      <c r="G61" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7">
+    </row>
+    <row r="62" spans="1:4">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -3463,11 +3280,8 @@
       <c r="D62" t="s">
         <v>552</v>
       </c>
-      <c r="G62" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7">
+    </row>
+    <row r="63" spans="1:4">
       <c r="A63" t="s">
         <v>68</v>
       </c>
@@ -3480,11 +3294,8 @@
       <c r="D63" t="s">
         <v>552</v>
       </c>
-      <c r="G63" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7">
+    </row>
+    <row r="64" spans="1:4">
       <c r="A64" t="s">
         <v>69</v>
       </c>
@@ -3497,11 +3308,8 @@
       <c r="D64" t="s">
         <v>552</v>
       </c>
-      <c r="G64" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7">
+    </row>
+    <row r="65" spans="1:4">
       <c r="A65" t="s">
         <v>70</v>
       </c>
@@ -3514,11 +3322,8 @@
       <c r="D65" t="s">
         <v>552</v>
       </c>
-      <c r="G65" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7">
+    </row>
+    <row r="66" spans="1:4">
       <c r="A66" t="s">
         <v>71</v>
       </c>
@@ -3531,11 +3336,8 @@
       <c r="D66" t="s">
         <v>552</v>
       </c>
-      <c r="G66" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7">
+    </row>
+    <row r="67" spans="1:4">
       <c r="A67" t="s">
         <v>72</v>
       </c>
@@ -3548,11 +3350,8 @@
       <c r="D67" t="s">
         <v>552</v>
       </c>
-      <c r="G67" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7">
+    </row>
+    <row r="68" spans="1:4">
       <c r="A68" t="s">
         <v>73</v>
       </c>
@@ -3565,11 +3364,8 @@
       <c r="D68" t="s">
         <v>552</v>
       </c>
-      <c r="G68" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
+    </row>
+    <row r="69" spans="1:4">
       <c r="A69" t="s">
         <v>74</v>
       </c>
@@ -3582,11 +3378,8 @@
       <c r="D69" t="s">
         <v>552</v>
       </c>
-      <c r="G69" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7">
+    </row>
+    <row r="70" spans="1:4">
       <c r="A70" t="s">
         <v>75</v>
       </c>
@@ -3599,11 +3392,8 @@
       <c r="D70" t="s">
         <v>552</v>
       </c>
-      <c r="G70" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7">
+    </row>
+    <row r="71" spans="1:4">
       <c r="A71" t="s">
         <v>76</v>
       </c>
@@ -3616,11 +3406,8 @@
       <c r="D71" t="s">
         <v>552</v>
       </c>
-      <c r="G71" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7">
+    </row>
+    <row r="72" spans="1:4">
       <c r="A72" t="s">
         <v>77</v>
       </c>
@@ -3633,11 +3420,8 @@
       <c r="D72" t="s">
         <v>552</v>
       </c>
-      <c r="G72" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7">
+    </row>
+    <row r="73" spans="1:4">
       <c r="A73" t="s">
         <v>78</v>
       </c>
@@ -3650,11 +3434,8 @@
       <c r="D73" t="s">
         <v>552</v>
       </c>
-      <c r="G73" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7">
+    </row>
+    <row r="74" spans="1:4">
       <c r="A74" t="s">
         <v>79</v>
       </c>
@@ -3667,11 +3448,8 @@
       <c r="D74" t="s">
         <v>552</v>
       </c>
-      <c r="G74" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7">
+    </row>
+    <row r="75" spans="1:4">
       <c r="A75" t="s">
         <v>80</v>
       </c>
@@ -3684,11 +3462,8 @@
       <c r="D75" t="s">
         <v>552</v>
       </c>
-      <c r="G75" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7">
+    </row>
+    <row r="76" spans="1:4">
       <c r="A76" t="s">
         <v>81</v>
       </c>
@@ -3701,11 +3476,8 @@
       <c r="D76" t="s">
         <v>552</v>
       </c>
-      <c r="G76" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7">
+    </row>
+    <row r="77" spans="1:4">
       <c r="A77" t="s">
         <v>82</v>
       </c>
@@ -3718,11 +3490,8 @@
       <c r="D77" t="s">
         <v>552</v>
       </c>
-      <c r="G77" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7">
+    </row>
+    <row r="78" spans="1:4">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -3735,11 +3504,8 @@
       <c r="D78" t="s">
         <v>552</v>
       </c>
-      <c r="G78" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7">
+    </row>
+    <row r="79" spans="1:4">
       <c r="A79" t="s">
         <v>84</v>
       </c>
@@ -3752,11 +3518,8 @@
       <c r="D79" t="s">
         <v>552</v>
       </c>
-      <c r="G79" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7">
+    </row>
+    <row r="80" spans="1:4">
       <c r="A80" t="s">
         <v>85</v>
       </c>
@@ -3769,11 +3532,8 @@
       <c r="D80" t="s">
         <v>552</v>
       </c>
-      <c r="G80" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7">
+    </row>
+    <row r="81" spans="1:4">
       <c r="A81" t="s">
         <v>86</v>
       </c>
@@ -3786,11 +3546,8 @@
       <c r="D81" t="s">
         <v>552</v>
       </c>
-      <c r="G81" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7">
+    </row>
+    <row r="82" spans="1:4">
       <c r="A82" t="s">
         <v>87</v>
       </c>
@@ -3803,11 +3560,8 @@
       <c r="D82" t="s">
         <v>552</v>
       </c>
-      <c r="G82" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7">
+    </row>
+    <row r="83" spans="1:4">
       <c r="A83" t="s">
         <v>88</v>
       </c>
@@ -3820,11 +3574,8 @@
       <c r="D83" t="s">
         <v>552</v>
       </c>
-      <c r="G83" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7">
+    </row>
+    <row r="84" spans="1:4">
       <c r="A84" t="s">
         <v>89</v>
       </c>
@@ -3837,11 +3588,8 @@
       <c r="D84" t="s">
         <v>552</v>
       </c>
-      <c r="G84" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7">
+    </row>
+    <row r="85" spans="1:4">
       <c r="A85" t="s">
         <v>90</v>
       </c>
@@ -3854,11 +3602,8 @@
       <c r="D85" t="s">
         <v>552</v>
       </c>
-      <c r="G85" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7">
+    </row>
+    <row r="86" spans="1:4">
       <c r="A86" t="s">
         <v>91</v>
       </c>
@@ -3871,11 +3616,8 @@
       <c r="D86" t="s">
         <v>552</v>
       </c>
-      <c r="G86" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7">
+    </row>
+    <row r="87" spans="1:4">
       <c r="A87" t="s">
         <v>92</v>
       </c>
@@ -3888,11 +3630,8 @@
       <c r="D87" t="s">
         <v>552</v>
       </c>
-      <c r="G87" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7">
+    </row>
+    <row r="88" spans="1:4">
       <c r="A88" t="s">
         <v>93</v>
       </c>
@@ -3905,11 +3644,8 @@
       <c r="D88" t="s">
         <v>552</v>
       </c>
-      <c r="G88" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7">
+    </row>
+    <row r="89" spans="1:4">
       <c r="A89" t="s">
         <v>94</v>
       </c>
@@ -3922,11 +3658,8 @@
       <c r="D89" t="s">
         <v>552</v>
       </c>
-      <c r="G89" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7">
+    </row>
+    <row r="90" spans="1:4">
       <c r="A90" t="s">
         <v>95</v>
       </c>
@@ -3939,11 +3672,8 @@
       <c r="D90" t="s">
         <v>552</v>
       </c>
-      <c r="G90" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7">
+    </row>
+    <row r="91" spans="1:4">
       <c r="A91" t="s">
         <v>96</v>
       </c>
@@ -3956,11 +3686,8 @@
       <c r="D91" t="s">
         <v>552</v>
       </c>
-      <c r="G91" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7">
+    </row>
+    <row r="92" spans="1:4">
       <c r="A92" t="s">
         <v>97</v>
       </c>
@@ -3973,11 +3700,8 @@
       <c r="D92" t="s">
         <v>552</v>
       </c>
-      <c r="G92" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7">
+    </row>
+    <row r="93" spans="1:4">
       <c r="A93" t="s">
         <v>98</v>
       </c>
@@ -3990,11 +3714,8 @@
       <c r="D93" t="s">
         <v>552</v>
       </c>
-      <c r="G93" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7">
+    </row>
+    <row r="94" spans="1:4">
       <c r="A94" t="s">
         <v>99</v>
       </c>
@@ -4007,11 +3728,8 @@
       <c r="D94" t="s">
         <v>552</v>
       </c>
-      <c r="G94" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7">
+    </row>
+    <row r="95" spans="1:4">
       <c r="A95" t="s">
         <v>100</v>
       </c>
@@ -4024,11 +3742,8 @@
       <c r="D95" t="s">
         <v>552</v>
       </c>
-      <c r="G95" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7">
+    </row>
+    <row r="96" spans="1:4">
       <c r="A96" t="s">
         <v>101</v>
       </c>
@@ -4041,11 +3756,8 @@
       <c r="D96" t="s">
         <v>552</v>
       </c>
-      <c r="G96" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7">
+    </row>
+    <row r="97" spans="1:4">
       <c r="A97" t="s">
         <v>102</v>
       </c>
@@ -4058,11 +3770,8 @@
       <c r="D97" t="s">
         <v>552</v>
       </c>
-      <c r="G97" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7">
+    </row>
+    <row r="98" spans="1:4">
       <c r="A98" t="s">
         <v>103</v>
       </c>
@@ -4075,11 +3784,8 @@
       <c r="D98" t="s">
         <v>552</v>
       </c>
-      <c r="G98" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7">
+    </row>
+    <row r="99" spans="1:4">
       <c r="A99" t="s">
         <v>104</v>
       </c>
@@ -4092,11 +3798,8 @@
       <c r="D99" t="s">
         <v>552</v>
       </c>
-      <c r="G99" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7">
+    </row>
+    <row r="100" spans="1:4">
       <c r="A100" t="s">
         <v>105</v>
       </c>
@@ -4109,11 +3812,8 @@
       <c r="D100" t="s">
         <v>552</v>
       </c>
-      <c r="G100" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7">
+    </row>
+    <row r="101" spans="1:4">
       <c r="A101" t="s">
         <v>106</v>
       </c>
@@ -4126,11 +3826,8 @@
       <c r="D101" t="s">
         <v>552</v>
       </c>
-      <c r="G101" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7">
+    </row>
+    <row r="102" spans="1:4">
       <c r="A102" t="s">
         <v>107</v>
       </c>
@@ -4143,11 +3840,8 @@
       <c r="D102" t="s">
         <v>552</v>
       </c>
-      <c r="G102" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7">
+    </row>
+    <row r="103" spans="1:4">
       <c r="A103" t="s">
         <v>108</v>
       </c>
@@ -4160,11 +3854,8 @@
       <c r="D103" t="s">
         <v>552</v>
       </c>
-      <c r="G103" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7">
+    </row>
+    <row r="104" spans="1:4">
       <c r="A104" t="s">
         <v>109</v>
       </c>
@@ -4177,11 +3868,8 @@
       <c r="D104" t="s">
         <v>552</v>
       </c>
-      <c r="G104" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7">
+    </row>
+    <row r="105" spans="1:4">
       <c r="A105" t="s">
         <v>110</v>
       </c>
@@ -4194,11 +3882,8 @@
       <c r="D105" t="s">
         <v>552</v>
       </c>
-      <c r="G105" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7">
+    </row>
+    <row r="106" spans="1:4">
       <c r="A106" t="s">
         <v>111</v>
       </c>
@@ -4211,11 +3896,8 @@
       <c r="D106" t="s">
         <v>552</v>
       </c>
-      <c r="G106" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7">
+    </row>
+    <row r="107" spans="1:4">
       <c r="A107" t="s">
         <v>112</v>
       </c>
@@ -4228,11 +3910,8 @@
       <c r="D107" t="s">
         <v>552</v>
       </c>
-      <c r="G107" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7">
+    </row>
+    <row r="108" spans="1:4">
       <c r="A108" t="s">
         <v>113</v>
       </c>
@@ -4245,11 +3924,8 @@
       <c r="D108" t="s">
         <v>552</v>
       </c>
-      <c r="G108" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7">
+    </row>
+    <row r="109" spans="1:4">
       <c r="A109" t="s">
         <v>114</v>
       </c>
@@ -4262,11 +3938,8 @@
       <c r="D109" t="s">
         <v>552</v>
       </c>
-      <c r="G109" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7">
+    </row>
+    <row r="110" spans="1:4">
       <c r="A110" t="s">
         <v>115</v>
       </c>
@@ -4279,11 +3952,8 @@
       <c r="D110" t="s">
         <v>552</v>
       </c>
-      <c r="G110" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7">
+    </row>
+    <row r="111" spans="1:4">
       <c r="A111" t="s">
         <v>116</v>
       </c>
@@ -4296,11 +3966,8 @@
       <c r="D111" t="s">
         <v>552</v>
       </c>
-      <c r="G111" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7">
+    </row>
+    <row r="112" spans="1:4">
       <c r="A112" t="s">
         <v>117</v>
       </c>
@@ -4313,11 +3980,8 @@
       <c r="D112" t="s">
         <v>552</v>
       </c>
-      <c r="G112" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7">
+    </row>
+    <row r="113" spans="1:6">
       <c r="A113" t="s">
         <v>118</v>
       </c>
@@ -4330,11 +3994,8 @@
       <c r="D113" t="s">
         <v>552</v>
       </c>
-      <c r="G113" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7">
+    </row>
+    <row r="114" spans="1:6">
       <c r="A114" t="s">
         <v>119</v>
       </c>
@@ -4347,11 +4008,8 @@
       <c r="D114" t="s">
         <v>552</v>
       </c>
-      <c r="G114" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7">
+    </row>
+    <row r="115" spans="1:6">
       <c r="A115" t="s">
         <v>120</v>
       </c>
@@ -4364,11 +4022,8 @@
       <c r="D115" t="s">
         <v>552</v>
       </c>
-      <c r="G115" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7">
+    </row>
+    <row r="116" spans="1:6">
       <c r="A116" t="s">
         <v>121</v>
       </c>
@@ -4381,11 +4036,8 @@
       <c r="D116" t="s">
         <v>552</v>
       </c>
-      <c r="G116" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7">
+    </row>
+    <row r="117" spans="1:6">
       <c r="A117" t="s">
         <v>122</v>
       </c>
@@ -4398,11 +4050,8 @@
       <c r="D117" t="s">
         <v>552</v>
       </c>
-      <c r="G117" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7">
+    </row>
+    <row r="118" spans="1:6">
       <c r="A118" t="s">
         <v>123</v>
       </c>
@@ -4415,11 +4064,8 @@
       <c r="D118" t="s">
         <v>552</v>
       </c>
-      <c r="G118" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7">
+    </row>
+    <row r="119" spans="1:6">
       <c r="A119" t="s">
         <v>124</v>
       </c>
@@ -4438,11 +4084,8 @@
       <c r="F119" t="s">
         <v>636</v>
       </c>
-      <c r="G119" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7">
+    </row>
+    <row r="120" spans="1:6">
       <c r="A120" t="s">
         <v>125</v>
       </c>
@@ -4458,11 +4101,8 @@
       <c r="E120" t="s">
         <v>583</v>
       </c>
-      <c r="G120" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="121" spans="1:7">
+    </row>
+    <row r="121" spans="1:6">
       <c r="A121" t="s">
         <v>126</v>
       </c>
@@ -4475,11 +4115,8 @@
       <c r="D121" t="s">
         <v>552</v>
       </c>
-      <c r="G121" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="122" spans="1:7">
+    </row>
+    <row r="122" spans="1:6">
       <c r="A122" t="s">
         <v>127</v>
       </c>
@@ -4492,11 +4129,8 @@
       <c r="D122" t="s">
         <v>555</v>
       </c>
-      <c r="G122" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="123" spans="1:7">
+    </row>
+    <row r="123" spans="1:6">
       <c r="A123" t="s">
         <v>128</v>
       </c>
@@ -4515,11 +4149,8 @@
       <c r="F123" t="s">
         <v>637</v>
       </c>
-      <c r="G123" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7">
+    </row>
+    <row r="124" spans="1:6">
       <c r="A124" t="s">
         <v>129</v>
       </c>
@@ -4532,11 +4163,8 @@
       <c r="D124" t="s">
         <v>552</v>
       </c>
-      <c r="G124" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="125" spans="1:7">
+    </row>
+    <row r="125" spans="1:6">
       <c r="A125" t="s">
         <v>130</v>
       </c>
@@ -4549,11 +4177,8 @@
       <c r="D125" t="s">
         <v>552</v>
       </c>
-      <c r="G125" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7">
+    </row>
+    <row r="126" spans="1:6">
       <c r="A126" t="s">
         <v>131</v>
       </c>
@@ -4566,11 +4191,8 @@
       <c r="D126" t="s">
         <v>552</v>
       </c>
-      <c r="G126" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="127" spans="1:7">
+    </row>
+    <row r="127" spans="1:6">
       <c r="A127" t="s">
         <v>132</v>
       </c>
@@ -4583,11 +4205,8 @@
       <c r="D127" t="s">
         <v>552</v>
       </c>
-      <c r="G127" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7">
+    </row>
+    <row r="128" spans="1:6">
       <c r="A128" t="s">
         <v>133</v>
       </c>
@@ -4603,11 +4222,8 @@
       <c r="E128" t="s">
         <v>585</v>
       </c>
-      <c r="G128" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7">
+    </row>
+    <row r="129" spans="1:6">
       <c r="A129" t="s">
         <v>134</v>
       </c>
@@ -4626,11 +4242,8 @@
       <c r="F129" t="s">
         <v>638</v>
       </c>
-      <c r="G129" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7">
+    </row>
+    <row r="130" spans="1:6">
       <c r="A130" t="s">
         <v>135</v>
       </c>
@@ -4643,11 +4256,8 @@
       <c r="D130" t="s">
         <v>552</v>
       </c>
-      <c r="G130" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7">
+    </row>
+    <row r="131" spans="1:6">
       <c r="A131" t="s">
         <v>136</v>
       </c>
@@ -4661,7 +4271,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="132" spans="1:7">
+    <row r="132" spans="1:6">
       <c r="A132" t="s">
         <v>137</v>
       </c>
@@ -4677,11 +4287,8 @@
       <c r="E132" t="s">
         <v>588</v>
       </c>
-      <c r="G132" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7">
+    </row>
+    <row r="133" spans="1:6">
       <c r="A133" t="s">
         <v>138</v>
       </c>
@@ -4697,11 +4304,8 @@
       <c r="E133" t="s">
         <v>589</v>
       </c>
-      <c r="G133" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7">
+    </row>
+    <row r="134" spans="1:6">
       <c r="A134" t="s">
         <v>139</v>
       </c>
@@ -4712,7 +4316,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="135" spans="1:7">
+    <row r="135" spans="1:6">
       <c r="A135" t="s">
         <v>140</v>
       </c>
@@ -4723,7 +4327,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="136" spans="1:7">
+    <row r="136" spans="1:6">
       <c r="A136" t="s">
         <v>141</v>
       </c>
@@ -4736,11 +4340,8 @@
       <c r="D136" t="s">
         <v>552</v>
       </c>
-      <c r="G136" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7">
+    </row>
+    <row r="137" spans="1:6">
       <c r="A137" t="s">
         <v>142</v>
       </c>
@@ -4753,11 +4354,8 @@
       <c r="D137" t="s">
         <v>558</v>
       </c>
-      <c r="G137" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7">
+    </row>
+    <row r="138" spans="1:6">
       <c r="A138" t="s">
         <v>143</v>
       </c>
@@ -4768,7 +4366,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="139" spans="1:7">
+    <row r="139" spans="1:6">
       <c r="A139" t="s">
         <v>144</v>
       </c>
@@ -4779,7 +4377,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="140" spans="1:7">
+    <row r="140" spans="1:6">
       <c r="A140" t="s">
         <v>145</v>
       </c>
@@ -4790,7 +4388,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="141" spans="1:7">
+    <row r="141" spans="1:6">
       <c r="A141" t="s">
         <v>146</v>
       </c>
@@ -4803,11 +4401,8 @@
       <c r="D141" t="s">
         <v>552</v>
       </c>
-      <c r="G141" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7">
+    </row>
+    <row r="142" spans="1:6">
       <c r="A142" t="s">
         <v>147</v>
       </c>
@@ -4826,11 +4421,8 @@
       <c r="F142" t="s">
         <v>639</v>
       </c>
-      <c r="G142" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7">
+    </row>
+    <row r="143" spans="1:6">
       <c r="A143" t="s">
         <v>148</v>
       </c>
@@ -4843,11 +4435,8 @@
       <c r="D143" t="s">
         <v>562</v>
       </c>
-      <c r="G143" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7">
+    </row>
+    <row r="144" spans="1:6">
       <c r="A144" t="s">
         <v>149</v>
       </c>
@@ -4861,7 +4450,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="145" spans="1:7">
+    <row r="145" spans="1:6">
       <c r="A145" t="s">
         <v>150</v>
       </c>
@@ -4872,7 +4461,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="146" spans="1:7">
+    <row r="146" spans="1:6">
       <c r="A146" t="s">
         <v>151</v>
       </c>
@@ -4888,11 +4477,8 @@
       <c r="F146" t="s">
         <v>640</v>
       </c>
-      <c r="G146" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7">
+    </row>
+    <row r="147" spans="1:6">
       <c r="A147" t="s">
         <v>152</v>
       </c>
@@ -4911,11 +4497,8 @@
       <c r="F147" t="s">
         <v>641</v>
       </c>
-      <c r="G147" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7">
+    </row>
+    <row r="148" spans="1:6">
       <c r="A148" t="s">
         <v>153</v>
       </c>
@@ -4931,11 +4514,8 @@
       <c r="E148" t="s">
         <v>593</v>
       </c>
-      <c r="G148" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7">
+    </row>
+    <row r="149" spans="1:6">
       <c r="A149" t="s">
         <v>154</v>
       </c>
@@ -4951,11 +4531,8 @@
       <c r="E149" t="s">
         <v>594</v>
       </c>
-      <c r="G149" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7">
+    </row>
+    <row r="150" spans="1:6">
       <c r="A150" t="s">
         <v>155</v>
       </c>
@@ -4971,11 +4548,8 @@
       <c r="E150" t="s">
         <v>595</v>
       </c>
-      <c r="G150" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7">
+    </row>
+    <row r="151" spans="1:6">
       <c r="A151" t="s">
         <v>156</v>
       </c>
@@ -4991,11 +4565,8 @@
       <c r="E151" t="s">
         <v>596</v>
       </c>
-      <c r="G151" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7">
+    </row>
+    <row r="152" spans="1:6">
       <c r="A152" t="s">
         <v>157</v>
       </c>
@@ -5011,11 +4582,8 @@
       <c r="E152" t="s">
         <v>597</v>
       </c>
-      <c r="G152" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="153" spans="1:7">
+    </row>
+    <row r="153" spans="1:6">
       <c r="A153" t="s">
         <v>158</v>
       </c>
@@ -5026,7 +4594,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="154" spans="1:7">
+    <row r="154" spans="1:6">
       <c r="A154" t="s">
         <v>159</v>
       </c>
@@ -5042,11 +4610,8 @@
       <c r="E154" t="s">
         <v>598</v>
       </c>
-      <c r="G154" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7">
+    </row>
+    <row r="155" spans="1:6">
       <c r="A155" t="s">
         <v>160</v>
       </c>
@@ -5059,11 +4624,8 @@
       <c r="D155" t="s">
         <v>552</v>
       </c>
-      <c r="G155" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7">
+    </row>
+    <row r="156" spans="1:6">
       <c r="A156" t="s">
         <v>161</v>
       </c>
@@ -5076,11 +4638,8 @@
       <c r="D156" t="s">
         <v>552</v>
       </c>
-      <c r="G156" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7">
+    </row>
+    <row r="157" spans="1:6">
       <c r="A157" t="s">
         <v>162</v>
       </c>
@@ -5099,11 +4658,8 @@
       <c r="F157" t="s">
         <v>642</v>
       </c>
-      <c r="G157" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7">
+    </row>
+    <row r="158" spans="1:6">
       <c r="A158" t="s">
         <v>163</v>
       </c>
@@ -5119,11 +4675,8 @@
       <c r="E158" t="s">
         <v>600</v>
       </c>
-      <c r="G158" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="159" spans="1:7">
+    </row>
+    <row r="159" spans="1:6">
       <c r="A159" t="s">
         <v>164</v>
       </c>
@@ -5139,11 +4692,8 @@
       <c r="E159" t="s">
         <v>601</v>
       </c>
-      <c r="G159" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="160" spans="1:7">
+    </row>
+    <row r="160" spans="1:6">
       <c r="A160" t="s">
         <v>165</v>
       </c>
@@ -5159,11 +4709,8 @@
       <c r="E160" t="s">
         <v>602</v>
       </c>
-      <c r="G160" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7">
+    </row>
+    <row r="161" spans="1:6">
       <c r="A161" t="s">
         <v>166</v>
       </c>
@@ -5179,11 +4726,8 @@
       <c r="E161" t="s">
         <v>603</v>
       </c>
-      <c r="G161" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="162" spans="1:7">
+    </row>
+    <row r="162" spans="1:6">
       <c r="A162" t="s">
         <v>167</v>
       </c>
@@ -5196,11 +4740,8 @@
       <c r="D162" t="s">
         <v>552</v>
       </c>
-      <c r="G162" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7">
+    </row>
+    <row r="163" spans="1:6">
       <c r="A163" t="s">
         <v>168</v>
       </c>
@@ -5216,11 +4757,8 @@
       <c r="E163" t="s">
         <v>604</v>
       </c>
-      <c r="G163" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7">
+    </row>
+    <row r="164" spans="1:6">
       <c r="A164" t="s">
         <v>169</v>
       </c>
@@ -5236,11 +4774,8 @@
       <c r="E164" t="s">
         <v>605</v>
       </c>
-      <c r="G164" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7">
+    </row>
+    <row r="165" spans="1:6">
       <c r="A165" t="s">
         <v>170</v>
       </c>
@@ -5254,7 +4789,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="166" spans="1:7">
+    <row r="166" spans="1:6">
       <c r="A166" t="s">
         <v>171</v>
       </c>
@@ -5270,11 +4805,8 @@
       <c r="E166" t="s">
         <v>607</v>
       </c>
-      <c r="G166" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7">
+    </row>
+    <row r="167" spans="1:6">
       <c r="A167" t="s">
         <v>172</v>
       </c>
@@ -5290,11 +4822,8 @@
       <c r="E167" t="s">
         <v>608</v>
       </c>
-      <c r="G167" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="168" spans="1:7">
+    </row>
+    <row r="168" spans="1:6">
       <c r="A168" t="s">
         <v>173</v>
       </c>
@@ -5310,11 +4839,8 @@
       <c r="E168" t="s">
         <v>609</v>
       </c>
-      <c r="G168" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="169" spans="1:7">
+    </row>
+    <row r="169" spans="1:6">
       <c r="A169" t="s">
         <v>174</v>
       </c>
@@ -5330,11 +4856,8 @@
       <c r="E169" t="s">
         <v>610</v>
       </c>
-      <c r="G169" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7">
+    </row>
+    <row r="170" spans="1:6">
       <c r="A170" t="s">
         <v>175</v>
       </c>
@@ -5348,7 +4871,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="171" spans="1:7">
+    <row r="171" spans="1:6">
       <c r="A171" t="s">
         <v>176</v>
       </c>
@@ -5362,7 +4885,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="172" spans="1:7">
+    <row r="172" spans="1:6">
       <c r="A172" t="s">
         <v>177</v>
       </c>
@@ -5376,7 +4899,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="173" spans="1:7">
+    <row r="173" spans="1:6">
       <c r="A173" t="s">
         <v>178</v>
       </c>
@@ -5389,11 +4912,8 @@
       <c r="D173" t="s">
         <v>552</v>
       </c>
-      <c r="G173" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="174" spans="1:7">
+    </row>
+    <row r="174" spans="1:6">
       <c r="A174" t="s">
         <v>179</v>
       </c>
@@ -5409,11 +4929,8 @@
       <c r="F174" t="s">
         <v>643</v>
       </c>
-      <c r="G174" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="175" spans="1:7">
+    </row>
+    <row r="175" spans="1:6">
       <c r="A175" t="s">
         <v>180</v>
       </c>
@@ -5429,11 +4946,8 @@
       <c r="F175" t="s">
         <v>644</v>
       </c>
-      <c r="G175" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="176" spans="1:7">
+    </row>
+    <row r="176" spans="1:6">
       <c r="A176" t="s">
         <v>181</v>
       </c>
@@ -5444,7 +4958,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="177" spans="1:7">
+    <row r="177" spans="1:6">
       <c r="A177" t="s">
         <v>182</v>
       </c>
@@ -5455,7 +4969,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="178" spans="1:7">
+    <row r="178" spans="1:6">
       <c r="A178" t="s">
         <v>183</v>
       </c>
@@ -5466,7 +4980,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="179" spans="1:7">
+    <row r="179" spans="1:6">
       <c r="A179" t="s">
         <v>184</v>
       </c>
@@ -5485,11 +4999,8 @@
       <c r="F179" t="s">
         <v>645</v>
       </c>
-      <c r="G179" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="180" spans="1:7">
+    </row>
+    <row r="180" spans="1:6">
       <c r="A180" t="s">
         <v>185</v>
       </c>
@@ -5500,7 +5011,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="181" spans="1:7">
+    <row r="181" spans="1:6">
       <c r="A181" t="s">
         <v>186</v>
       </c>
@@ -5511,7 +5022,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="182" spans="1:7">
+    <row r="182" spans="1:6">
       <c r="A182" t="s">
         <v>187</v>
       </c>
@@ -5527,11 +5038,8 @@
       <c r="E182" t="s">
         <v>615</v>
       </c>
-      <c r="G182" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="183" spans="1:7">
+    </row>
+    <row r="183" spans="1:6">
       <c r="A183" t="s">
         <v>188</v>
       </c>
@@ -5547,11 +5055,8 @@
       <c r="F183" t="s">
         <v>646</v>
       </c>
-      <c r="G183" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="184" spans="1:7">
+    </row>
+    <row r="184" spans="1:6">
       <c r="A184" t="s">
         <v>189</v>
       </c>
@@ -5562,7 +5067,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="185" spans="1:7">
+    <row r="185" spans="1:6">
       <c r="A185" t="s">
         <v>190</v>
       </c>
@@ -5576,7 +5081,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="186" spans="1:7">
+    <row r="186" spans="1:6">
       <c r="A186" t="s">
         <v>191</v>
       </c>
@@ -5590,7 +5095,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="187" spans="1:7">
+    <row r="187" spans="1:6">
       <c r="A187" t="s">
         <v>192</v>
       </c>
@@ -5604,7 +5109,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="188" spans="1:7">
+    <row r="188" spans="1:6">
       <c r="A188" t="s">
         <v>193</v>
       </c>
@@ -5618,7 +5123,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="189" spans="1:7">
+    <row r="189" spans="1:6">
       <c r="A189" t="s">
         <v>194</v>
       </c>
@@ -5632,7 +5137,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="190" spans="1:7">
+    <row r="190" spans="1:6">
       <c r="A190" t="s">
         <v>195</v>
       </c>
@@ -5646,7 +5151,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="191" spans="1:7">
+    <row r="191" spans="1:6">
       <c r="A191" t="s">
         <v>196</v>
       </c>
@@ -5657,7 +5162,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="192" spans="1:7">
+    <row r="192" spans="1:6">
       <c r="A192" t="s">
         <v>197</v>
       </c>
@@ -5668,7 +5173,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="193" spans="1:7">
+    <row r="193" spans="1:6">
       <c r="A193" t="s">
         <v>198</v>
       </c>
@@ -5679,7 +5184,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="194" spans="1:7">
+    <row r="194" spans="1:6">
       <c r="A194" t="s">
         <v>199</v>
       </c>
@@ -5692,11 +5197,8 @@
       <c r="D194" t="s">
         <v>555</v>
       </c>
-      <c r="G194" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="195" spans="1:7">
+    </row>
+    <row r="195" spans="1:6">
       <c r="A195" t="s">
         <v>200</v>
       </c>
@@ -5709,11 +5211,8 @@
       <c r="D195" t="s">
         <v>555</v>
       </c>
-      <c r="G195" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="196" spans="1:7">
+    </row>
+    <row r="196" spans="1:6">
       <c r="A196" t="s">
         <v>201</v>
       </c>
@@ -5729,11 +5228,8 @@
       <c r="F196" t="s">
         <v>648</v>
       </c>
-      <c r="G196" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="197" spans="1:7">
+    </row>
+    <row r="197" spans="1:6">
       <c r="A197" t="s">
         <v>202</v>
       </c>
@@ -5752,11 +5248,8 @@
       <c r="F197" t="s">
         <v>649</v>
       </c>
-      <c r="G197" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="198" spans="1:7">
+    </row>
+    <row r="198" spans="1:6">
       <c r="A198" t="s">
         <v>203</v>
       </c>
@@ -5775,11 +5268,8 @@
       <c r="F198" t="s">
         <v>650</v>
       </c>
-      <c r="G198" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="199" spans="1:7">
+    </row>
+    <row r="199" spans="1:6">
       <c r="A199" t="s">
         <v>204</v>
       </c>
@@ -5798,11 +5288,8 @@
       <c r="F199" t="s">
         <v>651</v>
       </c>
-      <c r="G199" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="200" spans="1:7">
+    </row>
+    <row r="200" spans="1:6">
       <c r="A200" t="s">
         <v>205</v>
       </c>
@@ -5815,11 +5302,8 @@
       <c r="D200" t="s">
         <v>552</v>
       </c>
-      <c r="G200" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="201" spans="1:7">
+    </row>
+    <row r="201" spans="1:6">
       <c r="A201" t="s">
         <v>206</v>
       </c>
@@ -5830,7 +5314,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="202" spans="1:7">
+    <row r="202" spans="1:6">
       <c r="A202" t="s">
         <v>207</v>
       </c>
@@ -5841,7 +5325,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="203" spans="1:7">
+    <row r="203" spans="1:6">
       <c r="A203" t="s">
         <v>208</v>
       </c>
@@ -5852,7 +5336,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="204" spans="1:7">
+    <row r="204" spans="1:6">
       <c r="A204" t="s">
         <v>209</v>
       </c>
@@ -5865,11 +5349,8 @@
       <c r="D204" t="s">
         <v>552</v>
       </c>
-      <c r="G204" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="205" spans="1:7">
+    </row>
+    <row r="205" spans="1:6">
       <c r="A205" t="s">
         <v>210</v>
       </c>
@@ -5880,7 +5361,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="206" spans="1:7">
+    <row r="206" spans="1:6">
       <c r="A206" t="s">
         <v>211</v>
       </c>
@@ -5891,7 +5372,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="207" spans="1:7">
+    <row r="207" spans="1:6">
       <c r="A207" t="s">
         <v>212</v>
       </c>
@@ -5907,11 +5388,8 @@
       <c r="E207" t="s">
         <v>624</v>
       </c>
-      <c r="G207" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="208" spans="1:7">
+    </row>
+    <row r="208" spans="1:6">
       <c r="A208" t="s">
         <v>213</v>
       </c>
@@ -5925,7 +5403,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="209" spans="1:7">
+    <row r="209" spans="1:5">
       <c r="A209" t="s">
         <v>214</v>
       </c>
@@ -5936,7 +5414,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="210" spans="1:7">
+    <row r="210" spans="1:5">
       <c r="A210" t="s">
         <v>215</v>
       </c>
@@ -5952,11 +5430,8 @@
       <c r="E210" t="s">
         <v>626</v>
       </c>
-      <c r="G210" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="211" spans="1:7">
+    </row>
+    <row r="211" spans="1:5">
       <c r="A211" t="s">
         <v>216</v>
       </c>
@@ -5969,11 +5444,8 @@
       <c r="D211" t="s">
         <v>552</v>
       </c>
-      <c r="G211" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="212" spans="1:7">
+    </row>
+    <row r="212" spans="1:5">
       <c r="A212" t="s">
         <v>217</v>
       </c>
@@ -5987,7 +5459,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="213" spans="1:7">
+    <row r="213" spans="1:5">
       <c r="A213" t="s">
         <v>218</v>
       </c>
@@ -6001,7 +5473,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="214" spans="1:7">
+    <row r="214" spans="1:5">
       <c r="A214" t="s">
         <v>219</v>
       </c>
@@ -6014,11 +5486,8 @@
       <c r="D214" t="s">
         <v>552</v>
       </c>
-      <c r="G214" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="215" spans="1:7">
+    </row>
+    <row r="215" spans="1:5">
       <c r="A215" t="s">
         <v>220</v>
       </c>
@@ -6031,11 +5500,8 @@
       <c r="D215" t="s">
         <v>552</v>
       </c>
-      <c r="G215" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="216" spans="1:7">
+    </row>
+    <row r="216" spans="1:5">
       <c r="A216" t="s">
         <v>221</v>
       </c>
@@ -6049,7 +5515,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="217" spans="1:7">
+    <row r="217" spans="1:5">
       <c r="A217" t="s">
         <v>222</v>
       </c>
@@ -6065,11 +5531,8 @@
       <c r="E217" t="s">
         <v>630</v>
       </c>
-      <c r="G217" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="218" spans="1:7">
+    </row>
+    <row r="218" spans="1:5">
       <c r="A218" t="s">
         <v>223</v>
       </c>
@@ -6085,11 +5548,8 @@
       <c r="E218" t="s">
         <v>630</v>
       </c>
-      <c r="G218" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="219" spans="1:7">
+    </row>
+    <row r="219" spans="1:5">
       <c r="A219" t="s">
         <v>224</v>
       </c>
@@ -6105,11 +5565,8 @@
       <c r="E219" t="s">
         <v>631</v>
       </c>
-      <c r="G219" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="220" spans="1:7">
+    </row>
+    <row r="220" spans="1:5">
       <c r="A220" t="s">
         <v>225</v>
       </c>
@@ -6120,7 +5577,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="221" spans="1:7">
+    <row r="221" spans="1:5">
       <c r="A221" t="s">
         <v>226</v>
       </c>
@@ -6133,11 +5590,8 @@
       <c r="D221" t="s">
         <v>552</v>
       </c>
-      <c r="G221" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="222" spans="1:7">
+    </row>
+    <row r="222" spans="1:5">
       <c r="A222" t="s">
         <v>227</v>
       </c>
@@ -6153,11 +5607,8 @@
       <c r="E222" t="s">
         <v>632</v>
       </c>
-      <c r="G222" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="223" spans="1:7">
+    </row>
+    <row r="223" spans="1:5">
       <c r="A223" t="s">
         <v>228</v>
       </c>
@@ -6170,11 +5621,8 @@
       <c r="D223" t="s">
         <v>552</v>
       </c>
-      <c r="G223" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="224" spans="1:7">
+    </row>
+    <row r="224" spans="1:5">
       <c r="A224" t="s">
         <v>229</v>
       </c>
@@ -6187,11 +5635,8 @@
       <c r="D224" t="s">
         <v>574</v>
       </c>
-      <c r="G224" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="225" spans="1:7">
+    </row>
+    <row r="225" spans="1:6">
       <c r="A225" t="s">
         <v>230</v>
       </c>
@@ -6207,11 +5652,8 @@
       <c r="F225" t="s">
         <v>652</v>
       </c>
-      <c r="G225" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="226" spans="1:7">
+    </row>
+    <row r="226" spans="1:6">
       <c r="A226" t="s">
         <v>231</v>
       </c>
@@ -6224,11 +5666,8 @@
       <c r="D226" t="s">
         <v>552</v>
       </c>
-      <c r="G226" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="227" spans="1:7">
+    </row>
+    <row r="227" spans="1:6">
       <c r="A227" t="s">
         <v>232</v>
       </c>
@@ -6239,7 +5678,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="228" spans="1:7">
+    <row r="228" spans="1:6">
       <c r="A228" t="s">
         <v>233</v>
       </c>
@@ -6252,11 +5691,8 @@
       <c r="D228" t="s">
         <v>552</v>
       </c>
-      <c r="G228" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="229" spans="1:7">
+    </row>
+    <row r="229" spans="1:6">
       <c r="A229" t="s">
         <v>234</v>
       </c>
@@ -6269,11 +5705,8 @@
       <c r="D229" t="s">
         <v>552</v>
       </c>
-      <c r="G229" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="230" spans="1:7">
+    </row>
+    <row r="230" spans="1:6">
       <c r="A230" t="s">
         <v>235</v>
       </c>
@@ -6286,11 +5719,8 @@
       <c r="D230" t="s">
         <v>552</v>
       </c>
-      <c r="G230" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="231" spans="1:7">
+    </row>
+    <row r="231" spans="1:6">
       <c r="A231" t="s">
         <v>236</v>
       </c>
@@ -6303,11 +5733,8 @@
       <c r="D231" t="s">
         <v>552</v>
       </c>
-      <c r="G231" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="232" spans="1:7">
+    </row>
+    <row r="232" spans="1:6">
       <c r="A232" t="s">
         <v>237</v>
       </c>
@@ -6320,11 +5747,8 @@
       <c r="D232" t="s">
         <v>552</v>
       </c>
-      <c r="G232" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="233" spans="1:7">
+    </row>
+    <row r="233" spans="1:6">
       <c r="A233" t="s">
         <v>238</v>
       </c>
@@ -6337,11 +5761,8 @@
       <c r="D233" t="s">
         <v>552</v>
       </c>
-      <c r="G233" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="234" spans="1:7">
+    </row>
+    <row r="234" spans="1:6">
       <c r="A234" t="s">
         <v>239</v>
       </c>
@@ -6354,11 +5775,8 @@
       <c r="D234" t="s">
         <v>552</v>
       </c>
-      <c r="G234" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="235" spans="1:7">
+    </row>
+    <row r="235" spans="1:6">
       <c r="A235" t="s">
         <v>240</v>
       </c>
@@ -6371,11 +5789,8 @@
       <c r="D235" t="s">
         <v>552</v>
       </c>
-      <c r="G235" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="236" spans="1:7">
+    </row>
+    <row r="236" spans="1:6">
       <c r="A236" t="s">
         <v>241</v>
       </c>
@@ -6388,11 +5803,8 @@
       <c r="D236" t="s">
         <v>552</v>
       </c>
-      <c r="G236" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="237" spans="1:7">
+    </row>
+    <row r="237" spans="1:6">
       <c r="A237" t="s">
         <v>242</v>
       </c>
@@ -6405,11 +5817,8 @@
       <c r="D237" t="s">
         <v>552</v>
       </c>
-      <c r="G237" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="238" spans="1:7">
+    </row>
+    <row r="238" spans="1:6">
       <c r="A238" t="s">
         <v>243</v>
       </c>
@@ -6422,11 +5831,8 @@
       <c r="D238" t="s">
         <v>552</v>
       </c>
-      <c r="G238" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="239" spans="1:7">
+    </row>
+    <row r="239" spans="1:6">
       <c r="A239" t="s">
         <v>244</v>
       </c>
@@ -6439,11 +5845,8 @@
       <c r="D239" t="s">
         <v>552</v>
       </c>
-      <c r="G239" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="240" spans="1:7">
+    </row>
+    <row r="240" spans="1:6">
       <c r="A240" t="s">
         <v>245</v>
       </c>
@@ -6456,11 +5859,8 @@
       <c r="D240" t="s">
         <v>552</v>
       </c>
-      <c r="G240" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="241" spans="1:7">
+    </row>
+    <row r="241" spans="1:4">
       <c r="A241" t="s">
         <v>246</v>
       </c>
@@ -6473,11 +5873,8 @@
       <c r="D241" t="s">
         <v>552</v>
       </c>
-      <c r="G241" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="242" spans="1:7">
+    </row>
+    <row r="242" spans="1:4">
       <c r="A242" t="s">
         <v>247</v>
       </c>
@@ -6490,11 +5887,8 @@
       <c r="D242" t="s">
         <v>552</v>
       </c>
-      <c r="G242" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="243" spans="1:7">
+    </row>
+    <row r="243" spans="1:4">
       <c r="A243" t="s">
         <v>248</v>
       </c>
@@ -6507,11 +5901,8 @@
       <c r="D243" t="s">
         <v>552</v>
       </c>
-      <c r="G243" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="244" spans="1:7">
+    </row>
+    <row r="244" spans="1:4">
       <c r="A244" t="s">
         <v>249</v>
       </c>
@@ -6524,11 +5915,8 @@
       <c r="D244" t="s">
         <v>552</v>
       </c>
-      <c r="G244" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="245" spans="1:7">
+    </row>
+    <row r="245" spans="1:4">
       <c r="A245" t="s">
         <v>250</v>
       </c>
@@ -6541,11 +5929,8 @@
       <c r="D245" t="s">
         <v>552</v>
       </c>
-      <c r="G245" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="246" spans="1:7">
+    </row>
+    <row r="246" spans="1:4">
       <c r="A246" t="s">
         <v>251</v>
       </c>
@@ -6558,11 +5943,8 @@
       <c r="D246" t="s">
         <v>552</v>
       </c>
-      <c r="G246" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="247" spans="1:7">
+    </row>
+    <row r="247" spans="1:4">
       <c r="A247" t="s">
         <v>252</v>
       </c>
@@ -6575,11 +5957,8 @@
       <c r="D247" t="s">
         <v>552</v>
       </c>
-      <c r="G247" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="248" spans="1:7">
+    </row>
+    <row r="248" spans="1:4">
       <c r="A248" t="s">
         <v>253</v>
       </c>
@@ -6592,11 +5971,8 @@
       <c r="D248" t="s">
         <v>552</v>
       </c>
-      <c r="G248" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="249" spans="1:7">
+    </row>
+    <row r="249" spans="1:4">
       <c r="A249" t="s">
         <v>254</v>
       </c>
@@ -6609,11 +5985,8 @@
       <c r="D249" t="s">
         <v>552</v>
       </c>
-      <c r="G249" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="250" spans="1:7">
+    </row>
+    <row r="250" spans="1:4">
       <c r="A250" t="s">
         <v>255</v>
       </c>
@@ -6626,11 +5999,8 @@
       <c r="D250" t="s">
         <v>552</v>
       </c>
-      <c r="G250" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="251" spans="1:7">
+    </row>
+    <row r="251" spans="1:4">
       <c r="A251" t="s">
         <v>256</v>
       </c>
@@ -6643,11 +6013,8 @@
       <c r="D251" t="s">
         <v>552</v>
       </c>
-      <c r="G251" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="252" spans="1:7">
+    </row>
+    <row r="252" spans="1:4">
       <c r="A252" t="s">
         <v>257</v>
       </c>
@@ -6660,11 +6027,8 @@
       <c r="D252" t="s">
         <v>552</v>
       </c>
-      <c r="G252" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="253" spans="1:7">
+    </row>
+    <row r="253" spans="1:4">
       <c r="A253" t="s">
         <v>258</v>
       </c>
@@ -6677,11 +6041,8 @@
       <c r="D253" t="s">
         <v>552</v>
       </c>
-      <c r="G253" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="254" spans="1:7">
+    </row>
+    <row r="254" spans="1:4">
       <c r="A254" t="s">
         <v>259</v>
       </c>
@@ -6694,11 +6055,8 @@
       <c r="D254" t="s">
         <v>552</v>
       </c>
-      <c r="G254" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="255" spans="1:7">
+    </row>
+    <row r="255" spans="1:4">
       <c r="A255" t="s">
         <v>260</v>
       </c>
@@ -6711,11 +6069,8 @@
       <c r="D255" t="s">
         <v>552</v>
       </c>
-      <c r="G255" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="256" spans="1:7">
+    </row>
+    <row r="256" spans="1:4">
       <c r="A256" t="s">
         <v>261</v>
       </c>
@@ -6728,11 +6083,8 @@
       <c r="D256" t="s">
         <v>552</v>
       </c>
-      <c r="G256" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="257" spans="1:7">
+    </row>
+    <row r="257" spans="1:4">
       <c r="A257" t="s">
         <v>262</v>
       </c>
@@ -6745,11 +6097,8 @@
       <c r="D257" t="s">
         <v>552</v>
       </c>
-      <c r="G257" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="258" spans="1:7">
+    </row>
+    <row r="258" spans="1:4">
       <c r="A258" t="s">
         <v>263</v>
       </c>
@@ -6762,11 +6111,8 @@
       <c r="D258" t="s">
         <v>552</v>
       </c>
-      <c r="G258" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="259" spans="1:7">
+    </row>
+    <row r="259" spans="1:4">
       <c r="A259" t="s">
         <v>264</v>
       </c>
@@ -6779,11 +6125,8 @@
       <c r="D259" t="s">
         <v>552</v>
       </c>
-      <c r="G259" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="260" spans="1:7">
+    </row>
+    <row r="260" spans="1:4">
       <c r="A260" t="s">
         <v>265</v>
       </c>
@@ -6796,11 +6139,8 @@
       <c r="D260" t="s">
         <v>552</v>
       </c>
-      <c r="G260" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="261" spans="1:7">
+    </row>
+    <row r="261" spans="1:4">
       <c r="A261" t="s">
         <v>266</v>
       </c>
@@ -6813,11 +6153,8 @@
       <c r="D261" t="s">
         <v>552</v>
       </c>
-      <c r="G261" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="262" spans="1:7">
+    </row>
+    <row r="262" spans="1:4">
       <c r="A262" t="s">
         <v>267</v>
       </c>
@@ -6830,11 +6167,8 @@
       <c r="D262" t="s">
         <v>552</v>
       </c>
-      <c r="G262" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="263" spans="1:7">
+    </row>
+    <row r="263" spans="1:4">
       <c r="A263" t="s">
         <v>268</v>
       </c>
@@ -6847,11 +6181,8 @@
       <c r="D263" t="s">
         <v>552</v>
       </c>
-      <c r="G263" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="264" spans="1:7">
+    </row>
+    <row r="264" spans="1:4">
       <c r="A264" t="s">
         <v>269</v>
       </c>
@@ -6864,11 +6195,8 @@
       <c r="D264" t="s">
         <v>552</v>
       </c>
-      <c r="G264" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="265" spans="1:7">
+    </row>
+    <row r="265" spans="1:4">
       <c r="A265" t="s">
         <v>270</v>
       </c>
@@ -6881,11 +6209,8 @@
       <c r="D265" t="s">
         <v>552</v>
       </c>
-      <c r="G265" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="266" spans="1:7">
+    </row>
+    <row r="266" spans="1:4">
       <c r="A266" t="s">
         <v>271</v>
       </c>
@@ -6898,11 +6223,8 @@
       <c r="D266" t="s">
         <v>577</v>
       </c>
-      <c r="G266" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="267" spans="1:7">
+    </row>
+    <row r="267" spans="1:4">
       <c r="A267" t="s">
         <v>272</v>
       </c>
@@ -6915,11 +6237,8 @@
       <c r="D267" t="s">
         <v>577</v>
       </c>
-      <c r="G267" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="268" spans="1:7">
+    </row>
+    <row r="268" spans="1:4">
       <c r="A268" t="s">
         <v>273</v>
       </c>
@@ -6932,11 +6251,8 @@
       <c r="D268" t="s">
         <v>577</v>
       </c>
-      <c r="G268" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="269" spans="1:7">
+    </row>
+    <row r="269" spans="1:4">
       <c r="A269" t="s">
         <v>274</v>
       </c>
@@ -6949,11 +6265,8 @@
       <c r="D269" t="s">
         <v>577</v>
       </c>
-      <c r="G269" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="270" spans="1:7">
+    </row>
+    <row r="270" spans="1:4">
       <c r="A270" t="s">
         <v>275</v>
       </c>
@@ -6966,11 +6279,8 @@
       <c r="D270" t="s">
         <v>577</v>
       </c>
-      <c r="G270" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="271" spans="1:7">
+    </row>
+    <row r="271" spans="1:4">
       <c r="A271" t="s">
         <v>276</v>
       </c>
@@ -6983,11 +6293,8 @@
       <c r="D271" t="s">
         <v>577</v>
       </c>
-      <c r="G271" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="272" spans="1:7">
+    </row>
+    <row r="272" spans="1:4">
       <c r="A272" t="s">
         <v>277</v>
       </c>
@@ -7000,11 +6307,8 @@
       <c r="D272" t="s">
         <v>577</v>
       </c>
-      <c r="G272" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="273" spans="1:7">
+    </row>
+    <row r="273" spans="1:4">
       <c r="A273" t="s">
         <v>278</v>
       </c>
@@ -7017,11 +6321,8 @@
       <c r="D273" t="s">
         <v>577</v>
       </c>
-      <c r="G273" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="274" spans="1:7">
+    </row>
+    <row r="274" spans="1:4">
       <c r="A274" t="s">
         <v>279</v>
       </c>
@@ -7034,11 +6335,8 @@
       <c r="D274" t="s">
         <v>577</v>
       </c>
-      <c r="G274" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="275" spans="1:7">
+    </row>
+    <row r="275" spans="1:4">
       <c r="A275" t="s">
         <v>280</v>
       </c>
@@ -7051,11 +6349,8 @@
       <c r="D275" t="s">
         <v>577</v>
       </c>
-      <c r="G275" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="276" spans="1:7">
+    </row>
+    <row r="276" spans="1:4">
       <c r="A276" t="s">
         <v>281</v>
       </c>
@@ -7068,11 +6363,8 @@
       <c r="D276" t="s">
         <v>577</v>
       </c>
-      <c r="G276" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="277" spans="1:7">
+    </row>
+    <row r="277" spans="1:4">
       <c r="A277" t="s">
         <v>282</v>
       </c>
@@ -7085,11 +6377,8 @@
       <c r="D277" t="s">
         <v>577</v>
       </c>
-      <c r="G277" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="278" spans="1:7">
+    </row>
+    <row r="278" spans="1:4">
       <c r="A278" t="s">
         <v>283</v>
       </c>
@@ -7102,11 +6391,8 @@
       <c r="D278" t="s">
         <v>577</v>
       </c>
-      <c r="G278" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="279" spans="1:7">
+    </row>
+    <row r="279" spans="1:4">
       <c r="A279" t="s">
         <v>284</v>
       </c>
@@ -7119,11 +6405,8 @@
       <c r="D279" t="s">
         <v>577</v>
       </c>
-      <c r="G279" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="280" spans="1:7">
+    </row>
+    <row r="280" spans="1:4">
       <c r="A280" t="s">
         <v>285</v>
       </c>
@@ -7136,11 +6419,8 @@
       <c r="D280" t="s">
         <v>566</v>
       </c>
-      <c r="G280" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="281" spans="1:7">
+    </row>
+    <row r="281" spans="1:4">
       <c r="A281" t="s">
         <v>286</v>
       </c>
@@ -7153,11 +6433,8 @@
       <c r="D281" t="s">
         <v>578</v>
       </c>
-      <c r="G281" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="282" spans="1:7">
+    </row>
+    <row r="282" spans="1:4">
       <c r="A282" t="s">
         <v>287</v>
       </c>
@@ -7170,11 +6447,8 @@
       <c r="D282" t="s">
         <v>566</v>
       </c>
-      <c r="G282" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="283" spans="1:7">
+    </row>
+    <row r="283" spans="1:4">
       <c r="A283" t="s">
         <v>288</v>
       </c>
@@ -7186,9 +6460,6 @@
       </c>
       <c r="D283" t="s">
         <v>566</v>
-      </c>
-      <c r="G283" t="s">
-        <v>653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert — prevent duplicate sends to 242 contacts
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1192" uniqueCount="653">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="654">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -1973,6 +1973,9 @@
   </si>
   <si>
     <t>www.cmacofct.com</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -2362,6 +2365,9 @@
       <c r="F2" t="s">
         <v>633</v>
       </c>
+      <c r="G2" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
@@ -2382,6 +2388,9 @@
       <c r="F3" t="s">
         <v>633</v>
       </c>
+      <c r="G3" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
@@ -2402,6 +2411,9 @@
       <c r="F4" t="s">
         <v>633</v>
       </c>
+      <c r="G4" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -2422,6 +2434,9 @@
       <c r="F5" t="s">
         <v>633</v>
       </c>
+      <c r="G5" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
@@ -2442,6 +2457,9 @@
       <c r="F6" t="s">
         <v>633</v>
       </c>
+      <c r="G6" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
@@ -2462,6 +2480,9 @@
       <c r="F7" t="s">
         <v>633</v>
       </c>
+      <c r="G7" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
@@ -2482,6 +2503,9 @@
       <c r="F8" t="s">
         <v>633</v>
       </c>
+      <c r="G8" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
@@ -2502,6 +2526,9 @@
       <c r="F9" t="s">
         <v>633</v>
       </c>
+      <c r="G9" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" t="s">
@@ -2522,6 +2549,9 @@
       <c r="F10" t="s">
         <v>633</v>
       </c>
+      <c r="G10" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
@@ -2542,6 +2572,9 @@
       <c r="F11" t="s">
         <v>633</v>
       </c>
+      <c r="G11" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
@@ -2562,6 +2595,9 @@
       <c r="F12" t="s">
         <v>633</v>
       </c>
+      <c r="G12" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
@@ -2582,6 +2618,9 @@
       <c r="F13" t="s">
         <v>633</v>
       </c>
+      <c r="G13" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
@@ -2602,6 +2641,9 @@
       <c r="F14" s="1" t="s">
         <v>634</v>
       </c>
+      <c r="G14" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
@@ -2622,6 +2664,9 @@
       <c r="F15" s="1" t="s">
         <v>635</v>
       </c>
+      <c r="G15" t="s">
+        <v>653</v>
+      </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
@@ -2636,8 +2681,11 @@
       <c r="D16" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="17" spans="1:4">
+      <c r="G16" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -2650,8 +2698,11 @@
       <c r="D17" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="18" spans="1:4">
+      <c r="G17" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -2664,8 +2715,11 @@
       <c r="D18" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="19" spans="1:4">
+      <c r="G18" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -2678,8 +2732,11 @@
       <c r="D19" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="20" spans="1:4">
+      <c r="G19" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -2692,8 +2749,11 @@
       <c r="D20" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="21" spans="1:4">
+      <c r="G20" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -2706,8 +2766,11 @@
       <c r="D21" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="22" spans="1:4">
+      <c r="G21" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -2720,8 +2783,11 @@
       <c r="D22" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="23" spans="1:4">
+      <c r="G22" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -2734,8 +2800,11 @@
       <c r="D23" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
+      <c r="G23" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -2748,8 +2817,11 @@
       <c r="D24" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="25" spans="1:4">
+      <c r="G24" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -2762,8 +2834,11 @@
       <c r="D25" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="26" spans="1:4">
+      <c r="G25" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -2776,8 +2851,11 @@
       <c r="D26" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="27" spans="1:4">
+      <c r="G26" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -2790,8 +2868,11 @@
       <c r="D27" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="28" spans="1:4">
+      <c r="G27" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -2804,8 +2885,11 @@
       <c r="D28" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="29" spans="1:4">
+      <c r="G28" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -2818,8 +2902,11 @@
       <c r="D29" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="30" spans="1:4">
+      <c r="G29" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -2832,8 +2919,11 @@
       <c r="D30" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="31" spans="1:4">
+      <c r="G30" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -2846,8 +2936,11 @@
       <c r="D31" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="32" spans="1:4">
+      <c r="G31" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -2860,8 +2953,11 @@
       <c r="D32" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
+      <c r="G32" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -2874,8 +2970,11 @@
       <c r="D33" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="34" spans="1:4">
+      <c r="G33" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -2888,8 +2987,11 @@
       <c r="D34" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="35" spans="1:4">
+      <c r="G34" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -2902,8 +3004,11 @@
       <c r="D35" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="36" spans="1:4">
+      <c r="G35" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -2916,8 +3021,11 @@
       <c r="D36" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="37" spans="1:4">
+      <c r="G36" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -2930,8 +3038,11 @@
       <c r="D37" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="38" spans="1:4">
+      <c r="G37" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -2944,8 +3055,11 @@
       <c r="D38" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
+      <c r="G38" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -2958,8 +3072,11 @@
       <c r="D39" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="40" spans="1:4">
+      <c r="G39" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7">
       <c r="A40" t="s">
         <v>45</v>
       </c>
@@ -2972,8 +3089,11 @@
       <c r="D40" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="41" spans="1:4">
+      <c r="G40" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7">
       <c r="A41" t="s">
         <v>46</v>
       </c>
@@ -2986,8 +3106,11 @@
       <c r="D41" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="42" spans="1:4">
+      <c r="G41" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -3000,8 +3123,11 @@
       <c r="D42" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="43" spans="1:4">
+      <c r="G42" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -3014,8 +3140,11 @@
       <c r="D43" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="44" spans="1:4">
+      <c r="G43" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -3028,8 +3157,11 @@
       <c r="D44" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="45" spans="1:4">
+      <c r="G44" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -3042,8 +3174,11 @@
       <c r="D45" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="46" spans="1:4">
+      <c r="G45" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -3056,8 +3191,11 @@
       <c r="D46" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="47" spans="1:4">
+      <c r="G46" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -3070,8 +3208,11 @@
       <c r="D47" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="48" spans="1:4">
+      <c r="G47" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -3084,8 +3225,11 @@
       <c r="D48" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="49" spans="1:4">
+      <c r="G48" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -3098,8 +3242,11 @@
       <c r="D49" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="50" spans="1:4">
+      <c r="G49" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -3112,8 +3259,11 @@
       <c r="D50" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="51" spans="1:4">
+      <c r="G50" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7">
       <c r="A51" t="s">
         <v>56</v>
       </c>
@@ -3126,8 +3276,11 @@
       <c r="D51" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="52" spans="1:4">
+      <c r="G51" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -3140,8 +3293,11 @@
       <c r="D52" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="53" spans="1:4">
+      <c r="G52" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -3154,8 +3310,11 @@
       <c r="D53" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="54" spans="1:4">
+      <c r="G53" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -3168,8 +3327,11 @@
       <c r="D54" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="55" spans="1:4">
+      <c r="G54" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7">
       <c r="A55" t="s">
         <v>60</v>
       </c>
@@ -3182,8 +3344,11 @@
       <c r="D55" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="56" spans="1:4">
+      <c r="G55" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7">
       <c r="A56" t="s">
         <v>61</v>
       </c>
@@ -3196,8 +3361,11 @@
       <c r="D56" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="57" spans="1:4">
+      <c r="G56" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7">
       <c r="A57" t="s">
         <v>62</v>
       </c>
@@ -3210,8 +3378,11 @@
       <c r="D57" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="58" spans="1:4">
+      <c r="G57" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7">
       <c r="A58" t="s">
         <v>63</v>
       </c>
@@ -3224,8 +3395,11 @@
       <c r="D58" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="59" spans="1:4">
+      <c r="G58" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -3238,8 +3412,11 @@
       <c r="D59" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="60" spans="1:4">
+      <c r="G59" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7">
       <c r="A60" t="s">
         <v>65</v>
       </c>
@@ -3252,8 +3429,11 @@
       <c r="D60" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="61" spans="1:4">
+      <c r="G60" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7">
       <c r="A61" t="s">
         <v>66</v>
       </c>
@@ -3266,8 +3446,11 @@
       <c r="D61" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="62" spans="1:4">
+      <c r="G61" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -3280,8 +3463,11 @@
       <c r="D62" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="63" spans="1:4">
+      <c r="G62" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7">
       <c r="A63" t="s">
         <v>68</v>
       </c>
@@ -3294,8 +3480,11 @@
       <c r="D63" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="64" spans="1:4">
+      <c r="G63" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7">
       <c r="A64" t="s">
         <v>69</v>
       </c>
@@ -3308,8 +3497,11 @@
       <c r="D64" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="65" spans="1:4">
+      <c r="G64" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7">
       <c r="A65" t="s">
         <v>70</v>
       </c>
@@ -3322,8 +3514,11 @@
       <c r="D65" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="66" spans="1:4">
+      <c r="G65" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7">
       <c r="A66" t="s">
         <v>71</v>
       </c>
@@ -3336,8 +3531,11 @@
       <c r="D66" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="67" spans="1:4">
+      <c r="G66" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7">
       <c r="A67" t="s">
         <v>72</v>
       </c>
@@ -3350,8 +3548,11 @@
       <c r="D67" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="68" spans="1:4">
+      <c r="G67" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7">
       <c r="A68" t="s">
         <v>73</v>
       </c>
@@ -3364,8 +3565,11 @@
       <c r="D68" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="69" spans="1:4">
+      <c r="G68" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7">
       <c r="A69" t="s">
         <v>74</v>
       </c>
@@ -3378,8 +3582,11 @@
       <c r="D69" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="70" spans="1:4">
+      <c r="G69" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7">
       <c r="A70" t="s">
         <v>75</v>
       </c>
@@ -3392,8 +3599,11 @@
       <c r="D70" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="71" spans="1:4">
+      <c r="G70" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7">
       <c r="A71" t="s">
         <v>76</v>
       </c>
@@ -3406,8 +3616,11 @@
       <c r="D71" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="72" spans="1:4">
+      <c r="G71" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7">
       <c r="A72" t="s">
         <v>77</v>
       </c>
@@ -3420,8 +3633,11 @@
       <c r="D72" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="73" spans="1:4">
+      <c r="G72" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7">
       <c r="A73" t="s">
         <v>78</v>
       </c>
@@ -3434,8 +3650,11 @@
       <c r="D73" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="74" spans="1:4">
+      <c r="G73" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7">
       <c r="A74" t="s">
         <v>79</v>
       </c>
@@ -3448,8 +3667,11 @@
       <c r="D74" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="75" spans="1:4">
+      <c r="G74" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7">
       <c r="A75" t="s">
         <v>80</v>
       </c>
@@ -3462,8 +3684,11 @@
       <c r="D75" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="76" spans="1:4">
+      <c r="G75" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7">
       <c r="A76" t="s">
         <v>81</v>
       </c>
@@ -3476,8 +3701,11 @@
       <c r="D76" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="77" spans="1:4">
+      <c r="G76" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7">
       <c r="A77" t="s">
         <v>82</v>
       </c>
@@ -3490,8 +3718,11 @@
       <c r="D77" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="78" spans="1:4">
+      <c r="G77" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -3504,8 +3735,11 @@
       <c r="D78" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="79" spans="1:4">
+      <c r="G78" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7">
       <c r="A79" t="s">
         <v>84</v>
       </c>
@@ -3518,8 +3752,11 @@
       <c r="D79" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="80" spans="1:4">
+      <c r="G79" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7">
       <c r="A80" t="s">
         <v>85</v>
       </c>
@@ -3532,8 +3769,11 @@
       <c r="D80" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="81" spans="1:4">
+      <c r="G80" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7">
       <c r="A81" t="s">
         <v>86</v>
       </c>
@@ -3546,8 +3786,11 @@
       <c r="D81" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="82" spans="1:4">
+      <c r="G81" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7">
       <c r="A82" t="s">
         <v>87</v>
       </c>
@@ -3560,8 +3803,11 @@
       <c r="D82" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="83" spans="1:4">
+      <c r="G82" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7">
       <c r="A83" t="s">
         <v>88</v>
       </c>
@@ -3574,8 +3820,11 @@
       <c r="D83" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="84" spans="1:4">
+      <c r="G83" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7">
       <c r="A84" t="s">
         <v>89</v>
       </c>
@@ -3588,8 +3837,11 @@
       <c r="D84" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="85" spans="1:4">
+      <c r="G84" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7">
       <c r="A85" t="s">
         <v>90</v>
       </c>
@@ -3602,8 +3854,11 @@
       <c r="D85" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="86" spans="1:4">
+      <c r="G85" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7">
       <c r="A86" t="s">
         <v>91</v>
       </c>
@@ -3616,8 +3871,11 @@
       <c r="D86" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="87" spans="1:4">
+      <c r="G86" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7">
       <c r="A87" t="s">
         <v>92</v>
       </c>
@@ -3630,8 +3888,11 @@
       <c r="D87" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="88" spans="1:4">
+      <c r="G87" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7">
       <c r="A88" t="s">
         <v>93</v>
       </c>
@@ -3644,8 +3905,11 @@
       <c r="D88" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="89" spans="1:4">
+      <c r="G88" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7">
       <c r="A89" t="s">
         <v>94</v>
       </c>
@@ -3658,8 +3922,11 @@
       <c r="D89" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="90" spans="1:4">
+      <c r="G89" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7">
       <c r="A90" t="s">
         <v>95</v>
       </c>
@@ -3672,8 +3939,11 @@
       <c r="D90" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="91" spans="1:4">
+      <c r="G90" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7">
       <c r="A91" t="s">
         <v>96</v>
       </c>
@@ -3686,8 +3956,11 @@
       <c r="D91" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="92" spans="1:4">
+      <c r="G91" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7">
       <c r="A92" t="s">
         <v>97</v>
       </c>
@@ -3700,8 +3973,11 @@
       <c r="D92" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="93" spans="1:4">
+      <c r="G92" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7">
       <c r="A93" t="s">
         <v>98</v>
       </c>
@@ -3714,8 +3990,11 @@
       <c r="D93" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="94" spans="1:4">
+      <c r="G93" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7">
       <c r="A94" t="s">
         <v>99</v>
       </c>
@@ -3728,8 +4007,11 @@
       <c r="D94" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="95" spans="1:4">
+      <c r="G94" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7">
       <c r="A95" t="s">
         <v>100</v>
       </c>
@@ -3742,8 +4024,11 @@
       <c r="D95" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="96" spans="1:4">
+      <c r="G95" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7">
       <c r="A96" t="s">
         <v>101</v>
       </c>
@@ -3756,8 +4041,11 @@
       <c r="D96" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="97" spans="1:4">
+      <c r="G96" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7">
       <c r="A97" t="s">
         <v>102</v>
       </c>
@@ -3770,8 +4058,11 @@
       <c r="D97" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="98" spans="1:4">
+      <c r="G97" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7">
       <c r="A98" t="s">
         <v>103</v>
       </c>
@@ -3784,8 +4075,11 @@
       <c r="D98" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="99" spans="1:4">
+      <c r="G98" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7">
       <c r="A99" t="s">
         <v>104</v>
       </c>
@@ -3798,8 +4092,11 @@
       <c r="D99" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="100" spans="1:4">
+      <c r="G99" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7">
       <c r="A100" t="s">
         <v>105</v>
       </c>
@@ -3812,8 +4109,11 @@
       <c r="D100" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="101" spans="1:4">
+      <c r="G100" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7">
       <c r="A101" t="s">
         <v>106</v>
       </c>
@@ -3826,8 +4126,11 @@
       <c r="D101" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="102" spans="1:4">
+      <c r="G101" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7">
       <c r="A102" t="s">
         <v>107</v>
       </c>
@@ -3840,8 +4143,11 @@
       <c r="D102" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="103" spans="1:4">
+      <c r="G102" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7">
       <c r="A103" t="s">
         <v>108</v>
       </c>
@@ -3854,8 +4160,11 @@
       <c r="D103" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="104" spans="1:4">
+      <c r="G103" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7">
       <c r="A104" t="s">
         <v>109</v>
       </c>
@@ -3868,8 +4177,11 @@
       <c r="D104" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="105" spans="1:4">
+      <c r="G104" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7">
       <c r="A105" t="s">
         <v>110</v>
       </c>
@@ -3882,8 +4194,11 @@
       <c r="D105" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="106" spans="1:4">
+      <c r="G105" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7">
       <c r="A106" t="s">
         <v>111</v>
       </c>
@@ -3896,8 +4211,11 @@
       <c r="D106" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="107" spans="1:4">
+      <c r="G106" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7">
       <c r="A107" t="s">
         <v>112</v>
       </c>
@@ -3910,8 +4228,11 @@
       <c r="D107" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="108" spans="1:4">
+      <c r="G107" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7">
       <c r="A108" t="s">
         <v>113</v>
       </c>
@@ -3924,8 +4245,11 @@
       <c r="D108" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="109" spans="1:4">
+      <c r="G108" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7">
       <c r="A109" t="s">
         <v>114</v>
       </c>
@@ -3938,8 +4262,11 @@
       <c r="D109" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="110" spans="1:4">
+      <c r="G109" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7">
       <c r="A110" t="s">
         <v>115</v>
       </c>
@@ -3952,8 +4279,11 @@
       <c r="D110" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="111" spans="1:4">
+      <c r="G110" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7">
       <c r="A111" t="s">
         <v>116</v>
       </c>
@@ -3966,8 +4296,11 @@
       <c r="D111" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="112" spans="1:4">
+      <c r="G111" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7">
       <c r="A112" t="s">
         <v>117</v>
       </c>
@@ -3980,8 +4313,11 @@
       <c r="D112" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="113" spans="1:6">
+      <c r="G112" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7">
       <c r="A113" t="s">
         <v>118</v>
       </c>
@@ -3994,8 +4330,11 @@
       <c r="D113" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="114" spans="1:6">
+      <c r="G113" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7">
       <c r="A114" t="s">
         <v>119</v>
       </c>
@@ -4008,8 +4347,11 @@
       <c r="D114" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="115" spans="1:6">
+      <c r="G114" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7">
       <c r="A115" t="s">
         <v>120</v>
       </c>
@@ -4022,8 +4364,11 @@
       <c r="D115" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="116" spans="1:6">
+      <c r="G115" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7">
       <c r="A116" t="s">
         <v>121</v>
       </c>
@@ -4036,8 +4381,11 @@
       <c r="D116" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="117" spans="1:6">
+      <c r="G116" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7">
       <c r="A117" t="s">
         <v>122</v>
       </c>
@@ -4050,8 +4398,11 @@
       <c r="D117" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="118" spans="1:6">
+      <c r="G117" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7">
       <c r="A118" t="s">
         <v>123</v>
       </c>
@@ -4064,8 +4415,11 @@
       <c r="D118" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="119" spans="1:6">
+      <c r="G118" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7">
       <c r="A119" t="s">
         <v>124</v>
       </c>
@@ -4084,8 +4438,11 @@
       <c r="F119" t="s">
         <v>636</v>
       </c>
-    </row>
-    <row r="120" spans="1:6">
+      <c r="G119" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7">
       <c r="A120" t="s">
         <v>125</v>
       </c>
@@ -4101,8 +4458,11 @@
       <c r="E120" t="s">
         <v>583</v>
       </c>
-    </row>
-    <row r="121" spans="1:6">
+      <c r="G120" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7">
       <c r="A121" t="s">
         <v>126</v>
       </c>
@@ -4115,8 +4475,11 @@
       <c r="D121" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="122" spans="1:6">
+      <c r="G121" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7">
       <c r="A122" t="s">
         <v>127</v>
       </c>
@@ -4129,8 +4492,11 @@
       <c r="D122" t="s">
         <v>555</v>
       </c>
-    </row>
-    <row r="123" spans="1:6">
+      <c r="G122" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7">
       <c r="A123" t="s">
         <v>128</v>
       </c>
@@ -4149,8 +4515,11 @@
       <c r="F123" t="s">
         <v>637</v>
       </c>
-    </row>
-    <row r="124" spans="1:6">
+      <c r="G123" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7">
       <c r="A124" t="s">
         <v>129</v>
       </c>
@@ -4163,8 +4532,11 @@
       <c r="D124" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="125" spans="1:6">
+      <c r="G124" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7">
       <c r="A125" t="s">
         <v>130</v>
       </c>
@@ -4177,8 +4549,11 @@
       <c r="D125" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="126" spans="1:6">
+      <c r="G125" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7">
       <c r="A126" t="s">
         <v>131</v>
       </c>
@@ -4191,8 +4566,11 @@
       <c r="D126" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="127" spans="1:6">
+      <c r="G126" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7">
       <c r="A127" t="s">
         <v>132</v>
       </c>
@@ -4205,8 +4583,11 @@
       <c r="D127" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="128" spans="1:6">
+      <c r="G127" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7">
       <c r="A128" t="s">
         <v>133</v>
       </c>
@@ -4222,8 +4603,11 @@
       <c r="E128" t="s">
         <v>585</v>
       </c>
-    </row>
-    <row r="129" spans="1:6">
+      <c r="G128" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7">
       <c r="A129" t="s">
         <v>134</v>
       </c>
@@ -4242,8 +4626,11 @@
       <c r="F129" t="s">
         <v>638</v>
       </c>
-    </row>
-    <row r="130" spans="1:6">
+      <c r="G129" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7">
       <c r="A130" t="s">
         <v>135</v>
       </c>
@@ -4256,8 +4643,11 @@
       <c r="D130" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="131" spans="1:6">
+      <c r="G130" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7">
       <c r="A131" t="s">
         <v>136</v>
       </c>
@@ -4271,7 +4661,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:7">
       <c r="A132" t="s">
         <v>137</v>
       </c>
@@ -4287,8 +4677,11 @@
       <c r="E132" t="s">
         <v>588</v>
       </c>
-    </row>
-    <row r="133" spans="1:6">
+      <c r="G132" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7">
       <c r="A133" t="s">
         <v>138</v>
       </c>
@@ -4304,8 +4697,11 @@
       <c r="E133" t="s">
         <v>589</v>
       </c>
-    </row>
-    <row r="134" spans="1:6">
+      <c r="G133" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7">
       <c r="A134" t="s">
         <v>139</v>
       </c>
@@ -4316,7 +4712,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:7">
       <c r="A135" t="s">
         <v>140</v>
       </c>
@@ -4327,7 +4723,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:7">
       <c r="A136" t="s">
         <v>141</v>
       </c>
@@ -4340,8 +4736,11 @@
       <c r="D136" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="137" spans="1:6">
+      <c r="G136" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7">
       <c r="A137" t="s">
         <v>142</v>
       </c>
@@ -4354,8 +4753,11 @@
       <c r="D137" t="s">
         <v>558</v>
       </c>
-    </row>
-    <row r="138" spans="1:6">
+      <c r="G137" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7">
       <c r="A138" t="s">
         <v>143</v>
       </c>
@@ -4366,7 +4768,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:7">
       <c r="A139" t="s">
         <v>144</v>
       </c>
@@ -4377,7 +4779,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:7">
       <c r="A140" t="s">
         <v>145</v>
       </c>
@@ -4388,7 +4790,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="141" spans="1:6">
+    <row r="141" spans="1:7">
       <c r="A141" t="s">
         <v>146</v>
       </c>
@@ -4401,8 +4803,11 @@
       <c r="D141" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="142" spans="1:6">
+      <c r="G141" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7">
       <c r="A142" t="s">
         <v>147</v>
       </c>
@@ -4421,8 +4826,11 @@
       <c r="F142" t="s">
         <v>639</v>
       </c>
-    </row>
-    <row r="143" spans="1:6">
+      <c r="G142" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7">
       <c r="A143" t="s">
         <v>148</v>
       </c>
@@ -4435,8 +4843,11 @@
       <c r="D143" t="s">
         <v>562</v>
       </c>
-    </row>
-    <row r="144" spans="1:6">
+      <c r="G143" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7">
       <c r="A144" t="s">
         <v>149</v>
       </c>
@@ -4450,7 +4861,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:7">
       <c r="A145" t="s">
         <v>150</v>
       </c>
@@ -4461,7 +4872,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:7">
       <c r="A146" t="s">
         <v>151</v>
       </c>
@@ -4477,8 +4888,11 @@
       <c r="F146" t="s">
         <v>640</v>
       </c>
-    </row>
-    <row r="147" spans="1:6">
+      <c r="G146" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7">
       <c r="A147" t="s">
         <v>152</v>
       </c>
@@ -4497,8 +4911,11 @@
       <c r="F147" t="s">
         <v>641</v>
       </c>
-    </row>
-    <row r="148" spans="1:6">
+      <c r="G147" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7">
       <c r="A148" t="s">
         <v>153</v>
       </c>
@@ -4514,8 +4931,11 @@
       <c r="E148" t="s">
         <v>593</v>
       </c>
-    </row>
-    <row r="149" spans="1:6">
+      <c r="G148" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7">
       <c r="A149" t="s">
         <v>154</v>
       </c>
@@ -4531,8 +4951,11 @@
       <c r="E149" t="s">
         <v>594</v>
       </c>
-    </row>
-    <row r="150" spans="1:6">
+      <c r="G149" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7">
       <c r="A150" t="s">
         <v>155</v>
       </c>
@@ -4548,8 +4971,11 @@
       <c r="E150" t="s">
         <v>595</v>
       </c>
-    </row>
-    <row r="151" spans="1:6">
+      <c r="G150" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7">
       <c r="A151" t="s">
         <v>156</v>
       </c>
@@ -4565,8 +4991,11 @@
       <c r="E151" t="s">
         <v>596</v>
       </c>
-    </row>
-    <row r="152" spans="1:6">
+      <c r="G151" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7">
       <c r="A152" t="s">
         <v>157</v>
       </c>
@@ -4582,8 +5011,11 @@
       <c r="E152" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="153" spans="1:6">
+      <c r="G152" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7">
       <c r="A153" t="s">
         <v>158</v>
       </c>
@@ -4594,7 +5026,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="154" spans="1:6">
+    <row r="154" spans="1:7">
       <c r="A154" t="s">
         <v>159</v>
       </c>
@@ -4610,8 +5042,11 @@
       <c r="E154" t="s">
         <v>598</v>
       </c>
-    </row>
-    <row r="155" spans="1:6">
+      <c r="G154" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7">
       <c r="A155" t="s">
         <v>160</v>
       </c>
@@ -4624,8 +5059,11 @@
       <c r="D155" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="156" spans="1:6">
+      <c r="G155" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7">
       <c r="A156" t="s">
         <v>161</v>
       </c>
@@ -4638,8 +5076,11 @@
       <c r="D156" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="157" spans="1:6">
+      <c r="G156" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7">
       <c r="A157" t="s">
         <v>162</v>
       </c>
@@ -4658,8 +5099,11 @@
       <c r="F157" t="s">
         <v>642</v>
       </c>
-    </row>
-    <row r="158" spans="1:6">
+      <c r="G157" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7">
       <c r="A158" t="s">
         <v>163</v>
       </c>
@@ -4675,8 +5119,11 @@
       <c r="E158" t="s">
         <v>600</v>
       </c>
-    </row>
-    <row r="159" spans="1:6">
+      <c r="G158" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7">
       <c r="A159" t="s">
         <v>164</v>
       </c>
@@ -4692,8 +5139,11 @@
       <c r="E159" t="s">
         <v>601</v>
       </c>
-    </row>
-    <row r="160" spans="1:6">
+      <c r="G159" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7">
       <c r="A160" t="s">
         <v>165</v>
       </c>
@@ -4709,8 +5159,11 @@
       <c r="E160" t="s">
         <v>602</v>
       </c>
-    </row>
-    <row r="161" spans="1:6">
+      <c r="G160" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7">
       <c r="A161" t="s">
         <v>166</v>
       </c>
@@ -4726,8 +5179,11 @@
       <c r="E161" t="s">
         <v>603</v>
       </c>
-    </row>
-    <row r="162" spans="1:6">
+      <c r="G161" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7">
       <c r="A162" t="s">
         <v>167</v>
       </c>
@@ -4740,8 +5196,11 @@
       <c r="D162" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="163" spans="1:6">
+      <c r="G162" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7">
       <c r="A163" t="s">
         <v>168</v>
       </c>
@@ -4757,8 +5216,11 @@
       <c r="E163" t="s">
         <v>604</v>
       </c>
-    </row>
-    <row r="164" spans="1:6">
+      <c r="G163" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7">
       <c r="A164" t="s">
         <v>169</v>
       </c>
@@ -4774,8 +5236,11 @@
       <c r="E164" t="s">
         <v>605</v>
       </c>
-    </row>
-    <row r="165" spans="1:6">
+      <c r="G164" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7">
       <c r="A165" t="s">
         <v>170</v>
       </c>
@@ -4789,7 +5254,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:7">
       <c r="A166" t="s">
         <v>171</v>
       </c>
@@ -4805,8 +5270,11 @@
       <c r="E166" t="s">
         <v>607</v>
       </c>
-    </row>
-    <row r="167" spans="1:6">
+      <c r="G166" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7">
       <c r="A167" t="s">
         <v>172</v>
       </c>
@@ -4822,8 +5290,11 @@
       <c r="E167" t="s">
         <v>608</v>
       </c>
-    </row>
-    <row r="168" spans="1:6">
+      <c r="G167" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7">
       <c r="A168" t="s">
         <v>173</v>
       </c>
@@ -4839,8 +5310,11 @@
       <c r="E168" t="s">
         <v>609</v>
       </c>
-    </row>
-    <row r="169" spans="1:6">
+      <c r="G168" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7">
       <c r="A169" t="s">
         <v>174</v>
       </c>
@@ -4856,8 +5330,11 @@
       <c r="E169" t="s">
         <v>610</v>
       </c>
-    </row>
-    <row r="170" spans="1:6">
+      <c r="G169" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7">
       <c r="A170" t="s">
         <v>175</v>
       </c>
@@ -4871,7 +5348,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="171" spans="1:6">
+    <row r="171" spans="1:7">
       <c r="A171" t="s">
         <v>176</v>
       </c>
@@ -4885,7 +5362,7 @@
         <v>612</v>
       </c>
     </row>
-    <row r="172" spans="1:6">
+    <row r="172" spans="1:7">
       <c r="A172" t="s">
         <v>177</v>
       </c>
@@ -4899,7 +5376,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="173" spans="1:6">
+    <row r="173" spans="1:7">
       <c r="A173" t="s">
         <v>178</v>
       </c>
@@ -4912,8 +5389,11 @@
       <c r="D173" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="174" spans="1:6">
+      <c r="G173" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7">
       <c r="A174" t="s">
         <v>179</v>
       </c>
@@ -4929,8 +5409,11 @@
       <c r="F174" t="s">
         <v>643</v>
       </c>
-    </row>
-    <row r="175" spans="1:6">
+      <c r="G174" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7">
       <c r="A175" t="s">
         <v>180</v>
       </c>
@@ -4946,8 +5429,11 @@
       <c r="F175" t="s">
         <v>644</v>
       </c>
-    </row>
-    <row r="176" spans="1:6">
+      <c r="G175" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7">
       <c r="A176" t="s">
         <v>181</v>
       </c>
@@ -4958,7 +5444,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:7">
       <c r="A177" t="s">
         <v>182</v>
       </c>
@@ -4969,7 +5455,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:7">
       <c r="A178" t="s">
         <v>183</v>
       </c>
@@ -4980,7 +5466,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:7">
       <c r="A179" t="s">
         <v>184</v>
       </c>
@@ -4999,8 +5485,11 @@
       <c r="F179" t="s">
         <v>645</v>
       </c>
-    </row>
-    <row r="180" spans="1:6">
+      <c r="G179" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7">
       <c r="A180" t="s">
         <v>185</v>
       </c>
@@ -5011,7 +5500,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="181" spans="1:6">
+    <row r="181" spans="1:7">
       <c r="A181" t="s">
         <v>186</v>
       </c>
@@ -5022,7 +5511,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="182" spans="1:6">
+    <row r="182" spans="1:7">
       <c r="A182" t="s">
         <v>187</v>
       </c>
@@ -5038,8 +5527,11 @@
       <c r="E182" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="183" spans="1:6">
+      <c r="G182" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7">
       <c r="A183" t="s">
         <v>188</v>
       </c>
@@ -5055,8 +5547,11 @@
       <c r="F183" t="s">
         <v>646</v>
       </c>
-    </row>
-    <row r="184" spans="1:6">
+      <c r="G183" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7">
       <c r="A184" t="s">
         <v>189</v>
       </c>
@@ -5067,7 +5562,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="185" spans="1:6">
+    <row r="185" spans="1:7">
       <c r="A185" t="s">
         <v>190</v>
       </c>
@@ -5081,7 +5576,7 @@
         <v>647</v>
       </c>
     </row>
-    <row r="186" spans="1:6">
+    <row r="186" spans="1:7">
       <c r="A186" t="s">
         <v>191</v>
       </c>
@@ -5095,7 +5590,7 @@
         <v>616</v>
       </c>
     </row>
-    <row r="187" spans="1:6">
+    <row r="187" spans="1:7">
       <c r="A187" t="s">
         <v>192</v>
       </c>
@@ -5109,7 +5604,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="188" spans="1:6">
+    <row r="188" spans="1:7">
       <c r="A188" t="s">
         <v>193</v>
       </c>
@@ -5123,7 +5618,7 @@
         <v>618</v>
       </c>
     </row>
-    <row r="189" spans="1:6">
+    <row r="189" spans="1:7">
       <c r="A189" t="s">
         <v>194</v>
       </c>
@@ -5137,7 +5632,7 @@
         <v>619</v>
       </c>
     </row>
-    <row r="190" spans="1:6">
+    <row r="190" spans="1:7">
       <c r="A190" t="s">
         <v>195</v>
       </c>
@@ -5151,7 +5646,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="191" spans="1:6">
+    <row r="191" spans="1:7">
       <c r="A191" t="s">
         <v>196</v>
       </c>
@@ -5162,7 +5657,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="192" spans="1:6">
+    <row r="192" spans="1:7">
       <c r="A192" t="s">
         <v>197</v>
       </c>
@@ -5173,7 +5668,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="193" spans="1:6">
+    <row r="193" spans="1:7">
       <c r="A193" t="s">
         <v>198</v>
       </c>
@@ -5184,7 +5679,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="194" spans="1:6">
+    <row r="194" spans="1:7">
       <c r="A194" t="s">
         <v>199</v>
       </c>
@@ -5197,8 +5692,11 @@
       <c r="D194" t="s">
         <v>555</v>
       </c>
-    </row>
-    <row r="195" spans="1:6">
+      <c r="G194" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7">
       <c r="A195" t="s">
         <v>200</v>
       </c>
@@ -5211,8 +5709,11 @@
       <c r="D195" t="s">
         <v>555</v>
       </c>
-    </row>
-    <row r="196" spans="1:6">
+      <c r="G195" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7">
       <c r="A196" t="s">
         <v>201</v>
       </c>
@@ -5228,8 +5729,11 @@
       <c r="F196" t="s">
         <v>648</v>
       </c>
-    </row>
-    <row r="197" spans="1:6">
+      <c r="G196" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7">
       <c r="A197" t="s">
         <v>202</v>
       </c>
@@ -5248,8 +5752,11 @@
       <c r="F197" t="s">
         <v>649</v>
       </c>
-    </row>
-    <row r="198" spans="1:6">
+      <c r="G197" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7">
       <c r="A198" t="s">
         <v>203</v>
       </c>
@@ -5268,8 +5775,11 @@
       <c r="F198" t="s">
         <v>650</v>
       </c>
-    </row>
-    <row r="199" spans="1:6">
+      <c r="G198" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7">
       <c r="A199" t="s">
         <v>204</v>
       </c>
@@ -5288,8 +5798,11 @@
       <c r="F199" t="s">
         <v>651</v>
       </c>
-    </row>
-    <row r="200" spans="1:6">
+      <c r="G199" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7">
       <c r="A200" t="s">
         <v>205</v>
       </c>
@@ -5302,8 +5815,11 @@
       <c r="D200" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="201" spans="1:6">
+      <c r="G200" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7">
       <c r="A201" t="s">
         <v>206</v>
       </c>
@@ -5314,7 +5830,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="202" spans="1:6">
+    <row r="202" spans="1:7">
       <c r="A202" t="s">
         <v>207</v>
       </c>
@@ -5325,7 +5841,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="203" spans="1:6">
+    <row r="203" spans="1:7">
       <c r="A203" t="s">
         <v>208</v>
       </c>
@@ -5336,7 +5852,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="204" spans="1:6">
+    <row r="204" spans="1:7">
       <c r="A204" t="s">
         <v>209</v>
       </c>
@@ -5349,8 +5865,11 @@
       <c r="D204" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="205" spans="1:6">
+      <c r="G204" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7">
       <c r="A205" t="s">
         <v>210</v>
       </c>
@@ -5361,7 +5880,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="206" spans="1:6">
+    <row r="206" spans="1:7">
       <c r="A206" t="s">
         <v>211</v>
       </c>
@@ -5372,7 +5891,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="207" spans="1:6">
+    <row r="207" spans="1:7">
       <c r="A207" t="s">
         <v>212</v>
       </c>
@@ -5388,8 +5907,11 @@
       <c r="E207" t="s">
         <v>624</v>
       </c>
-    </row>
-    <row r="208" spans="1:6">
+      <c r="G207" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7">
       <c r="A208" t="s">
         <v>213</v>
       </c>
@@ -5403,7 +5925,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="209" spans="1:5">
+    <row r="209" spans="1:7">
       <c r="A209" t="s">
         <v>214</v>
       </c>
@@ -5414,7 +5936,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="210" spans="1:5">
+    <row r="210" spans="1:7">
       <c r="A210" t="s">
         <v>215</v>
       </c>
@@ -5430,8 +5952,11 @@
       <c r="E210" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="211" spans="1:5">
+      <c r="G210" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7">
       <c r="A211" t="s">
         <v>216</v>
       </c>
@@ -5444,8 +5969,11 @@
       <c r="D211" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="212" spans="1:5">
+      <c r="G211" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7">
       <c r="A212" t="s">
         <v>217</v>
       </c>
@@ -5459,7 +5987,7 @@
         <v>627</v>
       </c>
     </row>
-    <row r="213" spans="1:5">
+    <row r="213" spans="1:7">
       <c r="A213" t="s">
         <v>218</v>
       </c>
@@ -5473,7 +6001,7 @@
         <v>628</v>
       </c>
     </row>
-    <row r="214" spans="1:5">
+    <row r="214" spans="1:7">
       <c r="A214" t="s">
         <v>219</v>
       </c>
@@ -5486,8 +6014,11 @@
       <c r="D214" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="215" spans="1:5">
+      <c r="G214" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7">
       <c r="A215" t="s">
         <v>220</v>
       </c>
@@ -5500,8 +6031,11 @@
       <c r="D215" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="216" spans="1:5">
+      <c r="G215" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7">
       <c r="A216" t="s">
         <v>221</v>
       </c>
@@ -5515,7 +6049,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="217" spans="1:5">
+    <row r="217" spans="1:7">
       <c r="A217" t="s">
         <v>222</v>
       </c>
@@ -5531,8 +6065,11 @@
       <c r="E217" t="s">
         <v>630</v>
       </c>
-    </row>
-    <row r="218" spans="1:5">
+      <c r="G217" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7">
       <c r="A218" t="s">
         <v>223</v>
       </c>
@@ -5548,8 +6085,11 @@
       <c r="E218" t="s">
         <v>630</v>
       </c>
-    </row>
-    <row r="219" spans="1:5">
+      <c r="G218" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7">
       <c r="A219" t="s">
         <v>224</v>
       </c>
@@ -5565,8 +6105,11 @@
       <c r="E219" t="s">
         <v>631</v>
       </c>
-    </row>
-    <row r="220" spans="1:5">
+      <c r="G219" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7">
       <c r="A220" t="s">
         <v>225</v>
       </c>
@@ -5577,7 +6120,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="221" spans="1:5">
+    <row r="221" spans="1:7">
       <c r="A221" t="s">
         <v>226</v>
       </c>
@@ -5590,8 +6133,11 @@
       <c r="D221" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="222" spans="1:5">
+      <c r="G221" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7">
       <c r="A222" t="s">
         <v>227</v>
       </c>
@@ -5607,8 +6153,11 @@
       <c r="E222" t="s">
         <v>632</v>
       </c>
-    </row>
-    <row r="223" spans="1:5">
+      <c r="G222" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7">
       <c r="A223" t="s">
         <v>228</v>
       </c>
@@ -5621,8 +6170,11 @@
       <c r="D223" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="224" spans="1:5">
+      <c r="G223" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7">
       <c r="A224" t="s">
         <v>229</v>
       </c>
@@ -5635,8 +6187,11 @@
       <c r="D224" t="s">
         <v>574</v>
       </c>
-    </row>
-    <row r="225" spans="1:6">
+      <c r="G224" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7">
       <c r="A225" t="s">
         <v>230</v>
       </c>
@@ -5652,8 +6207,11 @@
       <c r="F225" t="s">
         <v>652</v>
       </c>
-    </row>
-    <row r="226" spans="1:6">
+      <c r="G225" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7">
       <c r="A226" t="s">
         <v>231</v>
       </c>
@@ -5666,8 +6224,11 @@
       <c r="D226" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="227" spans="1:6">
+      <c r="G226" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7">
       <c r="A227" t="s">
         <v>232</v>
       </c>
@@ -5678,7 +6239,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="228" spans="1:6">
+    <row r="228" spans="1:7">
       <c r="A228" t="s">
         <v>233</v>
       </c>
@@ -5691,8 +6252,11 @@
       <c r="D228" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="229" spans="1:6">
+      <c r="G228" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7">
       <c r="A229" t="s">
         <v>234</v>
       </c>
@@ -5705,8 +6269,11 @@
       <c r="D229" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="230" spans="1:6">
+      <c r="G229" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7">
       <c r="A230" t="s">
         <v>235</v>
       </c>
@@ -5719,8 +6286,11 @@
       <c r="D230" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="231" spans="1:6">
+      <c r="G230" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7">
       <c r="A231" t="s">
         <v>236</v>
       </c>
@@ -5733,8 +6303,11 @@
       <c r="D231" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="232" spans="1:6">
+      <c r="G231" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7">
       <c r="A232" t="s">
         <v>237</v>
       </c>
@@ -5747,8 +6320,11 @@
       <c r="D232" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="233" spans="1:6">
+      <c r="G232" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7">
       <c r="A233" t="s">
         <v>238</v>
       </c>
@@ -5761,8 +6337,11 @@
       <c r="D233" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="234" spans="1:6">
+      <c r="G233" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7">
       <c r="A234" t="s">
         <v>239</v>
       </c>
@@ -5775,8 +6354,11 @@
       <c r="D234" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="235" spans="1:6">
+      <c r="G234" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7">
       <c r="A235" t="s">
         <v>240</v>
       </c>
@@ -5789,8 +6371,11 @@
       <c r="D235" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="236" spans="1:6">
+      <c r="G235" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7">
       <c r="A236" t="s">
         <v>241</v>
       </c>
@@ -5803,8 +6388,11 @@
       <c r="D236" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="237" spans="1:6">
+      <c r="G236" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7">
       <c r="A237" t="s">
         <v>242</v>
       </c>
@@ -5817,8 +6405,11 @@
       <c r="D237" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="238" spans="1:6">
+      <c r="G237" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7">
       <c r="A238" t="s">
         <v>243</v>
       </c>
@@ -5831,8 +6422,11 @@
       <c r="D238" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="239" spans="1:6">
+      <c r="G238" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7">
       <c r="A239" t="s">
         <v>244</v>
       </c>
@@ -5845,8 +6439,11 @@
       <c r="D239" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="240" spans="1:6">
+      <c r="G239" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7">
       <c r="A240" t="s">
         <v>245</v>
       </c>
@@ -5859,8 +6456,11 @@
       <c r="D240" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="241" spans="1:4">
+      <c r="G240" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7">
       <c r="A241" t="s">
         <v>246</v>
       </c>
@@ -5873,8 +6473,11 @@
       <c r="D241" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="242" spans="1:4">
+      <c r="G241" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7">
       <c r="A242" t="s">
         <v>247</v>
       </c>
@@ -5887,8 +6490,11 @@
       <c r="D242" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="243" spans="1:4">
+      <c r="G242" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7">
       <c r="A243" t="s">
         <v>248</v>
       </c>
@@ -5901,8 +6507,11 @@
       <c r="D243" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="244" spans="1:4">
+      <c r="G243" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7">
       <c r="A244" t="s">
         <v>249</v>
       </c>
@@ -5915,8 +6524,11 @@
       <c r="D244" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="245" spans="1:4">
+      <c r="G244" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7">
       <c r="A245" t="s">
         <v>250</v>
       </c>
@@ -5929,8 +6541,11 @@
       <c r="D245" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="246" spans="1:4">
+      <c r="G245" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="246" spans="1:7">
       <c r="A246" t="s">
         <v>251</v>
       </c>
@@ -5943,8 +6558,11 @@
       <c r="D246" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="247" spans="1:4">
+      <c r="G246" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7">
       <c r="A247" t="s">
         <v>252</v>
       </c>
@@ -5957,8 +6575,11 @@
       <c r="D247" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="248" spans="1:4">
+      <c r="G247" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7">
       <c r="A248" t="s">
         <v>253</v>
       </c>
@@ -5971,8 +6592,11 @@
       <c r="D248" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="249" spans="1:4">
+      <c r="G248" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="249" spans="1:7">
       <c r="A249" t="s">
         <v>254</v>
       </c>
@@ -5985,8 +6609,11 @@
       <c r="D249" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="250" spans="1:4">
+      <c r="G249" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7">
       <c r="A250" t="s">
         <v>255</v>
       </c>
@@ -5999,8 +6626,11 @@
       <c r="D250" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="251" spans="1:4">
+      <c r="G250" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7">
       <c r="A251" t="s">
         <v>256</v>
       </c>
@@ -6013,8 +6643,11 @@
       <c r="D251" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="252" spans="1:4">
+      <c r="G251" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7">
       <c r="A252" t="s">
         <v>257</v>
       </c>
@@ -6027,8 +6660,11 @@
       <c r="D252" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="253" spans="1:4">
+      <c r="G252" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="253" spans="1:7">
       <c r="A253" t="s">
         <v>258</v>
       </c>
@@ -6041,8 +6677,11 @@
       <c r="D253" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="254" spans="1:4">
+      <c r="G253" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7">
       <c r="A254" t="s">
         <v>259</v>
       </c>
@@ -6055,8 +6694,11 @@
       <c r="D254" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="255" spans="1:4">
+      <c r="G254" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="255" spans="1:7">
       <c r="A255" t="s">
         <v>260</v>
       </c>
@@ -6069,8 +6711,11 @@
       <c r="D255" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="256" spans="1:4">
+      <c r="G255" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="256" spans="1:7">
       <c r="A256" t="s">
         <v>261</v>
       </c>
@@ -6083,8 +6728,11 @@
       <c r="D256" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="257" spans="1:4">
+      <c r="G256" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7">
       <c r="A257" t="s">
         <v>262</v>
       </c>
@@ -6097,8 +6745,11 @@
       <c r="D257" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="258" spans="1:4">
+      <c r="G257" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="258" spans="1:7">
       <c r="A258" t="s">
         <v>263</v>
       </c>
@@ -6111,8 +6762,11 @@
       <c r="D258" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="259" spans="1:4">
+      <c r="G258" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7">
       <c r="A259" t="s">
         <v>264</v>
       </c>
@@ -6125,8 +6779,11 @@
       <c r="D259" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="260" spans="1:4">
+      <c r="G259" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7">
       <c r="A260" t="s">
         <v>265</v>
       </c>
@@ -6139,8 +6796,11 @@
       <c r="D260" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="261" spans="1:4">
+      <c r="G260" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7">
       <c r="A261" t="s">
         <v>266</v>
       </c>
@@ -6153,8 +6813,11 @@
       <c r="D261" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="262" spans="1:4">
+      <c r="G261" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7">
       <c r="A262" t="s">
         <v>267</v>
       </c>
@@ -6167,8 +6830,11 @@
       <c r="D262" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="263" spans="1:4">
+      <c r="G262" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="263" spans="1:7">
       <c r="A263" t="s">
         <v>268</v>
       </c>
@@ -6181,8 +6847,11 @@
       <c r="D263" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="264" spans="1:4">
+      <c r="G263" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="264" spans="1:7">
       <c r="A264" t="s">
         <v>269</v>
       </c>
@@ -6195,8 +6864,11 @@
       <c r="D264" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="265" spans="1:4">
+      <c r="G264" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="265" spans="1:7">
       <c r="A265" t="s">
         <v>270</v>
       </c>
@@ -6209,8 +6881,11 @@
       <c r="D265" t="s">
         <v>552</v>
       </c>
-    </row>
-    <row r="266" spans="1:4">
+      <c r="G265" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="266" spans="1:7">
       <c r="A266" t="s">
         <v>271</v>
       </c>
@@ -6223,8 +6898,11 @@
       <c r="D266" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="267" spans="1:4">
+      <c r="G266" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="267" spans="1:7">
       <c r="A267" t="s">
         <v>272</v>
       </c>
@@ -6237,8 +6915,11 @@
       <c r="D267" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="268" spans="1:4">
+      <c r="G267" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="268" spans="1:7">
       <c r="A268" t="s">
         <v>273</v>
       </c>
@@ -6251,8 +6932,11 @@
       <c r="D268" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="269" spans="1:4">
+      <c r="G268" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="269" spans="1:7">
       <c r="A269" t="s">
         <v>274</v>
       </c>
@@ -6265,8 +6949,11 @@
       <c r="D269" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="270" spans="1:4">
+      <c r="G269" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="270" spans="1:7">
       <c r="A270" t="s">
         <v>275</v>
       </c>
@@ -6279,8 +6966,11 @@
       <c r="D270" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="271" spans="1:4">
+      <c r="G270" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="271" spans="1:7">
       <c r="A271" t="s">
         <v>276</v>
       </c>
@@ -6293,8 +6983,11 @@
       <c r="D271" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="272" spans="1:4">
+      <c r="G271" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="272" spans="1:7">
       <c r="A272" t="s">
         <v>277</v>
       </c>
@@ -6307,8 +7000,11 @@
       <c r="D272" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="273" spans="1:4">
+      <c r="G272" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="273" spans="1:7">
       <c r="A273" t="s">
         <v>278</v>
       </c>
@@ -6321,8 +7017,11 @@
       <c r="D273" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="274" spans="1:4">
+      <c r="G273" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="274" spans="1:7">
       <c r="A274" t="s">
         <v>279</v>
       </c>
@@ -6335,8 +7034,11 @@
       <c r="D274" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="275" spans="1:4">
+      <c r="G274" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="275" spans="1:7">
       <c r="A275" t="s">
         <v>280</v>
       </c>
@@ -6349,8 +7051,11 @@
       <c r="D275" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="276" spans="1:4">
+      <c r="G275" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="276" spans="1:7">
       <c r="A276" t="s">
         <v>281</v>
       </c>
@@ -6363,8 +7068,11 @@
       <c r="D276" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="277" spans="1:4">
+      <c r="G276" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="277" spans="1:7">
       <c r="A277" t="s">
         <v>282</v>
       </c>
@@ -6377,8 +7085,11 @@
       <c r="D277" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="278" spans="1:4">
+      <c r="G277" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="278" spans="1:7">
       <c r="A278" t="s">
         <v>283</v>
       </c>
@@ -6391,8 +7102,11 @@
       <c r="D278" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="279" spans="1:4">
+      <c r="G278" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="279" spans="1:7">
       <c r="A279" t="s">
         <v>284</v>
       </c>
@@ -6405,8 +7119,11 @@
       <c r="D279" t="s">
         <v>577</v>
       </c>
-    </row>
-    <row r="280" spans="1:4">
+      <c r="G279" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="280" spans="1:7">
       <c r="A280" t="s">
         <v>285</v>
       </c>
@@ -6419,8 +7136,11 @@
       <c r="D280" t="s">
         <v>566</v>
       </c>
-    </row>
-    <row r="281" spans="1:4">
+      <c r="G280" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="281" spans="1:7">
       <c r="A281" t="s">
         <v>286</v>
       </c>
@@ -6433,8 +7153,11 @@
       <c r="D281" t="s">
         <v>578</v>
       </c>
-    </row>
-    <row r="282" spans="1:4">
+      <c r="G281" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="282" spans="1:7">
       <c r="A282" t="s">
         <v>287</v>
       </c>
@@ -6447,8 +7170,11 @@
       <c r="D282" t="s">
         <v>566</v>
       </c>
-    </row>
-    <row r="283" spans="1:4">
+      <c r="G282" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="283" spans="1:7">
       <c r="A283" t="s">
         <v>288</v>
       </c>
@@ -6460,6 +7186,9 @@
       </c>
       <c r="D283" t="s">
         <v>566</v>
+      </c>
+      <c r="G283" t="s">
+        <v>653</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark Mowbray/Rondebosch batch complete
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1560" uniqueCount="703">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -7405,6 +7405,9 @@
       <c r="D287" t="s">
         <v>626</v>
       </c>
+      <c r="G287" t="s">
+        <v>702</v>
+      </c>
     </row>
     <row r="288" spans="1:7">
       <c r="A288" t="s">
@@ -7419,8 +7422,11 @@
       <c r="D288" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="289" spans="1:4">
+      <c r="G288" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="289" spans="1:7">
       <c r="A289" t="s">
         <v>294</v>
       </c>
@@ -7433,8 +7439,11 @@
       <c r="D289" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="290" spans="1:4">
+      <c r="G289" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="290" spans="1:7">
       <c r="A290" t="s">
         <v>295</v>
       </c>
@@ -7447,8 +7456,11 @@
       <c r="D290" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="291" spans="1:4">
+      <c r="G290" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="291" spans="1:7">
       <c r="A291" t="s">
         <v>296</v>
       </c>
@@ -7461,8 +7473,11 @@
       <c r="D291" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="292" spans="1:4">
+      <c r="G291" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="292" spans="1:7">
       <c r="A292" t="s">
         <v>297</v>
       </c>
@@ -7475,8 +7490,11 @@
       <c r="D292" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="293" spans="1:4">
+      <c r="G292" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="293" spans="1:7">
       <c r="A293" t="s">
         <v>298</v>
       </c>
@@ -7489,8 +7507,11 @@
       <c r="D293" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="294" spans="1:4">
+      <c r="G293" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="294" spans="1:7">
       <c r="A294" t="s">
         <v>299</v>
       </c>
@@ -7503,8 +7524,11 @@
       <c r="D294" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="295" spans="1:4">
+      <c r="G294" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="295" spans="1:7">
       <c r="A295" t="s">
         <v>135</v>
       </c>
@@ -7517,8 +7541,11 @@
       <c r="D295" t="s">
         <v>626</v>
       </c>
-    </row>
-    <row r="296" spans="1:4">
+      <c r="G295" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="296" spans="1:7">
       <c r="A296" t="s">
         <v>300</v>
       </c>
@@ -7531,8 +7558,11 @@
       <c r="D296" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="297" spans="1:4">
+      <c r="G296" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="297" spans="1:7">
       <c r="A297" t="s">
         <v>301</v>
       </c>
@@ -7545,8 +7575,11 @@
       <c r="D297" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="298" spans="1:4">
+      <c r="G297" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="298" spans="1:7">
       <c r="A298" t="s">
         <v>302</v>
       </c>
@@ -7559,8 +7592,11 @@
       <c r="D298" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="299" spans="1:4">
+      <c r="G298" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="299" spans="1:7">
       <c r="A299" t="s">
         <v>303</v>
       </c>
@@ -7573,8 +7609,11 @@
       <c r="D299" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="300" spans="1:4">
+      <c r="G299" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="300" spans="1:7">
       <c r="A300" t="s">
         <v>304</v>
       </c>
@@ -7587,8 +7626,11 @@
       <c r="D300" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="301" spans="1:4">
+      <c r="G300" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="301" spans="1:7">
       <c r="A301" t="s">
         <v>305</v>
       </c>
@@ -7601,8 +7643,11 @@
       <c r="D301" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="302" spans="1:4">
+      <c r="G301" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="302" spans="1:7">
       <c r="A302" t="s">
         <v>306</v>
       </c>
@@ -7615,8 +7660,11 @@
       <c r="D302" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="303" spans="1:4">
+      <c r="G302" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="303" spans="1:7">
       <c r="A303" t="s">
         <v>307</v>
       </c>
@@ -7629,8 +7677,11 @@
       <c r="D303" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="304" spans="1:4">
+      <c r="G303" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="304" spans="1:7">
       <c r="A304" t="s">
         <v>308</v>
       </c>
@@ -7643,8 +7694,11 @@
       <c r="D304" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="305" spans="1:4">
+      <c r="G304" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="305" spans="1:7">
       <c r="A305" t="s">
         <v>309</v>
       </c>
@@ -7657,8 +7711,11 @@
       <c r="D305" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="306" spans="1:4">
+      <c r="G305" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="306" spans="1:7">
       <c r="A306" t="s">
         <v>310</v>
       </c>
@@ -7671,8 +7728,11 @@
       <c r="D306" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="307" spans="1:4">
+      <c r="G306" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="307" spans="1:7">
       <c r="A307" t="s">
         <v>311</v>
       </c>
@@ -7685,8 +7745,11 @@
       <c r="D307" t="s">
         <v>615</v>
       </c>
-    </row>
-    <row r="308" spans="1:4">
+      <c r="G307" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="308" spans="1:7">
       <c r="A308" t="s">
         <v>312</v>
       </c>
@@ -7698,6 +7761,9 @@
       </c>
       <c r="D308" t="s">
         <v>627</v>
+      </c>
+      <c r="G308" t="s">
+        <v>702</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark 5 Mowbray/Rondebosch contacts as Sent
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1645" uniqueCount="745">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1650" uniqueCount="745">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -8111,7 +8111,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="321" spans="1:4">
+    <row r="321" spans="1:7">
       <c r="A321" t="s">
         <v>330</v>
       </c>
@@ -8124,8 +8124,11 @@
       <c r="D321" t="s">
         <v>653</v>
       </c>
-    </row>
-    <row r="322" spans="1:4">
+      <c r="G321" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="322" spans="1:7">
       <c r="A322" t="s">
         <v>300</v>
       </c>
@@ -8138,8 +8141,11 @@
       <c r="D322" t="s">
         <v>664</v>
       </c>
-    </row>
-    <row r="323" spans="1:4">
+      <c r="G322" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="323" spans="1:7">
       <c r="A323" t="s">
         <v>331</v>
       </c>
@@ -8152,8 +8158,11 @@
       <c r="D323" t="s">
         <v>653</v>
       </c>
-    </row>
-    <row r="324" spans="1:4">
+      <c r="G323" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="324" spans="1:7">
       <c r="A324" t="s">
         <v>332</v>
       </c>
@@ -8166,8 +8175,11 @@
       <c r="D324" t="s">
         <v>664</v>
       </c>
-    </row>
-    <row r="325" spans="1:4">
+      <c r="G324" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="325" spans="1:7">
       <c r="A325" t="s">
         <v>333</v>
       </c>
@@ -8179,6 +8191,9 @@
       </c>
       <c r="D325" t="s">
         <v>653</v>
+      </c>
+      <c r="G325" t="s">
+        <v>744</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manual scrape + send batch 20261015-1549
</commit_message>
<xml_diff>
--- a/results/master_contacts.xlsx
+++ b/results/master_contacts.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2289" uniqueCount="1018">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2328" uniqueCount="1018">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -10424,6 +10424,9 @@
       <c r="F406" s="1" t="s">
         <v>985</v>
       </c>
+      <c r="G406" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="407" spans="1:7">
       <c r="A407" t="s">
@@ -10444,6 +10447,9 @@
       <c r="F407" s="1" t="s">
         <v>985</v>
       </c>
+      <c r="G407" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="408" spans="1:7">
       <c r="A408" t="s">
@@ -10464,6 +10470,9 @@
       <c r="F408" s="1" t="s">
         <v>986</v>
       </c>
+      <c r="G408" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="409" spans="1:7">
       <c r="A409" t="s">
@@ -10484,6 +10493,9 @@
       <c r="F409" s="1" t="s">
         <v>987</v>
       </c>
+      <c r="G409" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="410" spans="1:7">
       <c r="A410" t="s">
@@ -10501,6 +10513,9 @@
       <c r="F410" s="1" t="s">
         <v>988</v>
       </c>
+      <c r="G410" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="411" spans="1:7">
       <c r="A411" t="s">
@@ -10521,6 +10536,9 @@
       <c r="F411" s="1" t="s">
         <v>989</v>
       </c>
+      <c r="G411" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="412" spans="1:7">
       <c r="A412" t="s">
@@ -10541,6 +10559,9 @@
       <c r="F412" s="1" t="s">
         <v>989</v>
       </c>
+      <c r="G412" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="413" spans="1:7">
       <c r="A413" t="s">
@@ -10561,6 +10582,9 @@
       <c r="F413" s="1" t="s">
         <v>990</v>
       </c>
+      <c r="G413" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="414" spans="1:7">
       <c r="A414" t="s">
@@ -10581,6 +10605,9 @@
       <c r="F414" s="1" t="s">
         <v>991</v>
       </c>
+      <c r="G414" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="415" spans="1:7">
       <c r="A415" t="s">
@@ -10601,6 +10628,9 @@
       <c r="F415" s="1" t="s">
         <v>992</v>
       </c>
+      <c r="G415" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="416" spans="1:7">
       <c r="A416" t="s">
@@ -10621,8 +10651,11 @@
       <c r="F416" s="1" t="s">
         <v>992</v>
       </c>
-    </row>
-    <row r="417" spans="1:6">
+      <c r="G416" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="417" spans="1:7">
       <c r="A417" t="s">
         <v>399</v>
       </c>
@@ -10641,8 +10674,11 @@
       <c r="F417" s="1" t="s">
         <v>993</v>
       </c>
-    </row>
-    <row r="418" spans="1:6">
+      <c r="G417" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="418" spans="1:7">
       <c r="A418" t="s">
         <v>400</v>
       </c>
@@ -10661,8 +10697,11 @@
       <c r="F418" s="1" t="s">
         <v>994</v>
       </c>
-    </row>
-    <row r="419" spans="1:6">
+      <c r="G418" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="419" spans="1:7">
       <c r="A419" t="s">
         <v>401</v>
       </c>
@@ -10681,8 +10720,11 @@
       <c r="F419" s="1" t="s">
         <v>995</v>
       </c>
-    </row>
-    <row r="420" spans="1:6">
+      <c r="G419" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="420" spans="1:7">
       <c r="A420" t="s">
         <v>402</v>
       </c>
@@ -10701,8 +10743,11 @@
       <c r="F420" s="1" t="s">
         <v>996</v>
       </c>
-    </row>
-    <row r="421" spans="1:6">
+      <c r="G420" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="421" spans="1:7">
       <c r="A421" t="s">
         <v>403</v>
       </c>
@@ -10721,8 +10766,11 @@
       <c r="F421" s="1" t="s">
         <v>997</v>
       </c>
-    </row>
-    <row r="422" spans="1:6">
+      <c r="G421" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="422" spans="1:7">
       <c r="A422" t="s">
         <v>404</v>
       </c>
@@ -10741,8 +10789,11 @@
       <c r="F422" s="1" t="s">
         <v>998</v>
       </c>
-    </row>
-    <row r="423" spans="1:6">
+      <c r="G422" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="423" spans="1:7">
       <c r="A423" t="s">
         <v>405</v>
       </c>
@@ -10761,8 +10812,11 @@
       <c r="F423" s="1" t="s">
         <v>999</v>
       </c>
-    </row>
-    <row r="424" spans="1:6">
+      <c r="G423" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="424" spans="1:7">
       <c r="A424" t="s">
         <v>405</v>
       </c>
@@ -10781,8 +10835,11 @@
       <c r="F424" s="1" t="s">
         <v>999</v>
       </c>
-    </row>
-    <row r="425" spans="1:6">
+      <c r="G424" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="425" spans="1:7">
       <c r="A425" t="s">
         <v>406</v>
       </c>
@@ -10801,8 +10858,11 @@
       <c r="F425" s="1" t="s">
         <v>1000</v>
       </c>
-    </row>
-    <row r="426" spans="1:6">
+      <c r="G425" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="426" spans="1:7">
       <c r="A426" t="s">
         <v>407</v>
       </c>
@@ -10821,8 +10881,11 @@
       <c r="F426" s="1" t="s">
         <v>1001</v>
       </c>
-    </row>
-    <row r="427" spans="1:6">
+      <c r="G426" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="427" spans="1:7">
       <c r="A427" t="s">
         <v>408</v>
       </c>
@@ -10841,8 +10904,11 @@
       <c r="F427" s="1" t="s">
         <v>1002</v>
       </c>
-    </row>
-    <row r="428" spans="1:6">
+      <c r="G427" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="428" spans="1:7">
       <c r="A428" t="s">
         <v>409</v>
       </c>
@@ -10861,8 +10927,11 @@
       <c r="F428" s="1" t="s">
         <v>1003</v>
       </c>
-    </row>
-    <row r="429" spans="1:6">
+      <c r="G428" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="429" spans="1:7">
       <c r="A429" t="s">
         <v>410</v>
       </c>
@@ -10878,8 +10947,11 @@
       <c r="F429" s="1" t="s">
         <v>1004</v>
       </c>
-    </row>
-    <row r="430" spans="1:6">
+      <c r="G429" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="430" spans="1:7">
       <c r="A430" t="s">
         <v>411</v>
       </c>
@@ -10898,8 +10970,11 @@
       <c r="F430" s="1" t="s">
         <v>1005</v>
       </c>
-    </row>
-    <row r="431" spans="1:6">
+      <c r="G430" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="431" spans="1:7">
       <c r="A431" t="s">
         <v>411</v>
       </c>
@@ -10918,8 +10993,11 @@
       <c r="F431" s="1" t="s">
         <v>1005</v>
       </c>
-    </row>
-    <row r="432" spans="1:6">
+      <c r="G431" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="432" spans="1:7">
       <c r="A432" t="s">
         <v>412</v>
       </c>
@@ -10938,8 +11016,11 @@
       <c r="F432" s="1" t="s">
         <v>1006</v>
       </c>
-    </row>
-    <row r="433" spans="1:6">
+      <c r="G432" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="433" spans="1:7">
       <c r="A433" t="s">
         <v>412</v>
       </c>
@@ -10958,8 +11039,11 @@
       <c r="F433" s="1" t="s">
         <v>1006</v>
       </c>
-    </row>
-    <row r="434" spans="1:6">
+      <c r="G433" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="434" spans="1:7">
       <c r="A434" t="s">
         <v>413</v>
       </c>
@@ -10975,8 +11059,11 @@
       <c r="F434" s="1" t="s">
         <v>1007</v>
       </c>
-    </row>
-    <row r="435" spans="1:6">
+      <c r="G434" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="435" spans="1:7">
       <c r="A435" t="s">
         <v>414</v>
       </c>
@@ -10992,8 +11079,11 @@
       <c r="F435" s="1" t="s">
         <v>1008</v>
       </c>
-    </row>
-    <row r="436" spans="1:6">
+      <c r="G435" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="436" spans="1:7">
       <c r="A436" t="s">
         <v>415</v>
       </c>
@@ -11012,8 +11102,11 @@
       <c r="F436" s="1" t="s">
         <v>1009</v>
       </c>
-    </row>
-    <row r="437" spans="1:6">
+      <c r="G436" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="437" spans="1:7">
       <c r="A437" t="s">
         <v>416</v>
       </c>
@@ -11032,8 +11125,11 @@
       <c r="F437" s="1" t="s">
         <v>1010</v>
       </c>
-    </row>
-    <row r="438" spans="1:6">
+      <c r="G437" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="438" spans="1:7">
       <c r="A438" t="s">
         <v>258</v>
       </c>
@@ -11052,8 +11148,11 @@
       <c r="F438" s="1" t="s">
         <v>1011</v>
       </c>
-    </row>
-    <row r="439" spans="1:6">
+      <c r="G438" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="439" spans="1:7">
       <c r="A439" t="s">
         <v>417</v>
       </c>
@@ -11072,8 +11171,11 @@
       <c r="F439" s="1" t="s">
         <v>1012</v>
       </c>
-    </row>
-    <row r="440" spans="1:6">
+      <c r="G439" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="440" spans="1:7">
       <c r="A440" t="s">
         <v>418</v>
       </c>
@@ -11092,8 +11194,11 @@
       <c r="F440" s="1" t="s">
         <v>1013</v>
       </c>
-    </row>
-    <row r="441" spans="1:6">
+      <c r="G440" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="441" spans="1:7">
       <c r="A441" t="s">
         <v>418</v>
       </c>
@@ -11112,8 +11217,11 @@
       <c r="F441" s="1" t="s">
         <v>1013</v>
       </c>
-    </row>
-    <row r="442" spans="1:6">
+      <c r="G441" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="442" spans="1:7">
       <c r="A442" t="s">
         <v>419</v>
       </c>
@@ -11132,8 +11240,11 @@
       <c r="F442" s="1" t="s">
         <v>1014</v>
       </c>
-    </row>
-    <row r="443" spans="1:6">
+      <c r="G442" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="443" spans="1:7">
       <c r="A443" t="s">
         <v>420</v>
       </c>
@@ -11149,8 +11260,11 @@
       <c r="F443" s="1" t="s">
         <v>1015</v>
       </c>
-    </row>
-    <row r="444" spans="1:6">
+      <c r="G443" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="444" spans="1:7">
       <c r="A444" t="s">
         <v>421</v>
       </c>
@@ -11168,6 +11282,9 @@
       </c>
       <c r="F444" s="1" t="s">
         <v>1016</v>
+      </c>
+      <c r="G444" t="s">
+        <v>1017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>